<commit_message>
Fix Vendor Payout location filter so Event + Payee rows populate
Replace unreliable AGGREGATE cross-sheet matching with FILTER against
EVENT ASSIGNMENT source rows (INT date + TRIM payee), then INDEX the
mirrored CONTRACT CALC amounts so ARVC and other payees pull through.

Co-authored-by: unmegonzales <unmegonzales@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/npo-payout/NPO_Payout_Vendor_Template.xlsx
+++ b/npo-payout/NPO_Payout_Vendor_Template.xlsx
@@ -3759,11 +3759,11 @@
     </row>
     <row r="18" ht="18.95" customHeight="1" s="130">
       <c r="A18" s="197">
-        <f>IFERROR(AGGREGATE(15,6,(ROW('CONTRACT CALC'!$A$13:$A$112)-ROW('CONTRACT CALC'!$A$13)+1)/((('CONTRACT CALC'!$A$13:$A$112)=$B$10)*(('CONTRACT CALC'!$B$13:$B$112)=$E$10)),1),"")</f>
+        <f>IFERROR(INDEX(FILTER(ROW('EVENT ASSIGNMENT'!$A$2:$A$101)-ROW('EVENT ASSIGNMENT'!$A$2)+1,(IFERROR(INT('EVENT ASSIGNMENT'!$A$2:$A$101),0)=INT($B$10))*(TRIM('EVENT ASSIGNMENT'!$F$2:$F$101)=TRIM($E$10))),1),"")</f>
         <v/>
       </c>
       <c r="B18" s="198">
-        <f>IF($A18="","",IFERROR(INDEX('CONTRACT CALC'!$D$13:$D$112,$A18),""))</f>
+        <f>IF($A18="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A18),""))</f>
         <v/>
       </c>
       <c r="C18" s="199">
@@ -3791,17 +3791,17 @@
         <v/>
       </c>
       <c r="I18" s="199">
-        <f>IF(OR($A18="",B18=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('CONTRACT CALC'!$C$13:$C$112,$A18))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('CONTRACT CALC'!$C$13:$C$112,$A18)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('CONTRACT CALC'!$D$13:$D$112,$A18))))</f>
+        <f>IF(OR($A18="",B18=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A18))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A18)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A18))))</f>
         <v/>
       </c>
     </row>
     <row r="19" ht="18.95" customHeight="1" s="130">
       <c r="A19" s="197">
-        <f>IFERROR(AGGREGATE(15,6,(ROW('CONTRACT CALC'!$A$13:$A$112)-ROW('CONTRACT CALC'!$A$13)+1)/((('CONTRACT CALC'!$A$13:$A$112)=$B$10)*(('CONTRACT CALC'!$B$13:$B$112)=$E$10)),2),"")</f>
+        <f>IFERROR(INDEX(FILTER(ROW('EVENT ASSIGNMENT'!$A$2:$A$101)-ROW('EVENT ASSIGNMENT'!$A$2)+1,(IFERROR(INT('EVENT ASSIGNMENT'!$A$2:$A$101),0)=INT($B$10))*(TRIM('EVENT ASSIGNMENT'!$F$2:$F$101)=TRIM($E$10))),2),"")</f>
         <v/>
       </c>
       <c r="B19" s="198">
-        <f>IF($A19="","",IFERROR(INDEX('CONTRACT CALC'!$D$13:$D$112,$A19),""))</f>
+        <f>IF($A19="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A19),""))</f>
         <v/>
       </c>
       <c r="C19" s="199">
@@ -3829,17 +3829,17 @@
         <v/>
       </c>
       <c r="I19" s="199">
-        <f>IF(OR($A19="",B19=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('CONTRACT CALC'!$C$13:$C$112,$A19))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('CONTRACT CALC'!$C$13:$C$112,$A19)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('CONTRACT CALC'!$D$13:$D$112,$A19))))</f>
+        <f>IF(OR($A19="",B19=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A19))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A19)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A19))))</f>
         <v/>
       </c>
     </row>
     <row r="20" ht="18.95" customHeight="1" s="130">
       <c r="A20" s="197">
-        <f>IFERROR(AGGREGATE(15,6,(ROW('CONTRACT CALC'!$A$13:$A$112)-ROW('CONTRACT CALC'!$A$13)+1)/((('CONTRACT CALC'!$A$13:$A$112)=$B$10)*(('CONTRACT CALC'!$B$13:$B$112)=$E$10)),3),"")</f>
+        <f>IFERROR(INDEX(FILTER(ROW('EVENT ASSIGNMENT'!$A$2:$A$101)-ROW('EVENT ASSIGNMENT'!$A$2)+1,(IFERROR(INT('EVENT ASSIGNMENT'!$A$2:$A$101),0)=INT($B$10))*(TRIM('EVENT ASSIGNMENT'!$F$2:$F$101)=TRIM($E$10))),3),"")</f>
         <v/>
       </c>
       <c r="B20" s="198">
-        <f>IF($A20="","",IFERROR(INDEX('CONTRACT CALC'!$D$13:$D$112,$A20),""))</f>
+        <f>IF($A20="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A20),""))</f>
         <v/>
       </c>
       <c r="C20" s="199">
@@ -3867,17 +3867,17 @@
         <v/>
       </c>
       <c r="I20" s="199">
-        <f>IF(OR($A20="",B20=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('CONTRACT CALC'!$C$13:$C$112,$A20))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('CONTRACT CALC'!$C$13:$C$112,$A20)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('CONTRACT CALC'!$D$13:$D$112,$A20))))</f>
+        <f>IF(OR($A20="",B20=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A20))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A20)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A20))))</f>
         <v/>
       </c>
     </row>
     <row r="21" ht="18.95" customHeight="1" s="130">
       <c r="A21" s="197">
-        <f>IFERROR(AGGREGATE(15,6,(ROW('CONTRACT CALC'!$A$13:$A$112)-ROW('CONTRACT CALC'!$A$13)+1)/((('CONTRACT CALC'!$A$13:$A$112)=$B$10)*(('CONTRACT CALC'!$B$13:$B$112)=$E$10)),4),"")</f>
+        <f>IFERROR(INDEX(FILTER(ROW('EVENT ASSIGNMENT'!$A$2:$A$101)-ROW('EVENT ASSIGNMENT'!$A$2)+1,(IFERROR(INT('EVENT ASSIGNMENT'!$A$2:$A$101),0)=INT($B$10))*(TRIM('EVENT ASSIGNMENT'!$F$2:$F$101)=TRIM($E$10))),4),"")</f>
         <v/>
       </c>
       <c r="B21" s="198">
-        <f>IF($A21="","",IFERROR(INDEX('CONTRACT CALC'!$D$13:$D$112,$A21),""))</f>
+        <f>IF($A21="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A21),""))</f>
         <v/>
       </c>
       <c r="C21" s="199">
@@ -3905,17 +3905,17 @@
         <v/>
       </c>
       <c r="I21" s="199">
-        <f>IF(OR($A21="",B21=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('CONTRACT CALC'!$C$13:$C$112,$A21))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('CONTRACT CALC'!$C$13:$C$112,$A21)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('CONTRACT CALC'!$D$13:$D$112,$A21))))</f>
+        <f>IF(OR($A21="",B21=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A21))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A21)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A21))))</f>
         <v/>
       </c>
     </row>
     <row r="22" ht="18.95" customHeight="1" s="130">
       <c r="A22" s="197">
-        <f>IFERROR(AGGREGATE(15,6,(ROW('CONTRACT CALC'!$A$13:$A$112)-ROW('CONTRACT CALC'!$A$13)+1)/((('CONTRACT CALC'!$A$13:$A$112)=$B$10)*(('CONTRACT CALC'!$B$13:$B$112)=$E$10)),5),"")</f>
+        <f>IFERROR(INDEX(FILTER(ROW('EVENT ASSIGNMENT'!$A$2:$A$101)-ROW('EVENT ASSIGNMENT'!$A$2)+1,(IFERROR(INT('EVENT ASSIGNMENT'!$A$2:$A$101),0)=INT($B$10))*(TRIM('EVENT ASSIGNMENT'!$F$2:$F$101)=TRIM($E$10))),5),"")</f>
         <v/>
       </c>
       <c r="B22" s="198">
-        <f>IF($A22="","",IFERROR(INDEX('CONTRACT CALC'!$D$13:$D$112,$A22),""))</f>
+        <f>IF($A22="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A22),""))</f>
         <v/>
       </c>
       <c r="C22" s="199">
@@ -3943,17 +3943,17 @@
         <v/>
       </c>
       <c r="I22" s="199">
-        <f>IF(OR($A22="",B22=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('CONTRACT CALC'!$C$13:$C$112,$A22))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('CONTRACT CALC'!$C$13:$C$112,$A22)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('CONTRACT CALC'!$D$13:$D$112,$A22))))</f>
+        <f>IF(OR($A22="",B22=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A22))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A22)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A22))))</f>
         <v/>
       </c>
     </row>
     <row r="23" ht="20.1" customHeight="1" s="130">
       <c r="A23" s="197">
-        <f>IFERROR(AGGREGATE(15,6,(ROW('CONTRACT CALC'!$A$13:$A$112)-ROW('CONTRACT CALC'!$A$13)+1)/((('CONTRACT CALC'!$A$13:$A$112)=$B$10)*(('CONTRACT CALC'!$B$13:$B$112)=$E$10)),6),"")</f>
+        <f>IFERROR(INDEX(FILTER(ROW('EVENT ASSIGNMENT'!$A$2:$A$101)-ROW('EVENT ASSIGNMENT'!$A$2)+1,(IFERROR(INT('EVENT ASSIGNMENT'!$A$2:$A$101),0)=INT($B$10))*(TRIM('EVENT ASSIGNMENT'!$F$2:$F$101)=TRIM($E$10))),6),"")</f>
         <v/>
       </c>
       <c r="B23" s="198">
-        <f>IF($A23="","",IFERROR(INDEX('CONTRACT CALC'!$D$13:$D$112,$A23),""))</f>
+        <f>IF($A23="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A23),""))</f>
         <v/>
       </c>
       <c r="C23" s="199">
@@ -3981,17 +3981,17 @@
         <v/>
       </c>
       <c r="I23" s="199">
-        <f>IF(OR($A23="",B23=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('CONTRACT CALC'!$C$13:$C$112,$A23))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('CONTRACT CALC'!$C$13:$C$112,$A23)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('CONTRACT CALC'!$D$13:$D$112,$A23))))</f>
+        <f>IF(OR($A23="",B23=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A23))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A23)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A23))))</f>
         <v/>
       </c>
     </row>
     <row r="24" ht="17.1" customHeight="1" s="130">
       <c r="A24" s="197">
-        <f>IFERROR(AGGREGATE(15,6,(ROW('CONTRACT CALC'!$A$13:$A$112)-ROW('CONTRACT CALC'!$A$13)+1)/((('CONTRACT CALC'!$A$13:$A$112)=$B$10)*(('CONTRACT CALC'!$B$13:$B$112)=$E$10)),7),"")</f>
+        <f>IFERROR(INDEX(FILTER(ROW('EVENT ASSIGNMENT'!$A$2:$A$101)-ROW('EVENT ASSIGNMENT'!$A$2)+1,(IFERROR(INT('EVENT ASSIGNMENT'!$A$2:$A$101),0)=INT($B$10))*(TRIM('EVENT ASSIGNMENT'!$F$2:$F$101)=TRIM($E$10))),7),"")</f>
         <v/>
       </c>
       <c r="B24" s="198">
-        <f>IF($A24="","",IFERROR(INDEX('CONTRACT CALC'!$D$13:$D$112,$A24),""))</f>
+        <f>IF($A24="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A24),""))</f>
         <v/>
       </c>
       <c r="C24" s="199">
@@ -4019,17 +4019,17 @@
         <v/>
       </c>
       <c r="I24" s="199">
-        <f>IF(OR($A24="",B24=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('CONTRACT CALC'!$C$13:$C$112,$A24))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('CONTRACT CALC'!$C$13:$C$112,$A24)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('CONTRACT CALC'!$D$13:$D$112,$A24))))</f>
+        <f>IF(OR($A24="",B24=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A24))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A24)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A24))))</f>
         <v/>
       </c>
     </row>
     <row r="25" ht="20.1" customHeight="1" s="130">
       <c r="A25" s="197">
-        <f>IFERROR(AGGREGATE(15,6,(ROW('CONTRACT CALC'!$A$13:$A$112)-ROW('CONTRACT CALC'!$A$13)+1)/((('CONTRACT CALC'!$A$13:$A$112)=$B$10)*(('CONTRACT CALC'!$B$13:$B$112)=$E$10)),8),"")</f>
+        <f>IFERROR(INDEX(FILTER(ROW('EVENT ASSIGNMENT'!$A$2:$A$101)-ROW('EVENT ASSIGNMENT'!$A$2)+1,(IFERROR(INT('EVENT ASSIGNMENT'!$A$2:$A$101),0)=INT($B$10))*(TRIM('EVENT ASSIGNMENT'!$F$2:$F$101)=TRIM($E$10))),8),"")</f>
         <v/>
       </c>
       <c r="B25" s="198">
-        <f>IF($A25="","",IFERROR(INDEX('CONTRACT CALC'!$D$13:$D$112,$A25),""))</f>
+        <f>IF($A25="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A25),""))</f>
         <v/>
       </c>
       <c r="C25" s="199">
@@ -4057,17 +4057,17 @@
         <v/>
       </c>
       <c r="I25" s="199">
-        <f>IF(OR($A25="",B25=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('CONTRACT CALC'!$C$13:$C$112,$A25))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('CONTRACT CALC'!$C$13:$C$112,$A25)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('CONTRACT CALC'!$D$13:$D$112,$A25))))</f>
+        <f>IF(OR($A25="",B25=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A25))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A25)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A25))))</f>
         <v/>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1" s="130">
       <c r="A26" s="197">
-        <f>IFERROR(AGGREGATE(15,6,(ROW('CONTRACT CALC'!$A$13:$A$112)-ROW('CONTRACT CALC'!$A$13)+1)/((('CONTRACT CALC'!$A$13:$A$112)=$B$10)*(('CONTRACT CALC'!$B$13:$B$112)=$E$10)),9),"")</f>
+        <f>IFERROR(INDEX(FILTER(ROW('EVENT ASSIGNMENT'!$A$2:$A$101)-ROW('EVENT ASSIGNMENT'!$A$2)+1,(IFERROR(INT('EVENT ASSIGNMENT'!$A$2:$A$101),0)=INT($B$10))*(TRIM('EVENT ASSIGNMENT'!$F$2:$F$101)=TRIM($E$10))),9),"")</f>
         <v/>
       </c>
       <c r="B26" s="198">
-        <f>IF($A26="","",IFERROR(INDEX('CONTRACT CALC'!$D$13:$D$112,$A26),""))</f>
+        <f>IF($A26="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A26),""))</f>
         <v/>
       </c>
       <c r="C26" s="199">
@@ -4095,17 +4095,17 @@
         <v/>
       </c>
       <c r="I26" s="199">
-        <f>IF(OR($A26="",B26=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('CONTRACT CALC'!$C$13:$C$112,$A26))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('CONTRACT CALC'!$C$13:$C$112,$A26)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('CONTRACT CALC'!$D$13:$D$112,$A26))))</f>
+        <f>IF(OR($A26="",B26=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A26))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A26)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A26))))</f>
         <v/>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1" s="130">
       <c r="A27" s="197">
-        <f>IFERROR(AGGREGATE(15,6,(ROW('CONTRACT CALC'!$A$13:$A$112)-ROW('CONTRACT CALC'!$A$13)+1)/((('CONTRACT CALC'!$A$13:$A$112)=$B$10)*(('CONTRACT CALC'!$B$13:$B$112)=$E$10)),10),"")</f>
+        <f>IFERROR(INDEX(FILTER(ROW('EVENT ASSIGNMENT'!$A$2:$A$101)-ROW('EVENT ASSIGNMENT'!$A$2)+1,(IFERROR(INT('EVENT ASSIGNMENT'!$A$2:$A$101),0)=INT($B$10))*(TRIM('EVENT ASSIGNMENT'!$F$2:$F$101)=TRIM($E$10))),10),"")</f>
         <v/>
       </c>
       <c r="B27" s="198">
-        <f>IF($A27="","",IFERROR(INDEX('CONTRACT CALC'!$D$13:$D$112,$A27),""))</f>
+        <f>IF($A27="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A27),""))</f>
         <v/>
       </c>
       <c r="C27" s="199">
@@ -4133,17 +4133,17 @@
         <v/>
       </c>
       <c r="I27" s="199">
-        <f>IF(OR($A27="",B27=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('CONTRACT CALC'!$C$13:$C$112,$A27))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('CONTRACT CALC'!$C$13:$C$112,$A27)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('CONTRACT CALC'!$D$13:$D$112,$A27))))</f>
+        <f>IF(OR($A27="",B27=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A27))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A27)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A27))))</f>
         <v/>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1" s="130">
       <c r="A28" s="197">
-        <f>IFERROR(AGGREGATE(15,6,(ROW('CONTRACT CALC'!$A$13:$A$112)-ROW('CONTRACT CALC'!$A$13)+1)/((('CONTRACT CALC'!$A$13:$A$112)=$B$10)*(('CONTRACT CALC'!$B$13:$B$112)=$E$10)),11),"")</f>
+        <f>IFERROR(INDEX(FILTER(ROW('EVENT ASSIGNMENT'!$A$2:$A$101)-ROW('EVENT ASSIGNMENT'!$A$2)+1,(IFERROR(INT('EVENT ASSIGNMENT'!$A$2:$A$101),0)=INT($B$10))*(TRIM('EVENT ASSIGNMENT'!$F$2:$F$101)=TRIM($E$10))),11),"")</f>
         <v/>
       </c>
       <c r="B28" s="198">
-        <f>IF($A28="","",IFERROR(INDEX('CONTRACT CALC'!$D$13:$D$112,$A28),""))</f>
+        <f>IF($A28="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A28),""))</f>
         <v/>
       </c>
       <c r="C28" s="199">
@@ -4171,17 +4171,17 @@
         <v/>
       </c>
       <c r="I28" s="199">
-        <f>IF(OR($A28="",B28=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('CONTRACT CALC'!$C$13:$C$112,$A28))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('CONTRACT CALC'!$C$13:$C$112,$A28)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('CONTRACT CALC'!$D$13:$D$112,$A28))))</f>
+        <f>IF(OR($A28="",B28=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A28))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A28)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A28))))</f>
         <v/>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1" s="130">
       <c r="A29" s="197">
-        <f>IFERROR(AGGREGATE(15,6,(ROW('CONTRACT CALC'!$A$13:$A$112)-ROW('CONTRACT CALC'!$A$13)+1)/((('CONTRACT CALC'!$A$13:$A$112)=$B$10)*(('CONTRACT CALC'!$B$13:$B$112)=$E$10)),12),"")</f>
+        <f>IFERROR(INDEX(FILTER(ROW('EVENT ASSIGNMENT'!$A$2:$A$101)-ROW('EVENT ASSIGNMENT'!$A$2)+1,(IFERROR(INT('EVENT ASSIGNMENT'!$A$2:$A$101),0)=INT($B$10))*(TRIM('EVENT ASSIGNMENT'!$F$2:$F$101)=TRIM($E$10))),12),"")</f>
         <v/>
       </c>
       <c r="B29" s="198">
-        <f>IF($A29="","",IFERROR(INDEX('CONTRACT CALC'!$D$13:$D$112,$A29),""))</f>
+        <f>IF($A29="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A29),""))</f>
         <v/>
       </c>
       <c r="C29" s="199">
@@ -4209,17 +4209,17 @@
         <v/>
       </c>
       <c r="I29" s="199">
-        <f>IF(OR($A29="",B29=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('CONTRACT CALC'!$C$13:$C$112,$A29))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('CONTRACT CALC'!$C$13:$C$112,$A29)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('CONTRACT CALC'!$D$13:$D$112,$A29))))</f>
+        <f>IF(OR($A29="",B29=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A29))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A29)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A29))))</f>
         <v/>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1" s="130">
       <c r="A30" s="197">
-        <f>IFERROR(AGGREGATE(15,6,(ROW('CONTRACT CALC'!$A$13:$A$112)-ROW('CONTRACT CALC'!$A$13)+1)/((('CONTRACT CALC'!$A$13:$A$112)=$B$10)*(('CONTRACT CALC'!$B$13:$B$112)=$E$10)),13),"")</f>
+        <f>IFERROR(INDEX(FILTER(ROW('EVENT ASSIGNMENT'!$A$2:$A$101)-ROW('EVENT ASSIGNMENT'!$A$2)+1,(IFERROR(INT('EVENT ASSIGNMENT'!$A$2:$A$101),0)=INT($B$10))*(TRIM('EVENT ASSIGNMENT'!$F$2:$F$101)=TRIM($E$10))),13),"")</f>
         <v/>
       </c>
       <c r="B30" s="198">
-        <f>IF($A30="","",IFERROR(INDEX('CONTRACT CALC'!$D$13:$D$112,$A30),""))</f>
+        <f>IF($A30="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A30),""))</f>
         <v/>
       </c>
       <c r="C30" s="199">
@@ -4247,17 +4247,17 @@
         <v/>
       </c>
       <c r="I30" s="199">
-        <f>IF(OR($A30="",B30=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('CONTRACT CALC'!$C$13:$C$112,$A30))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('CONTRACT CALC'!$C$13:$C$112,$A30)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('CONTRACT CALC'!$D$13:$D$112,$A30))))</f>
+        <f>IF(OR($A30="",B30=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A30))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A30)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A30))))</f>
         <v/>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1" s="130" thickBot="1">
       <c r="A31" s="197">
-        <f>IFERROR(AGGREGATE(15,6,(ROW('CONTRACT CALC'!$A$13:$A$112)-ROW('CONTRACT CALC'!$A$13)+1)/((('CONTRACT CALC'!$A$13:$A$112)=$B$10)*(('CONTRACT CALC'!$B$13:$B$112)=$E$10)),14),"")</f>
+        <f>IFERROR(INDEX(FILTER(ROW('EVENT ASSIGNMENT'!$A$2:$A$101)-ROW('EVENT ASSIGNMENT'!$A$2)+1,(IFERROR(INT('EVENT ASSIGNMENT'!$A$2:$A$101),0)=INT($B$10))*(TRIM('EVENT ASSIGNMENT'!$F$2:$F$101)=TRIM($E$10))),14),"")</f>
         <v/>
       </c>
       <c r="B31" s="198">
-        <f>IF($A31="","",IFERROR(INDEX('CONTRACT CALC'!$D$13:$D$112,$A31),""))</f>
+        <f>IF($A31="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A31),""))</f>
         <v/>
       </c>
       <c r="C31" s="199">
@@ -4285,17 +4285,17 @@
         <v/>
       </c>
       <c r="I31" s="199">
-        <f>IF(OR($A31="",B31=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('CONTRACT CALC'!$C$13:$C$112,$A31))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('CONTRACT CALC'!$C$13:$C$112,$A31)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('CONTRACT CALC'!$D$13:$D$112,$A31))))</f>
+        <f>IF(OR($A31="",B31=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A31))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A31)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A31))))</f>
         <v/>
       </c>
     </row>
     <row r="32" ht="20.25" customHeight="1" s="130">
       <c r="A32" s="197">
-        <f>IFERROR(AGGREGATE(15,6,(ROW('CONTRACT CALC'!$A$13:$A$112)-ROW('CONTRACT CALC'!$A$13)+1)/((('CONTRACT CALC'!$A$13:$A$112)=$B$10)*(('CONTRACT CALC'!$B$13:$B$112)=$E$10)),15),"")</f>
+        <f>IFERROR(INDEX(FILTER(ROW('EVENT ASSIGNMENT'!$A$2:$A$101)-ROW('EVENT ASSIGNMENT'!$A$2)+1,(IFERROR(INT('EVENT ASSIGNMENT'!$A$2:$A$101),0)=INT($B$10))*(TRIM('EVENT ASSIGNMENT'!$F$2:$F$101)=TRIM($E$10))),15),"")</f>
         <v/>
       </c>
       <c r="B32" s="201">
-        <f>IF($A32="","",IFERROR(INDEX('CONTRACT CALC'!$D$13:$D$112,$A32),""))</f>
+        <f>IF($A32="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A32),""))</f>
         <v/>
       </c>
       <c r="C32" s="202">
@@ -4323,17 +4323,17 @@
         <v/>
       </c>
       <c r="I32" s="202">
-        <f>IF(OR($A32="",B32=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('CONTRACT CALC'!$C$13:$C$112,$A32))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('CONTRACT CALC'!$C$13:$C$112,$A32)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('CONTRACT CALC'!$D$13:$D$112,$A32))))</f>
+        <f>IF(OR($A32="",B32=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A32))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A32)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A32))))</f>
         <v/>
       </c>
     </row>
     <row r="33" ht="6" customHeight="1" s="130">
       <c r="A33" s="197">
-        <f>IFERROR(AGGREGATE(15,6,(ROW('CONTRACT CALC'!$A$13:$A$112)-ROW('CONTRACT CALC'!$A$13)+1)/((('CONTRACT CALC'!$A$13:$A$112)=$B$10)*(('CONTRACT CALC'!$B$13:$B$112)=$E$10)),16),"")</f>
+        <f>IFERROR(INDEX(FILTER(ROW('EVENT ASSIGNMENT'!$A$2:$A$101)-ROW('EVENT ASSIGNMENT'!$A$2)+1,(IFERROR(INT('EVENT ASSIGNMENT'!$A$2:$A$101),0)=INT($B$10))*(TRIM('EVENT ASSIGNMENT'!$F$2:$F$101)=TRIM($E$10))),16),"")</f>
         <v/>
       </c>
       <c r="B33" s="203">
-        <f>IF($A33="","",IFERROR(INDEX('CONTRACT CALC'!$D$13:$D$112,$A33),""))</f>
+        <f>IF($A33="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A33),""))</f>
         <v/>
       </c>
       <c r="C33" s="204">
@@ -4361,17 +4361,17 @@
         <v/>
       </c>
       <c r="I33" s="204">
-        <f>IF(OR($A33="",B33=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('CONTRACT CALC'!$C$13:$C$112,$A33))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('CONTRACT CALC'!$C$13:$C$112,$A33)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('CONTRACT CALC'!$D$13:$D$112,$A33))))</f>
+        <f>IF(OR($A33="",B33=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A33))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A33)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A33))))</f>
         <v/>
       </c>
     </row>
     <row r="34" ht="13.5" customHeight="1" s="130" thickBot="1">
       <c r="A34" s="197">
-        <f>IFERROR(AGGREGATE(15,6,(ROW('CONTRACT CALC'!$A$13:$A$112)-ROW('CONTRACT CALC'!$A$13)+1)/((('CONTRACT CALC'!$A$13:$A$112)=$B$10)*(('CONTRACT CALC'!$B$13:$B$112)=$E$10)),17),"")</f>
+        <f>IFERROR(INDEX(FILTER(ROW('EVENT ASSIGNMENT'!$A$2:$A$101)-ROW('EVENT ASSIGNMENT'!$A$2)+1,(IFERROR(INT('EVENT ASSIGNMENT'!$A$2:$A$101),0)=INT($B$10))*(TRIM('EVENT ASSIGNMENT'!$F$2:$F$101)=TRIM($E$10))),17),"")</f>
         <v/>
       </c>
       <c r="B34" s="201">
-        <f>IF($A34="","",IFERROR(INDEX('CONTRACT CALC'!$D$13:$D$112,$A34),""))</f>
+        <f>IF($A34="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A34),""))</f>
         <v/>
       </c>
       <c r="C34" s="202">
@@ -4399,17 +4399,17 @@
         <v/>
       </c>
       <c r="I34" s="202">
-        <f>IF(OR($A34="",B34=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('CONTRACT CALC'!$C$13:$C$112,$A34))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('CONTRACT CALC'!$C$13:$C$112,$A34)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('CONTRACT CALC'!$D$13:$D$112,$A34))))</f>
+        <f>IF(OR($A34="",B34=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A34))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A34)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A34))))</f>
         <v/>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1" s="130" thickBot="1">
       <c r="A35" s="197">
-        <f>IFERROR(AGGREGATE(15,6,(ROW('CONTRACT CALC'!$A$13:$A$112)-ROW('CONTRACT CALC'!$A$13)+1)/((('CONTRACT CALC'!$A$13:$A$112)=$B$10)*(('CONTRACT CALC'!$B$13:$B$112)=$E$10)),18),"")</f>
+        <f>IFERROR(INDEX(FILTER(ROW('EVENT ASSIGNMENT'!$A$2:$A$101)-ROW('EVENT ASSIGNMENT'!$A$2)+1,(IFERROR(INT('EVENT ASSIGNMENT'!$A$2:$A$101),0)=INT($B$10))*(TRIM('EVENT ASSIGNMENT'!$F$2:$F$101)=TRIM($E$10))),18),"")</f>
         <v/>
       </c>
       <c r="B35" s="205">
-        <f>IF($A35="","",IFERROR(INDEX('CONTRACT CALC'!$D$13:$D$112,$A35),""))</f>
+        <f>IF($A35="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A35),""))</f>
         <v/>
       </c>
       <c r="C35" s="199">
@@ -4437,17 +4437,17 @@
         <v/>
       </c>
       <c r="I35" s="199">
-        <f>IF(OR($A35="",B35=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('CONTRACT CALC'!$C$13:$C$112,$A35))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('CONTRACT CALC'!$C$13:$C$112,$A35)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('CONTRACT CALC'!$D$13:$D$112,$A35))))</f>
+        <f>IF(OR($A35="",B35=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A35))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A35)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A35))))</f>
         <v/>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1" s="130">
       <c r="A36" s="197">
-        <f>IFERROR(AGGREGATE(15,6,(ROW('CONTRACT CALC'!$A$13:$A$112)-ROW('CONTRACT CALC'!$A$13)+1)/((('CONTRACT CALC'!$A$13:$A$112)=$B$10)*(('CONTRACT CALC'!$B$13:$B$112)=$E$10)),19),"")</f>
+        <f>IFERROR(INDEX(FILTER(ROW('EVENT ASSIGNMENT'!$A$2:$A$101)-ROW('EVENT ASSIGNMENT'!$A$2)+1,(IFERROR(INT('EVENT ASSIGNMENT'!$A$2:$A$101),0)=INT($B$10))*(TRIM('EVENT ASSIGNMENT'!$F$2:$F$101)=TRIM($E$10))),19),"")</f>
         <v/>
       </c>
       <c r="B36" s="198">
-        <f>IF($A36="","",IFERROR(INDEX('CONTRACT CALC'!$D$13:$D$112,$A36),""))</f>
+        <f>IF($A36="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A36),""))</f>
         <v/>
       </c>
       <c r="C36" s="199">
@@ -4475,17 +4475,17 @@
         <v/>
       </c>
       <c r="I36" s="199">
-        <f>IF(OR($A36="",B36=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('CONTRACT CALC'!$C$13:$C$112,$A36))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('CONTRACT CALC'!$C$13:$C$112,$A36)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('CONTRACT CALC'!$D$13:$D$112,$A36))))</f>
+        <f>IF(OR($A36="",B36=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A36))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A36)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A36))))</f>
         <v/>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1" s="130">
       <c r="A37" s="197">
-        <f>IFERROR(AGGREGATE(15,6,(ROW('CONTRACT CALC'!$A$13:$A$112)-ROW('CONTRACT CALC'!$A$13)+1)/((('CONTRACT CALC'!$A$13:$A$112)=$B$10)*(('CONTRACT CALC'!$B$13:$B$112)=$E$10)),20),"")</f>
+        <f>IFERROR(INDEX(FILTER(ROW('EVENT ASSIGNMENT'!$A$2:$A$101)-ROW('EVENT ASSIGNMENT'!$A$2)+1,(IFERROR(INT('EVENT ASSIGNMENT'!$A$2:$A$101),0)=INT($B$10))*(TRIM('EVENT ASSIGNMENT'!$F$2:$F$101)=TRIM($E$10))),20),"")</f>
         <v/>
       </c>
       <c r="B37" s="198">
-        <f>IF($A37="","",IFERROR(INDEX('CONTRACT CALC'!$D$13:$D$112,$A37),""))</f>
+        <f>IF($A37="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A37),""))</f>
         <v/>
       </c>
       <c r="C37" s="199">
@@ -4513,17 +4513,17 @@
         <v/>
       </c>
       <c r="I37" s="199">
-        <f>IF(OR($A37="",B37=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('CONTRACT CALC'!$C$13:$C$112,$A37))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('CONTRACT CALC'!$C$13:$C$112,$A37)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('CONTRACT CALC'!$D$13:$D$112,$A37))))</f>
+        <f>IF(OR($A37="",B37=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A37))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A37)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A37))))</f>
         <v/>
       </c>
     </row>
     <row r="38" ht="16.5" customHeight="1" s="130">
       <c r="A38" s="197">
-        <f>IFERROR(AGGREGATE(15,6,(ROW('CONTRACT CALC'!$A$13:$A$112)-ROW('CONTRACT CALC'!$A$13)+1)/((('CONTRACT CALC'!$A$13:$A$112)=$B$10)*(('CONTRACT CALC'!$B$13:$B$112)=$E$10)),21),"")</f>
+        <f>IFERROR(INDEX(FILTER(ROW('EVENT ASSIGNMENT'!$A$2:$A$101)-ROW('EVENT ASSIGNMENT'!$A$2)+1,(IFERROR(INT('EVENT ASSIGNMENT'!$A$2:$A$101),0)=INT($B$10))*(TRIM('EVENT ASSIGNMENT'!$F$2:$F$101)=TRIM($E$10))),21),"")</f>
         <v/>
       </c>
       <c r="B38" s="198">
-        <f>IF($A38="","",IFERROR(INDEX('CONTRACT CALC'!$D$13:$D$112,$A38),""))</f>
+        <f>IF($A38="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A38),""))</f>
         <v/>
       </c>
       <c r="C38" s="199">
@@ -4551,17 +4551,17 @@
         <v/>
       </c>
       <c r="I38" s="199">
-        <f>IF(OR($A38="",B38=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('CONTRACT CALC'!$C$13:$C$112,$A38))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('CONTRACT CALC'!$C$13:$C$112,$A38)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('CONTRACT CALC'!$D$13:$D$112,$A38))))</f>
+        <f>IF(OR($A38="",B38=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A38))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A38)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A38))))</f>
         <v/>
       </c>
     </row>
     <row r="39" ht="20.1" customHeight="1" s="130">
       <c r="A39" s="208">
-        <f>IFERROR(AGGREGATE(15,6,(ROW('CONTRACT CALC'!$A$13:$A$112)-ROW('CONTRACT CALC'!$A$13)+1)/((('CONTRACT CALC'!$A$13:$A$112)=$B$10)*(('CONTRACT CALC'!$B$13:$B$112)=$E$10)),22),"")</f>
+        <f>IFERROR(INDEX(FILTER(ROW('EVENT ASSIGNMENT'!$A$2:$A$101)-ROW('EVENT ASSIGNMENT'!$A$2)+1,(IFERROR(INT('EVENT ASSIGNMENT'!$A$2:$A$101),0)=INT($B$10))*(TRIM('EVENT ASSIGNMENT'!$F$2:$F$101)=TRIM($E$10))),22),"")</f>
         <v/>
       </c>
       <c r="B39" s="198">
-        <f>IF($A39="","",IFERROR(INDEX('CONTRACT CALC'!$D$13:$D$112,$A39),""))</f>
+        <f>IF($A39="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A39),""))</f>
         <v/>
       </c>
       <c r="C39" s="199">
@@ -4589,17 +4589,17 @@
         <v/>
       </c>
       <c r="I39" s="199">
-        <f>IF(OR($A39="",B39=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('CONTRACT CALC'!$C$13:$C$112,$A39))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('CONTRACT CALC'!$C$13:$C$112,$A39)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('CONTRACT CALC'!$D$13:$D$112,$A39))))</f>
+        <f>IF(OR($A39="",B39=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A39))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A39)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A39))))</f>
         <v/>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="208">
-        <f>IFERROR(AGGREGATE(15,6,(ROW('CONTRACT CALC'!$A$13:$A$112)-ROW('CONTRACT CALC'!$A$13)+1)/((('CONTRACT CALC'!$A$13:$A$112)=$B$10)*(('CONTRACT CALC'!$B$13:$B$112)=$E$10)),23),"")</f>
+        <f>IFERROR(INDEX(FILTER(ROW('EVENT ASSIGNMENT'!$A$2:$A$101)-ROW('EVENT ASSIGNMENT'!$A$2)+1,(IFERROR(INT('EVENT ASSIGNMENT'!$A$2:$A$101),0)=INT($B$10))*(TRIM('EVENT ASSIGNMENT'!$F$2:$F$101)=TRIM($E$10))),23),"")</f>
         <v/>
       </c>
       <c r="B40" s="198">
-        <f>IF($A40="","",IFERROR(INDEX('CONTRACT CALC'!$D$13:$D$112,$A40),""))</f>
+        <f>IF($A40="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A40),""))</f>
         <v/>
       </c>
       <c r="C40" s="199">
@@ -4627,17 +4627,17 @@
         <v/>
       </c>
       <c r="I40" s="199">
-        <f>IF(OR($A40="",B40=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('CONTRACT CALC'!$C$13:$C$112,$A40))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('CONTRACT CALC'!$C$13:$C$112,$A40)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('CONTRACT CALC'!$D$13:$D$112,$A40))))</f>
+        <f>IF(OR($A40="",B40=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A40))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A40)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A40))))</f>
         <v/>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="130">
       <c r="A41" s="208">
-        <f>IFERROR(AGGREGATE(15,6,(ROW('CONTRACT CALC'!$A$13:$A$112)-ROW('CONTRACT CALC'!$A$13)+1)/((('CONTRACT CALC'!$A$13:$A$112)=$B$10)*(('CONTRACT CALC'!$B$13:$B$112)=$E$10)),24),"")</f>
+        <f>IFERROR(INDEX(FILTER(ROW('EVENT ASSIGNMENT'!$A$2:$A$101)-ROW('EVENT ASSIGNMENT'!$A$2)+1,(IFERROR(INT('EVENT ASSIGNMENT'!$A$2:$A$101),0)=INT($B$10))*(TRIM('EVENT ASSIGNMENT'!$F$2:$F$101)=TRIM($E$10))),24),"")</f>
         <v/>
       </c>
       <c r="B41" s="198">
-        <f>IF($A41="","",IFERROR(INDEX('CONTRACT CALC'!$D$13:$D$112,$A41),""))</f>
+        <f>IF($A41="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A41),""))</f>
         <v/>
       </c>
       <c r="C41" s="199">
@@ -4665,17 +4665,17 @@
         <v/>
       </c>
       <c r="I41" s="199">
-        <f>IF(OR($A41="",B41=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('CONTRACT CALC'!$C$13:$C$112,$A41))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('CONTRACT CALC'!$C$13:$C$112,$A41)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('CONTRACT CALC'!$D$13:$D$112,$A41))))</f>
+        <f>IF(OR($A41="",B41=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A41))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A41)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A41))))</f>
         <v/>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="208">
-        <f>IFERROR(AGGREGATE(15,6,(ROW('CONTRACT CALC'!$A$13:$A$112)-ROW('CONTRACT CALC'!$A$13)+1)/((('CONTRACT CALC'!$A$13:$A$112)=$B$10)*(('CONTRACT CALC'!$B$13:$B$112)=$E$10)),25),"")</f>
+        <f>IFERROR(INDEX(FILTER(ROW('EVENT ASSIGNMENT'!$A$2:$A$101)-ROW('EVENT ASSIGNMENT'!$A$2)+1,(IFERROR(INT('EVENT ASSIGNMENT'!$A$2:$A$101),0)=INT($B$10))*(TRIM('EVENT ASSIGNMENT'!$F$2:$F$101)=TRIM($E$10))),25),"")</f>
         <v/>
       </c>
       <c r="B42" s="198">
-        <f>IF($A42="","",IFERROR(INDEX('CONTRACT CALC'!$D$13:$D$112,$A42),""))</f>
+        <f>IF($A42="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A42),""))</f>
         <v/>
       </c>
       <c r="C42" s="199">
@@ -4703,7 +4703,7 @@
         <v/>
       </c>
       <c r="I42" s="199">
-        <f>IF(OR($A42="",B42=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('CONTRACT CALC'!$C$13:$C$112,$A42))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('CONTRACT CALC'!$C$13:$C$112,$A42)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('CONTRACT CALC'!$D$13:$D$112,$A42))))</f>
+        <f>IF(OR($A42="",B42=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A42))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A42)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A42))))</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix blank Vendor Payout rows by dropping FILTER helper dependency
Excel repaired away openpyxl-written FILTER formulas in hidden column A,
so every detail row that tested $A18="" stayed blank. Match Event+Payee
with classic AGGREGATE against EVENT ASSIGNMENT and make SERVICE AREA
self-contained so the payout no longer depends on a helper column.

Co-authored-by: unmegonzales <unmegonzales@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/npo-payout/NPO_Payout_Vendor_Template.xlsx
+++ b/npo-payout/NPO_Payout_Vendor_Template.xlsx
@@ -3464,7 +3464,7 @@
   <dimension ref="A1:L80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="12.75"/>
   <cols>
-    <col hidden="1" width="4" customWidth="1" style="130" min="1" max="1"/>
+    <col width="6" customWidth="1" style="130" min="1" max="1"/>
     <col width="24" customWidth="1" style="130" min="2" max="2"/>
     <col width="15" customWidth="1" style="130" min="3" max="3"/>
     <col width="17" bestFit="1" customWidth="1" style="130" min="4" max="4"/>
@@ -3759,19 +3759,19 @@
     </row>
     <row r="18" ht="18.95" customHeight="1" s="130">
       <c r="A18" s="197">
-        <f>IFERROR(INDEX(FILTER(ROW('EVENT ASSIGNMENT'!$A$2:$A$101)-ROW('EVENT ASSIGNMENT'!$A$2)+1,(IFERROR(INT('EVENT ASSIGNMENT'!$A$2:$A$101),0)=INT($B$10))*(TRIM('EVENT ASSIGNMENT'!$F$2:$F$101)=TRIM($E$10))),1),"")</f>
+        <f>IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),1),"")</f>
         <v/>
       </c>
       <c r="B18" s="198">
-        <f>IF($A18="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A18),""))</f>
+        <f>IFERROR(INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),1),"")),"")</f>
         <v/>
       </c>
       <c r="C18" s="199">
-        <f>IF(OR($A18="",B18=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,$A18)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A18),""))</f>
+        <f>IF(B18="","",IFERROR(INDEX('CONTRACT CALC'!$G:$G,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),1),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),1),""))+11),""))</f>
         <v/>
       </c>
       <c r="D18" s="199">
-        <f>IF(OR($A18="",B18=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,$A18)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A18),""))</f>
+        <f>IF(B18="","",IFERROR(INDEX('CONTRACT CALC'!$I:$I,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),1),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),1),""))+11),""))</f>
         <v/>
       </c>
       <c r="E18" s="199">
@@ -3779,7 +3779,7 @@
         <v/>
       </c>
       <c r="F18" s="199">
-        <f>IF(OR($A18="",B18=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,$A18)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A18),""))</f>
+        <f>IF(B18="","",IFERROR(INDEX('CONTRACT CALC'!$H:$H,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),1),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),1),""))+11),""))</f>
         <v/>
       </c>
       <c r="G18" s="199">
@@ -3791,25 +3791,25 @@
         <v/>
       </c>
       <c r="I18" s="199">
-        <f>IF(OR($A18="",B18=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A18))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A18)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A18))))</f>
+        <f>IF(B18="","",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),1),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),1),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),1),"")))))</f>
         <v/>
       </c>
     </row>
     <row r="19" ht="18.95" customHeight="1" s="130">
       <c r="A19" s="197">
-        <f>IFERROR(INDEX(FILTER(ROW('EVENT ASSIGNMENT'!$A$2:$A$101)-ROW('EVENT ASSIGNMENT'!$A$2)+1,(IFERROR(INT('EVENT ASSIGNMENT'!$A$2:$A$101),0)=INT($B$10))*(TRIM('EVENT ASSIGNMENT'!$F$2:$F$101)=TRIM($E$10))),2),"")</f>
+        <f>IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),2),"")</f>
         <v/>
       </c>
       <c r="B19" s="198">
-        <f>IF($A19="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A19),""))</f>
+        <f>IFERROR(INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),2),"")),"")</f>
         <v/>
       </c>
       <c r="C19" s="199">
-        <f>IF(OR($A19="",B19=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,$A19)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A19),""))</f>
+        <f>IF(B19="","",IFERROR(INDEX('CONTRACT CALC'!$G:$G,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),2),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),2),""))+11),""))</f>
         <v/>
       </c>
       <c r="D19" s="199">
-        <f>IF(OR($A19="",B19=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,$A19)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A19),""))</f>
+        <f>IF(B19="","",IFERROR(INDEX('CONTRACT CALC'!$I:$I,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),2),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),2),""))+11),""))</f>
         <v/>
       </c>
       <c r="E19" s="199">
@@ -3817,7 +3817,7 @@
         <v/>
       </c>
       <c r="F19" s="199">
-        <f>IF(OR($A19="",B19=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,$A19)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A19),""))</f>
+        <f>IF(B19="","",IFERROR(INDEX('CONTRACT CALC'!$H:$H,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),2),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),2),""))+11),""))</f>
         <v/>
       </c>
       <c r="G19" s="199">
@@ -3829,25 +3829,25 @@
         <v/>
       </c>
       <c r="I19" s="199">
-        <f>IF(OR($A19="",B19=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A19))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A19)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A19))))</f>
+        <f>IF(B19="","",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),2),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),2),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),2),"")))))</f>
         <v/>
       </c>
     </row>
     <row r="20" ht="18.95" customHeight="1" s="130">
       <c r="A20" s="197">
-        <f>IFERROR(INDEX(FILTER(ROW('EVENT ASSIGNMENT'!$A$2:$A$101)-ROW('EVENT ASSIGNMENT'!$A$2)+1,(IFERROR(INT('EVENT ASSIGNMENT'!$A$2:$A$101),0)=INT($B$10))*(TRIM('EVENT ASSIGNMENT'!$F$2:$F$101)=TRIM($E$10))),3),"")</f>
+        <f>IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),3),"")</f>
         <v/>
       </c>
       <c r="B20" s="198">
-        <f>IF($A20="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A20),""))</f>
+        <f>IFERROR(INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),3),"")),"")</f>
         <v/>
       </c>
       <c r="C20" s="199">
-        <f>IF(OR($A20="",B20=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,$A20)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A20),""))</f>
+        <f>IF(B20="","",IFERROR(INDEX('CONTRACT CALC'!$G:$G,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),3),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),3),""))+11),""))</f>
         <v/>
       </c>
       <c r="D20" s="199">
-        <f>IF(OR($A20="",B20=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,$A20)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A20),""))</f>
+        <f>IF(B20="","",IFERROR(INDEX('CONTRACT CALC'!$I:$I,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),3),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),3),""))+11),""))</f>
         <v/>
       </c>
       <c r="E20" s="199">
@@ -3855,7 +3855,7 @@
         <v/>
       </c>
       <c r="F20" s="199">
-        <f>IF(OR($A20="",B20=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,$A20)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A20),""))</f>
+        <f>IF(B20="","",IFERROR(INDEX('CONTRACT CALC'!$H:$H,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),3),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),3),""))+11),""))</f>
         <v/>
       </c>
       <c r="G20" s="199">
@@ -3867,25 +3867,25 @@
         <v/>
       </c>
       <c r="I20" s="199">
-        <f>IF(OR($A20="",B20=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A20))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A20)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A20))))</f>
+        <f>IF(B20="","",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),3),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),3),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),3),"")))))</f>
         <v/>
       </c>
     </row>
     <row r="21" ht="18.95" customHeight="1" s="130">
       <c r="A21" s="197">
-        <f>IFERROR(INDEX(FILTER(ROW('EVENT ASSIGNMENT'!$A$2:$A$101)-ROW('EVENT ASSIGNMENT'!$A$2)+1,(IFERROR(INT('EVENT ASSIGNMENT'!$A$2:$A$101),0)=INT($B$10))*(TRIM('EVENT ASSIGNMENT'!$F$2:$F$101)=TRIM($E$10))),4),"")</f>
+        <f>IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),4),"")</f>
         <v/>
       </c>
       <c r="B21" s="198">
-        <f>IF($A21="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A21),""))</f>
+        <f>IFERROR(INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),4),"")),"")</f>
         <v/>
       </c>
       <c r="C21" s="199">
-        <f>IF(OR($A21="",B21=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,$A21)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A21),""))</f>
+        <f>IF(B21="","",IFERROR(INDEX('CONTRACT CALC'!$G:$G,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),4),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),4),""))+11),""))</f>
         <v/>
       </c>
       <c r="D21" s="199">
-        <f>IF(OR($A21="",B21=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,$A21)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A21),""))</f>
+        <f>IF(B21="","",IFERROR(INDEX('CONTRACT CALC'!$I:$I,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),4),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),4),""))+11),""))</f>
         <v/>
       </c>
       <c r="E21" s="199">
@@ -3893,7 +3893,7 @@
         <v/>
       </c>
       <c r="F21" s="199">
-        <f>IF(OR($A21="",B21=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,$A21)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A21),""))</f>
+        <f>IF(B21="","",IFERROR(INDEX('CONTRACT CALC'!$H:$H,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),4),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),4),""))+11),""))</f>
         <v/>
       </c>
       <c r="G21" s="199">
@@ -3905,25 +3905,25 @@
         <v/>
       </c>
       <c r="I21" s="199">
-        <f>IF(OR($A21="",B21=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A21))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A21)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A21))))</f>
+        <f>IF(B21="","",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),4),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),4),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),4),"")))))</f>
         <v/>
       </c>
     </row>
     <row r="22" ht="18.95" customHeight="1" s="130">
       <c r="A22" s="197">
-        <f>IFERROR(INDEX(FILTER(ROW('EVENT ASSIGNMENT'!$A$2:$A$101)-ROW('EVENT ASSIGNMENT'!$A$2)+1,(IFERROR(INT('EVENT ASSIGNMENT'!$A$2:$A$101),0)=INT($B$10))*(TRIM('EVENT ASSIGNMENT'!$F$2:$F$101)=TRIM($E$10))),5),"")</f>
+        <f>IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),5),"")</f>
         <v/>
       </c>
       <c r="B22" s="198">
-        <f>IF($A22="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A22),""))</f>
+        <f>IFERROR(INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),5),"")),"")</f>
         <v/>
       </c>
       <c r="C22" s="199">
-        <f>IF(OR($A22="",B22=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,$A22)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A22),""))</f>
+        <f>IF(B22="","",IFERROR(INDEX('CONTRACT CALC'!$G:$G,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),5),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),5),""))+11),""))</f>
         <v/>
       </c>
       <c r="D22" s="199">
-        <f>IF(OR($A22="",B22=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,$A22)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A22),""))</f>
+        <f>IF(B22="","",IFERROR(INDEX('CONTRACT CALC'!$I:$I,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),5),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),5),""))+11),""))</f>
         <v/>
       </c>
       <c r="E22" s="199">
@@ -3931,7 +3931,7 @@
         <v/>
       </c>
       <c r="F22" s="199">
-        <f>IF(OR($A22="",B22=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,$A22)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A22),""))</f>
+        <f>IF(B22="","",IFERROR(INDEX('CONTRACT CALC'!$H:$H,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),5),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),5),""))+11),""))</f>
         <v/>
       </c>
       <c r="G22" s="199">
@@ -3943,25 +3943,25 @@
         <v/>
       </c>
       <c r="I22" s="199">
-        <f>IF(OR($A22="",B22=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A22))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A22)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A22))))</f>
+        <f>IF(B22="","",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),5),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),5),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),5),"")))))</f>
         <v/>
       </c>
     </row>
     <row r="23" ht="20.1" customHeight="1" s="130">
       <c r="A23" s="197">
-        <f>IFERROR(INDEX(FILTER(ROW('EVENT ASSIGNMENT'!$A$2:$A$101)-ROW('EVENT ASSIGNMENT'!$A$2)+1,(IFERROR(INT('EVENT ASSIGNMENT'!$A$2:$A$101),0)=INT($B$10))*(TRIM('EVENT ASSIGNMENT'!$F$2:$F$101)=TRIM($E$10))),6),"")</f>
+        <f>IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),6),"")</f>
         <v/>
       </c>
       <c r="B23" s="198">
-        <f>IF($A23="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A23),""))</f>
+        <f>IFERROR(INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),6),"")),"")</f>
         <v/>
       </c>
       <c r="C23" s="199">
-        <f>IF(OR($A23="",B23=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,$A23)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A23),""))</f>
+        <f>IF(B23="","",IFERROR(INDEX('CONTRACT CALC'!$G:$G,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),6),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),6),""))+11),""))</f>
         <v/>
       </c>
       <c r="D23" s="199">
-        <f>IF(OR($A23="",B23=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,$A23)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A23),""))</f>
+        <f>IF(B23="","",IFERROR(INDEX('CONTRACT CALC'!$I:$I,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),6),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),6),""))+11),""))</f>
         <v/>
       </c>
       <c r="E23" s="199">
@@ -3969,7 +3969,7 @@
         <v/>
       </c>
       <c r="F23" s="199">
-        <f>IF(OR($A23="",B23=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,$A23)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A23),""))</f>
+        <f>IF(B23="","",IFERROR(INDEX('CONTRACT CALC'!$H:$H,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),6),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),6),""))+11),""))</f>
         <v/>
       </c>
       <c r="G23" s="199">
@@ -3981,25 +3981,25 @@
         <v/>
       </c>
       <c r="I23" s="199">
-        <f>IF(OR($A23="",B23=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A23))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A23)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A23))))</f>
+        <f>IF(B23="","",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),6),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),6),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),6),"")))))</f>
         <v/>
       </c>
     </row>
     <row r="24" ht="17.1" customHeight="1" s="130">
       <c r="A24" s="197">
-        <f>IFERROR(INDEX(FILTER(ROW('EVENT ASSIGNMENT'!$A$2:$A$101)-ROW('EVENT ASSIGNMENT'!$A$2)+1,(IFERROR(INT('EVENT ASSIGNMENT'!$A$2:$A$101),0)=INT($B$10))*(TRIM('EVENT ASSIGNMENT'!$F$2:$F$101)=TRIM($E$10))),7),"")</f>
+        <f>IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),7),"")</f>
         <v/>
       </c>
       <c r="B24" s="198">
-        <f>IF($A24="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A24),""))</f>
+        <f>IFERROR(INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),7),"")),"")</f>
         <v/>
       </c>
       <c r="C24" s="199">
-        <f>IF(OR($A24="",B24=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,$A24)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A24),""))</f>
+        <f>IF(B24="","",IFERROR(INDEX('CONTRACT CALC'!$G:$G,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),7),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),7),""))+11),""))</f>
         <v/>
       </c>
       <c r="D24" s="199">
-        <f>IF(OR($A24="",B24=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,$A24)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A24),""))</f>
+        <f>IF(B24="","",IFERROR(INDEX('CONTRACT CALC'!$I:$I,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),7),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),7),""))+11),""))</f>
         <v/>
       </c>
       <c r="E24" s="199">
@@ -4007,7 +4007,7 @@
         <v/>
       </c>
       <c r="F24" s="199">
-        <f>IF(OR($A24="",B24=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,$A24)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A24),""))</f>
+        <f>IF(B24="","",IFERROR(INDEX('CONTRACT CALC'!$H:$H,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),7),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),7),""))+11),""))</f>
         <v/>
       </c>
       <c r="G24" s="199">
@@ -4019,25 +4019,25 @@
         <v/>
       </c>
       <c r="I24" s="199">
-        <f>IF(OR($A24="",B24=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A24))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A24)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A24))))</f>
+        <f>IF(B24="","",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),7),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),7),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),7),"")))))</f>
         <v/>
       </c>
     </row>
     <row r="25" ht="20.1" customHeight="1" s="130">
       <c r="A25" s="197">
-        <f>IFERROR(INDEX(FILTER(ROW('EVENT ASSIGNMENT'!$A$2:$A$101)-ROW('EVENT ASSIGNMENT'!$A$2)+1,(IFERROR(INT('EVENT ASSIGNMENT'!$A$2:$A$101),0)=INT($B$10))*(TRIM('EVENT ASSIGNMENT'!$F$2:$F$101)=TRIM($E$10))),8),"")</f>
+        <f>IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),8),"")</f>
         <v/>
       </c>
       <c r="B25" s="198">
-        <f>IF($A25="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A25),""))</f>
+        <f>IFERROR(INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),8),"")),"")</f>
         <v/>
       </c>
       <c r="C25" s="199">
-        <f>IF(OR($A25="",B25=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,$A25)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A25),""))</f>
+        <f>IF(B25="","",IFERROR(INDEX('CONTRACT CALC'!$G:$G,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),8),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),8),""))+11),""))</f>
         <v/>
       </c>
       <c r="D25" s="199">
-        <f>IF(OR($A25="",B25=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,$A25)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A25),""))</f>
+        <f>IF(B25="","",IFERROR(INDEX('CONTRACT CALC'!$I:$I,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),8),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),8),""))+11),""))</f>
         <v/>
       </c>
       <c r="E25" s="199">
@@ -4045,7 +4045,7 @@
         <v/>
       </c>
       <c r="F25" s="199">
-        <f>IF(OR($A25="",B25=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,$A25)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A25),""))</f>
+        <f>IF(B25="","",IFERROR(INDEX('CONTRACT CALC'!$H:$H,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),8),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),8),""))+11),""))</f>
         <v/>
       </c>
       <c r="G25" s="200">
@@ -4057,25 +4057,25 @@
         <v/>
       </c>
       <c r="I25" s="199">
-        <f>IF(OR($A25="",B25=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A25))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A25)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A25))))</f>
+        <f>IF(B25="","",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),8),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),8),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),8),"")))))</f>
         <v/>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1" s="130">
       <c r="A26" s="197">
-        <f>IFERROR(INDEX(FILTER(ROW('EVENT ASSIGNMENT'!$A$2:$A$101)-ROW('EVENT ASSIGNMENT'!$A$2)+1,(IFERROR(INT('EVENT ASSIGNMENT'!$A$2:$A$101),0)=INT($B$10))*(TRIM('EVENT ASSIGNMENT'!$F$2:$F$101)=TRIM($E$10))),9),"")</f>
+        <f>IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),9),"")</f>
         <v/>
       </c>
       <c r="B26" s="198">
-        <f>IF($A26="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A26),""))</f>
+        <f>IFERROR(INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),9),"")),"")</f>
         <v/>
       </c>
       <c r="C26" s="199">
-        <f>IF(OR($A26="",B26=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,$A26)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A26),""))</f>
+        <f>IF(B26="","",IFERROR(INDEX('CONTRACT CALC'!$G:$G,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),9),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),9),""))+11),""))</f>
         <v/>
       </c>
       <c r="D26" s="199">
-        <f>IF(OR($A26="",B26=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,$A26)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A26),""))</f>
+        <f>IF(B26="","",IFERROR(INDEX('CONTRACT CALC'!$I:$I,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),9),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),9),""))+11),""))</f>
         <v/>
       </c>
       <c r="E26" s="199">
@@ -4083,7 +4083,7 @@
         <v/>
       </c>
       <c r="F26" s="199">
-        <f>IF(OR($A26="",B26=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,$A26)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A26),""))</f>
+        <f>IF(B26="","",IFERROR(INDEX('CONTRACT CALC'!$H:$H,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),9),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),9),""))+11),""))</f>
         <v/>
       </c>
       <c r="G26" s="199">
@@ -4095,25 +4095,25 @@
         <v/>
       </c>
       <c r="I26" s="199">
-        <f>IF(OR($A26="",B26=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A26))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A26)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A26))))</f>
+        <f>IF(B26="","",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),9),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),9),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),9),"")))))</f>
         <v/>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1" s="130">
       <c r="A27" s="197">
-        <f>IFERROR(INDEX(FILTER(ROW('EVENT ASSIGNMENT'!$A$2:$A$101)-ROW('EVENT ASSIGNMENT'!$A$2)+1,(IFERROR(INT('EVENT ASSIGNMENT'!$A$2:$A$101),0)=INT($B$10))*(TRIM('EVENT ASSIGNMENT'!$F$2:$F$101)=TRIM($E$10))),10),"")</f>
+        <f>IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),10),"")</f>
         <v/>
       </c>
       <c r="B27" s="198">
-        <f>IF($A27="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A27),""))</f>
+        <f>IFERROR(INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),10),"")),"")</f>
         <v/>
       </c>
       <c r="C27" s="199">
-        <f>IF(OR($A27="",B27=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,$A27)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A27),""))</f>
+        <f>IF(B27="","",IFERROR(INDEX('CONTRACT CALC'!$G:$G,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),10),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),10),""))+11),""))</f>
         <v/>
       </c>
       <c r="D27" s="199">
-        <f>IF(OR($A27="",B27=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,$A27)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A27),""))</f>
+        <f>IF(B27="","",IFERROR(INDEX('CONTRACT CALC'!$I:$I,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),10),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),10),""))+11),""))</f>
         <v/>
       </c>
       <c r="E27" s="199">
@@ -4121,7 +4121,7 @@
         <v/>
       </c>
       <c r="F27" s="199">
-        <f>IF(OR($A27="",B27=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,$A27)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A27),""))</f>
+        <f>IF(B27="","",IFERROR(INDEX('CONTRACT CALC'!$H:$H,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),10),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),10),""))+11),""))</f>
         <v/>
       </c>
       <c r="G27" s="199">
@@ -4133,25 +4133,25 @@
         <v/>
       </c>
       <c r="I27" s="199">
-        <f>IF(OR($A27="",B27=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A27))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A27)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A27))))</f>
+        <f>IF(B27="","",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),10),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),10),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),10),"")))))</f>
         <v/>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1" s="130">
       <c r="A28" s="197">
-        <f>IFERROR(INDEX(FILTER(ROW('EVENT ASSIGNMENT'!$A$2:$A$101)-ROW('EVENT ASSIGNMENT'!$A$2)+1,(IFERROR(INT('EVENT ASSIGNMENT'!$A$2:$A$101),0)=INT($B$10))*(TRIM('EVENT ASSIGNMENT'!$F$2:$F$101)=TRIM($E$10))),11),"")</f>
+        <f>IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),11),"")</f>
         <v/>
       </c>
       <c r="B28" s="198">
-        <f>IF($A28="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A28),""))</f>
+        <f>IFERROR(INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),11),"")),"")</f>
         <v/>
       </c>
       <c r="C28" s="199">
-        <f>IF(OR($A28="",B28=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,$A28)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A28),""))</f>
+        <f>IF(B28="","",IFERROR(INDEX('CONTRACT CALC'!$G:$G,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),11),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),11),""))+11),""))</f>
         <v/>
       </c>
       <c r="D28" s="199">
-        <f>IF(OR($A28="",B28=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,$A28)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A28),""))</f>
+        <f>IF(B28="","",IFERROR(INDEX('CONTRACT CALC'!$I:$I,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),11),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),11),""))+11),""))</f>
         <v/>
       </c>
       <c r="E28" s="199">
@@ -4159,7 +4159,7 @@
         <v/>
       </c>
       <c r="F28" s="199">
-        <f>IF(OR($A28="",B28=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,$A28)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A28),""))</f>
+        <f>IF(B28="","",IFERROR(INDEX('CONTRACT CALC'!$H:$H,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),11),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),11),""))+11),""))</f>
         <v/>
       </c>
       <c r="G28" s="199">
@@ -4171,25 +4171,25 @@
         <v/>
       </c>
       <c r="I28" s="199">
-        <f>IF(OR($A28="",B28=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A28))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A28)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A28))))</f>
+        <f>IF(B28="","",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),11),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),11),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),11),"")))))</f>
         <v/>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1" s="130">
       <c r="A29" s="197">
-        <f>IFERROR(INDEX(FILTER(ROW('EVENT ASSIGNMENT'!$A$2:$A$101)-ROW('EVENT ASSIGNMENT'!$A$2)+1,(IFERROR(INT('EVENT ASSIGNMENT'!$A$2:$A$101),0)=INT($B$10))*(TRIM('EVENT ASSIGNMENT'!$F$2:$F$101)=TRIM($E$10))),12),"")</f>
+        <f>IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),12),"")</f>
         <v/>
       </c>
       <c r="B29" s="198">
-        <f>IF($A29="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A29),""))</f>
+        <f>IFERROR(INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),12),"")),"")</f>
         <v/>
       </c>
       <c r="C29" s="199">
-        <f>IF(OR($A29="",B29=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,$A29)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A29),""))</f>
+        <f>IF(B29="","",IFERROR(INDEX('CONTRACT CALC'!$G:$G,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),12),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),12),""))+11),""))</f>
         <v/>
       </c>
       <c r="D29" s="199">
-        <f>IF(OR($A29="",B29=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,$A29)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A29),""))</f>
+        <f>IF(B29="","",IFERROR(INDEX('CONTRACT CALC'!$I:$I,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),12),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),12),""))+11),""))</f>
         <v/>
       </c>
       <c r="E29" s="199">
@@ -4197,7 +4197,7 @@
         <v/>
       </c>
       <c r="F29" s="199">
-        <f>IF(OR($A29="",B29=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,$A29)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A29),""))</f>
+        <f>IF(B29="","",IFERROR(INDEX('CONTRACT CALC'!$H:$H,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),12),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),12),""))+11),""))</f>
         <v/>
       </c>
       <c r="G29" s="199">
@@ -4209,25 +4209,25 @@
         <v/>
       </c>
       <c r="I29" s="199">
-        <f>IF(OR($A29="",B29=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A29))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A29)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A29))))</f>
+        <f>IF(B29="","",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),12),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),12),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),12),"")))))</f>
         <v/>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1" s="130">
       <c r="A30" s="197">
-        <f>IFERROR(INDEX(FILTER(ROW('EVENT ASSIGNMENT'!$A$2:$A$101)-ROW('EVENT ASSIGNMENT'!$A$2)+1,(IFERROR(INT('EVENT ASSIGNMENT'!$A$2:$A$101),0)=INT($B$10))*(TRIM('EVENT ASSIGNMENT'!$F$2:$F$101)=TRIM($E$10))),13),"")</f>
+        <f>IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),13),"")</f>
         <v/>
       </c>
       <c r="B30" s="198">
-        <f>IF($A30="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A30),""))</f>
+        <f>IFERROR(INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),13),"")),"")</f>
         <v/>
       </c>
       <c r="C30" s="199">
-        <f>IF(OR($A30="",B30=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,$A30)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A30),""))</f>
+        <f>IF(B30="","",IFERROR(INDEX('CONTRACT CALC'!$G:$G,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),13),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),13),""))+11),""))</f>
         <v/>
       </c>
       <c r="D30" s="199">
-        <f>IF(OR($A30="",B30=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,$A30)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A30),""))</f>
+        <f>IF(B30="","",IFERROR(INDEX('CONTRACT CALC'!$I:$I,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),13),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),13),""))+11),""))</f>
         <v/>
       </c>
       <c r="E30" s="199">
@@ -4235,7 +4235,7 @@
         <v/>
       </c>
       <c r="F30" s="199">
-        <f>IF(OR($A30="",B30=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,$A30)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A30),""))</f>
+        <f>IF(B30="","",IFERROR(INDEX('CONTRACT CALC'!$H:$H,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),13),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),13),""))+11),""))</f>
         <v/>
       </c>
       <c r="G30" s="199">
@@ -4247,25 +4247,25 @@
         <v/>
       </c>
       <c r="I30" s="199">
-        <f>IF(OR($A30="",B30=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A30))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A30)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A30))))</f>
+        <f>IF(B30="","",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),13),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),13),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),13),"")))))</f>
         <v/>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1" s="130" thickBot="1">
       <c r="A31" s="197">
-        <f>IFERROR(INDEX(FILTER(ROW('EVENT ASSIGNMENT'!$A$2:$A$101)-ROW('EVENT ASSIGNMENT'!$A$2)+1,(IFERROR(INT('EVENT ASSIGNMENT'!$A$2:$A$101),0)=INT($B$10))*(TRIM('EVENT ASSIGNMENT'!$F$2:$F$101)=TRIM($E$10))),14),"")</f>
+        <f>IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),14),"")</f>
         <v/>
       </c>
       <c r="B31" s="198">
-        <f>IF($A31="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A31),""))</f>
+        <f>IFERROR(INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),14),"")),"")</f>
         <v/>
       </c>
       <c r="C31" s="199">
-        <f>IF(OR($A31="",B31=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,$A31)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A31),""))</f>
+        <f>IF(B31="","",IFERROR(INDEX('CONTRACT CALC'!$G:$G,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),14),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),14),""))+11),""))</f>
         <v/>
       </c>
       <c r="D31" s="199">
-        <f>IF(OR($A31="",B31=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,$A31)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A31),""))</f>
+        <f>IF(B31="","",IFERROR(INDEX('CONTRACT CALC'!$I:$I,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),14),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),14),""))+11),""))</f>
         <v/>
       </c>
       <c r="E31" s="199">
@@ -4273,7 +4273,7 @@
         <v/>
       </c>
       <c r="F31" s="199">
-        <f>IF(OR($A31="",B31=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,$A31)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A31),""))</f>
+        <f>IF(B31="","",IFERROR(INDEX('CONTRACT CALC'!$H:$H,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),14),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),14),""))+11),""))</f>
         <v/>
       </c>
       <c r="G31" s="199">
@@ -4285,25 +4285,25 @@
         <v/>
       </c>
       <c r="I31" s="199">
-        <f>IF(OR($A31="",B31=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A31))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A31)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A31))))</f>
+        <f>IF(B31="","",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),14),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),14),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),14),"")))))</f>
         <v/>
       </c>
     </row>
     <row r="32" ht="20.25" customHeight="1" s="130">
       <c r="A32" s="197">
-        <f>IFERROR(INDEX(FILTER(ROW('EVENT ASSIGNMENT'!$A$2:$A$101)-ROW('EVENT ASSIGNMENT'!$A$2)+1,(IFERROR(INT('EVENT ASSIGNMENT'!$A$2:$A$101),0)=INT($B$10))*(TRIM('EVENT ASSIGNMENT'!$F$2:$F$101)=TRIM($E$10))),15),"")</f>
+        <f>IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),15),"")</f>
         <v/>
       </c>
       <c r="B32" s="201">
-        <f>IF($A32="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A32),""))</f>
+        <f>IFERROR(INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),15),"")),"")</f>
         <v/>
       </c>
       <c r="C32" s="202">
-        <f>IF(OR($A32="",B32=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,$A32)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A32),""))</f>
+        <f>IF(B32="","",IFERROR(INDEX('CONTRACT CALC'!$G:$G,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),15),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),15),""))+11),""))</f>
         <v/>
       </c>
       <c r="D32" s="202">
-        <f>IF(OR($A32="",B32=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,$A32)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A32),""))</f>
+        <f>IF(B32="","",IFERROR(INDEX('CONTRACT CALC'!$I:$I,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),15),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),15),""))+11),""))</f>
         <v/>
       </c>
       <c r="E32" s="202">
@@ -4311,7 +4311,7 @@
         <v/>
       </c>
       <c r="F32" s="199">
-        <f>IF(OR($A32="",B32=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,$A32)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A32),""))</f>
+        <f>IF(B32="","",IFERROR(INDEX('CONTRACT CALC'!$H:$H,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),15),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),15),""))+11),""))</f>
         <v/>
       </c>
       <c r="G32" s="202">
@@ -4323,25 +4323,25 @@
         <v/>
       </c>
       <c r="I32" s="202">
-        <f>IF(OR($A32="",B32=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A32))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A32)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A32))))</f>
+        <f>IF(B32="","",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),15),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),15),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),15),"")))))</f>
         <v/>
       </c>
     </row>
     <row r="33" ht="6" customHeight="1" s="130">
       <c r="A33" s="197">
-        <f>IFERROR(INDEX(FILTER(ROW('EVENT ASSIGNMENT'!$A$2:$A$101)-ROW('EVENT ASSIGNMENT'!$A$2)+1,(IFERROR(INT('EVENT ASSIGNMENT'!$A$2:$A$101),0)=INT($B$10))*(TRIM('EVENT ASSIGNMENT'!$F$2:$F$101)=TRIM($E$10))),16),"")</f>
+        <f>IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),16),"")</f>
         <v/>
       </c>
       <c r="B33" s="203">
-        <f>IF($A33="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A33),""))</f>
+        <f>IFERROR(INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),16),"")),"")</f>
         <v/>
       </c>
       <c r="C33" s="204">
-        <f>IF(OR($A33="",B33=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,$A33)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A33),""))</f>
+        <f>IF(B33="","",IFERROR(INDEX('CONTRACT CALC'!$G:$G,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),16),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),16),""))+11),""))</f>
         <v/>
       </c>
       <c r="D33" s="204">
-        <f>IF(OR($A33="",B33=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,$A33)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A33),""))</f>
+        <f>IF(B33="","",IFERROR(INDEX('CONTRACT CALC'!$I:$I,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),16),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),16),""))+11),""))</f>
         <v/>
       </c>
       <c r="E33" s="204">
@@ -4349,7 +4349,7 @@
         <v/>
       </c>
       <c r="F33" s="204">
-        <f>IF(OR($A33="",B33=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,$A33)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A33),""))</f>
+        <f>IF(B33="","",IFERROR(INDEX('CONTRACT CALC'!$H:$H,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),16),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),16),""))+11),""))</f>
         <v/>
       </c>
       <c r="G33" s="204">
@@ -4361,25 +4361,25 @@
         <v/>
       </c>
       <c r="I33" s="204">
-        <f>IF(OR($A33="",B33=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A33))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A33)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A33))))</f>
+        <f>IF(B33="","",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),16),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),16),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),16),"")))))</f>
         <v/>
       </c>
     </row>
     <row r="34" ht="13.5" customHeight="1" s="130" thickBot="1">
       <c r="A34" s="197">
-        <f>IFERROR(INDEX(FILTER(ROW('EVENT ASSIGNMENT'!$A$2:$A$101)-ROW('EVENT ASSIGNMENT'!$A$2)+1,(IFERROR(INT('EVENT ASSIGNMENT'!$A$2:$A$101),0)=INT($B$10))*(TRIM('EVENT ASSIGNMENT'!$F$2:$F$101)=TRIM($E$10))),17),"")</f>
+        <f>IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),17),"")</f>
         <v/>
       </c>
       <c r="B34" s="201">
-        <f>IF($A34="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A34),""))</f>
+        <f>IFERROR(INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),17),"")),"")</f>
         <v/>
       </c>
       <c r="C34" s="202">
-        <f>IF(OR($A34="",B34=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,$A34)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A34),""))</f>
+        <f>IF(B34="","",IFERROR(INDEX('CONTRACT CALC'!$G:$G,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),17),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),17),""))+11),""))</f>
         <v/>
       </c>
       <c r="D34" s="202">
-        <f>IF(OR($A34="",B34=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,$A34)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A34),""))</f>
+        <f>IF(B34="","",IFERROR(INDEX('CONTRACT CALC'!$I:$I,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),17),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),17),""))+11),""))</f>
         <v/>
       </c>
       <c r="E34" s="202">
@@ -4387,7 +4387,7 @@
         <v/>
       </c>
       <c r="F34" s="202">
-        <f>IF(OR($A34="",B34=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,$A34)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A34),""))</f>
+        <f>IF(B34="","",IFERROR(INDEX('CONTRACT CALC'!$H:$H,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),17),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),17),""))+11),""))</f>
         <v/>
       </c>
       <c r="G34" s="202">
@@ -4399,25 +4399,25 @@
         <v/>
       </c>
       <c r="I34" s="202">
-        <f>IF(OR($A34="",B34=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A34))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A34)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A34))))</f>
+        <f>IF(B34="","",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),17),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),17),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),17),"")))))</f>
         <v/>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1" s="130" thickBot="1">
       <c r="A35" s="197">
-        <f>IFERROR(INDEX(FILTER(ROW('EVENT ASSIGNMENT'!$A$2:$A$101)-ROW('EVENT ASSIGNMENT'!$A$2)+1,(IFERROR(INT('EVENT ASSIGNMENT'!$A$2:$A$101),0)=INT($B$10))*(TRIM('EVENT ASSIGNMENT'!$F$2:$F$101)=TRIM($E$10))),18),"")</f>
+        <f>IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),18),"")</f>
         <v/>
       </c>
       <c r="B35" s="205">
-        <f>IF($A35="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A35),""))</f>
+        <f>IFERROR(INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),18),"")),"")</f>
         <v/>
       </c>
       <c r="C35" s="199">
-        <f>IF(OR($A35="",B35=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,$A35)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A35),""))</f>
+        <f>IF(B35="","",IFERROR(INDEX('CONTRACT CALC'!$G:$G,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),18),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),18),""))+11),""))</f>
         <v/>
       </c>
       <c r="D35" s="199">
-        <f>IF(OR($A35="",B35=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,$A35)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A35),""))</f>
+        <f>IF(B35="","",IFERROR(INDEX('CONTRACT CALC'!$I:$I,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),18),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),18),""))+11),""))</f>
         <v/>
       </c>
       <c r="E35" s="206">
@@ -4425,7 +4425,7 @@
         <v/>
       </c>
       <c r="F35" s="199">
-        <f>IF(OR($A35="",B35=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,$A35)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A35),""))</f>
+        <f>IF(B35="","",IFERROR(INDEX('CONTRACT CALC'!$H:$H,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),18),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),18),""))+11),""))</f>
         <v/>
       </c>
       <c r="G35" s="199">
@@ -4437,25 +4437,25 @@
         <v/>
       </c>
       <c r="I35" s="199">
-        <f>IF(OR($A35="",B35=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A35))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A35)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A35))))</f>
+        <f>IF(B35="","",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),18),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),18),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),18),"")))))</f>
         <v/>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1" s="130">
       <c r="A36" s="197">
-        <f>IFERROR(INDEX(FILTER(ROW('EVENT ASSIGNMENT'!$A$2:$A$101)-ROW('EVENT ASSIGNMENT'!$A$2)+1,(IFERROR(INT('EVENT ASSIGNMENT'!$A$2:$A$101),0)=INT($B$10))*(TRIM('EVENT ASSIGNMENT'!$F$2:$F$101)=TRIM($E$10))),19),"")</f>
+        <f>IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),19),"")</f>
         <v/>
       </c>
       <c r="B36" s="198">
-        <f>IF($A36="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A36),""))</f>
+        <f>IFERROR(INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),19),"")),"")</f>
         <v/>
       </c>
       <c r="C36" s="199">
-        <f>IF(OR($A36="",B36=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,$A36)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A36),""))</f>
+        <f>IF(B36="","",IFERROR(INDEX('CONTRACT CALC'!$G:$G,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),19),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),19),""))+11),""))</f>
         <v/>
       </c>
       <c r="D36" s="199">
-        <f>IF(OR($A36="",B36=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,$A36)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A36),""))</f>
+        <f>IF(B36="","",IFERROR(INDEX('CONTRACT CALC'!$I:$I,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),19),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),19),""))+11),""))</f>
         <v/>
       </c>
       <c r="E36" s="207">
@@ -4463,7 +4463,7 @@
         <v/>
       </c>
       <c r="F36" s="207">
-        <f>IF(OR($A36="",B36=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,$A36)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A36),""))</f>
+        <f>IF(B36="","",IFERROR(INDEX('CONTRACT CALC'!$H:$H,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),19),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),19),""))+11),""))</f>
         <v/>
       </c>
       <c r="G36" s="207">
@@ -4475,25 +4475,25 @@
         <v/>
       </c>
       <c r="I36" s="199">
-        <f>IF(OR($A36="",B36=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A36))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A36)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A36))))</f>
+        <f>IF(B36="","",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),19),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),19),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),19),"")))))</f>
         <v/>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1" s="130">
       <c r="A37" s="197">
-        <f>IFERROR(INDEX(FILTER(ROW('EVENT ASSIGNMENT'!$A$2:$A$101)-ROW('EVENT ASSIGNMENT'!$A$2)+1,(IFERROR(INT('EVENT ASSIGNMENT'!$A$2:$A$101),0)=INT($B$10))*(TRIM('EVENT ASSIGNMENT'!$F$2:$F$101)=TRIM($E$10))),20),"")</f>
+        <f>IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),20),"")</f>
         <v/>
       </c>
       <c r="B37" s="198">
-        <f>IF($A37="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A37),""))</f>
+        <f>IFERROR(INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),20),"")),"")</f>
         <v/>
       </c>
       <c r="C37" s="199">
-        <f>IF(OR($A37="",B37=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,$A37)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A37),""))</f>
+        <f>IF(B37="","",IFERROR(INDEX('CONTRACT CALC'!$G:$G,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),20),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),20),""))+11),""))</f>
         <v/>
       </c>
       <c r="D37" s="199">
-        <f>IF(OR($A37="",B37=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,$A37)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A37),""))</f>
+        <f>IF(B37="","",IFERROR(INDEX('CONTRACT CALC'!$I:$I,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),20),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),20),""))+11),""))</f>
         <v/>
       </c>
       <c r="E37" s="199">
@@ -4501,7 +4501,7 @@
         <v/>
       </c>
       <c r="F37" s="199">
-        <f>IF(OR($A37="",B37=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,$A37)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A37),""))</f>
+        <f>IF(B37="","",IFERROR(INDEX('CONTRACT CALC'!$H:$H,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),20),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),20),""))+11),""))</f>
         <v/>
       </c>
       <c r="G37" s="199">
@@ -4513,25 +4513,25 @@
         <v/>
       </c>
       <c r="I37" s="199">
-        <f>IF(OR($A37="",B37=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A37))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A37)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A37))))</f>
+        <f>IF(B37="","",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),20),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),20),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),20),"")))))</f>
         <v/>
       </c>
     </row>
     <row r="38" ht="16.5" customHeight="1" s="130">
       <c r="A38" s="197">
-        <f>IFERROR(INDEX(FILTER(ROW('EVENT ASSIGNMENT'!$A$2:$A$101)-ROW('EVENT ASSIGNMENT'!$A$2)+1,(IFERROR(INT('EVENT ASSIGNMENT'!$A$2:$A$101),0)=INT($B$10))*(TRIM('EVENT ASSIGNMENT'!$F$2:$F$101)=TRIM($E$10))),21),"")</f>
+        <f>IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),21),"")</f>
         <v/>
       </c>
       <c r="B38" s="198">
-        <f>IF($A38="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A38),""))</f>
+        <f>IFERROR(INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),21),"")),"")</f>
         <v/>
       </c>
       <c r="C38" s="199">
-        <f>IF(OR($A38="",B38=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,$A38)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A38),""))</f>
+        <f>IF(B38="","",IFERROR(INDEX('CONTRACT CALC'!$G:$G,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),21),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),21),""))+11),""))</f>
         <v/>
       </c>
       <c r="D38" s="199">
-        <f>IF(OR($A38="",B38=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,$A38)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A38),""))</f>
+        <f>IF(B38="","",IFERROR(INDEX('CONTRACT CALC'!$I:$I,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),21),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),21),""))+11),""))</f>
         <v/>
       </c>
       <c r="E38" s="207">
@@ -4539,7 +4539,7 @@
         <v/>
       </c>
       <c r="F38" s="207">
-        <f>IF(OR($A38="",B38=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,$A38)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A38),""))</f>
+        <f>IF(B38="","",IFERROR(INDEX('CONTRACT CALC'!$H:$H,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),21),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),21),""))+11),""))</f>
         <v/>
       </c>
       <c r="G38" s="207">
@@ -4551,25 +4551,25 @@
         <v/>
       </c>
       <c r="I38" s="199">
-        <f>IF(OR($A38="",B38=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A38))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A38)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A38))))</f>
+        <f>IF(B38="","",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),21),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),21),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),21),"")))))</f>
         <v/>
       </c>
     </row>
     <row r="39" ht="20.1" customHeight="1" s="130">
       <c r="A39" s="208">
-        <f>IFERROR(INDEX(FILTER(ROW('EVENT ASSIGNMENT'!$A$2:$A$101)-ROW('EVENT ASSIGNMENT'!$A$2)+1,(IFERROR(INT('EVENT ASSIGNMENT'!$A$2:$A$101),0)=INT($B$10))*(TRIM('EVENT ASSIGNMENT'!$F$2:$F$101)=TRIM($E$10))),22),"")</f>
+        <f>IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),22),"")</f>
         <v/>
       </c>
       <c r="B39" s="198">
-        <f>IF($A39="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A39),""))</f>
+        <f>IFERROR(INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),22),"")),"")</f>
         <v/>
       </c>
       <c r="C39" s="199">
-        <f>IF(OR($A39="",B39=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,$A39)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A39),""))</f>
+        <f>IF(B39="","",IFERROR(INDEX('CONTRACT CALC'!$G:$G,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),22),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),22),""))+11),""))</f>
         <v/>
       </c>
       <c r="D39" s="199">
-        <f>IF(OR($A39="",B39=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,$A39)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A39),""))</f>
+        <f>IF(B39="","",IFERROR(INDEX('CONTRACT CALC'!$I:$I,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),22),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),22),""))+11),""))</f>
         <v/>
       </c>
       <c r="E39" s="199">
@@ -4577,7 +4577,7 @@
         <v/>
       </c>
       <c r="F39" s="199">
-        <f>IF(OR($A39="",B39=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,$A39)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A39),""))</f>
+        <f>IF(B39="","",IFERROR(INDEX('CONTRACT CALC'!$H:$H,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),22),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),22),""))+11),""))</f>
         <v/>
       </c>
       <c r="G39" s="199">
@@ -4589,25 +4589,25 @@
         <v/>
       </c>
       <c r="I39" s="199">
-        <f>IF(OR($A39="",B39=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A39))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A39)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A39))))</f>
+        <f>IF(B39="","",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),22),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),22),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),22),"")))))</f>
         <v/>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="208">
-        <f>IFERROR(INDEX(FILTER(ROW('EVENT ASSIGNMENT'!$A$2:$A$101)-ROW('EVENT ASSIGNMENT'!$A$2)+1,(IFERROR(INT('EVENT ASSIGNMENT'!$A$2:$A$101),0)=INT($B$10))*(TRIM('EVENT ASSIGNMENT'!$F$2:$F$101)=TRIM($E$10))),23),"")</f>
+        <f>IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),23),"")</f>
         <v/>
       </c>
       <c r="B40" s="198">
-        <f>IF($A40="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A40),""))</f>
+        <f>IFERROR(INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),23),"")),"")</f>
         <v/>
       </c>
       <c r="C40" s="199">
-        <f>IF(OR($A40="",B40=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,$A40)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A40),""))</f>
+        <f>IF(B40="","",IFERROR(INDEX('CONTRACT CALC'!$G:$G,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),23),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),23),""))+11),""))</f>
         <v/>
       </c>
       <c r="D40" s="199">
-        <f>IF(OR($A40="",B40=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,$A40)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A40),""))</f>
+        <f>IF(B40="","",IFERROR(INDEX('CONTRACT CALC'!$I:$I,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),23),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),23),""))+11),""))</f>
         <v/>
       </c>
       <c r="E40" s="199">
@@ -4615,7 +4615,7 @@
         <v/>
       </c>
       <c r="F40" s="199">
-        <f>IF(OR($A40="",B40=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,$A40)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A40),""))</f>
+        <f>IF(B40="","",IFERROR(INDEX('CONTRACT CALC'!$H:$H,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),23),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),23),""))+11),""))</f>
         <v/>
       </c>
       <c r="G40" s="199">
@@ -4627,25 +4627,25 @@
         <v/>
       </c>
       <c r="I40" s="199">
-        <f>IF(OR($A40="",B40=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A40))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A40)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A40))))</f>
+        <f>IF(B40="","",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),23),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),23),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),23),"")))))</f>
         <v/>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="130">
       <c r="A41" s="208">
-        <f>IFERROR(INDEX(FILTER(ROW('EVENT ASSIGNMENT'!$A$2:$A$101)-ROW('EVENT ASSIGNMENT'!$A$2)+1,(IFERROR(INT('EVENT ASSIGNMENT'!$A$2:$A$101),0)=INT($B$10))*(TRIM('EVENT ASSIGNMENT'!$F$2:$F$101)=TRIM($E$10))),24),"")</f>
+        <f>IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),24),"")</f>
         <v/>
       </c>
       <c r="B41" s="198">
-        <f>IF($A41="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A41),""))</f>
+        <f>IFERROR(INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),24),"")),"")</f>
         <v/>
       </c>
       <c r="C41" s="199">
-        <f>IF(OR($A41="",B41=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,$A41)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A41),""))</f>
+        <f>IF(B41="","",IFERROR(INDEX('CONTRACT CALC'!$G:$G,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),24),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),24),""))+11),""))</f>
         <v/>
       </c>
       <c r="D41" s="199">
-        <f>IF(OR($A41="",B41=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,$A41)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A41),""))</f>
+        <f>IF(B41="","",IFERROR(INDEX('CONTRACT CALC'!$I:$I,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),24),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),24),""))+11),""))</f>
         <v/>
       </c>
       <c r="E41" s="199">
@@ -4653,7 +4653,7 @@
         <v/>
       </c>
       <c r="F41" s="199">
-        <f>IF(OR($A41="",B41=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,$A41)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A41),""))</f>
+        <f>IF(B41="","",IFERROR(INDEX('CONTRACT CALC'!$H:$H,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),24),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),24),""))+11),""))</f>
         <v/>
       </c>
       <c r="G41" s="199">
@@ -4665,25 +4665,25 @@
         <v/>
       </c>
       <c r="I41" s="199">
-        <f>IF(OR($A41="",B41=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A41))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A41)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A41))))</f>
+        <f>IF(B41="","",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),24),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),24),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),24),"")))))</f>
         <v/>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="208">
-        <f>IFERROR(INDEX(FILTER(ROW('EVENT ASSIGNMENT'!$A$2:$A$101)-ROW('EVENT ASSIGNMENT'!$A$2)+1,(IFERROR(INT('EVENT ASSIGNMENT'!$A$2:$A$101),0)=INT($B$10))*(TRIM('EVENT ASSIGNMENT'!$F$2:$F$101)=TRIM($E$10))),25),"")</f>
+        <f>IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),25),"")</f>
         <v/>
       </c>
       <c r="B42" s="198">
-        <f>IF($A42="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A42),""))</f>
+        <f>IFERROR(INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),25),"")),"")</f>
         <v/>
       </c>
       <c r="C42" s="199">
-        <f>IF(OR($A42="",B42=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,$A42)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A42),""))</f>
+        <f>IF(B42="","",IFERROR(INDEX('CONTRACT CALC'!$G:$G,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),25),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),25),""))+11),""))</f>
         <v/>
       </c>
       <c r="D42" s="199">
-        <f>IF(OR($A42="",B42=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,$A42)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A42),""))</f>
+        <f>IF(B42="","",IFERROR(INDEX('CONTRACT CALC'!$I:$I,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),25),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),25),""))+11),""))</f>
         <v/>
       </c>
       <c r="E42" s="199">
@@ -4691,7 +4691,7 @@
         <v/>
       </c>
       <c r="F42" s="199">
-        <f>IF(OR($A42="",B42=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,$A42)*INDEX('CONTRACT CALC'!$F$13:$F$112,$A42),""))</f>
+        <f>IF(B42="","",IFERROR(INDEX('CONTRACT CALC'!$H:$H,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),25),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),25),""))+11),""))</f>
         <v/>
       </c>
       <c r="G42" s="199">
@@ -4703,7 +4703,7 @@
         <v/>
       </c>
       <c r="I42" s="199">
-        <f>IF(OR($A42="",B42=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A42))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,$A42)),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,$A42))))</f>
+        <f>IF(B42="","",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),25),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),25),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),25),"")))))</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Use INDEX/MATCH payout keys so ARVC locations populate in Excel
Add EVENT ASSIGNMENT seq/lookup-key helpers and drive VENDOR PAYOUT
detail rows with plain INDEX/MATCH (no FILTER/AGGREGATE arrays). This
avoids Excel repair dropping formulas and blanking the settlement.

Co-authored-by: unmegonzales <unmegonzales@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/npo-payout/NPO_Payout_Vendor_Template.xlsx
+++ b/npo-payout/NPO_Payout_Vendor_Template.xlsx
@@ -361,6 +361,11 @@
     <font>
       <name val="Aptos"/>
       <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Aptos"/>
+      <b val="1"/>
       <color rgb="FF17365D"/>
       <sz val="16"/>
     </font>
@@ -414,11 +419,6 @@
       <b val="1"/>
       <color rgb="FF17365D"/>
       <sz val="12"/>
-    </font>
-    <font>
-      <name val="Aptos"/>
-      <b val="1"/>
-      <sz val="10"/>
     </font>
     <font>
       <name val="Aptos"/>
@@ -1571,89 +1571,89 @@
     <xf numFmtId="167" fontId="34" fillId="15" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="49" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="47" fillId="10" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="50" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="48" fillId="10" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="48" fillId="11" borderId="38" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="49" fillId="11" borderId="38" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="49" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="175" fontId="50" fillId="11" borderId="39" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="175" fontId="51" fillId="11" borderId="39" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="51" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="52" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="48" fillId="12" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="49" fillId="12" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="174" fontId="48" fillId="19" borderId="32" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="174" fontId="49" fillId="19" borderId="32" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="48" fillId="19" borderId="32" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="49" fillId="19" borderId="32" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="49" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="51" fillId="0" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="50" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="52" fillId="0" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="51" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="52" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="51" fillId="0" borderId="43" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="52" fillId="0" borderId="43" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="52" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="52" fillId="13" borderId="54" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="53" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="53" fillId="13" borderId="54" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="52" fillId="13" borderId="54" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
+    <xf numFmtId="0" fontId="53" fillId="13" borderId="54" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="54" fillId="10" borderId="55" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="55" fillId="10" borderId="55" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="55" fillId="0" borderId="54" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="56" fillId="0" borderId="54" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="53" fillId="0" borderId="54" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="176" fontId="54" fillId="0" borderId="54" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="53" fillId="12" borderId="54" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="176" fontId="54" fillId="12" borderId="54" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="55" fillId="10" borderId="54" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="56" fillId="10" borderId="54" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="53" fillId="10" borderId="54" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="176" fontId="54" fillId="10" borderId="54" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="55" fillId="13" borderId="54" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="56" fillId="13" borderId="54" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="53" fillId="13" borderId="54" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="176" fontId="54" fillId="13" borderId="54" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="55" fillId="17" borderId="54" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="56" fillId="17" borderId="54" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="53" fillId="18" borderId="54" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="176" fontId="54" fillId="18" borderId="54" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="53" fillId="9" borderId="54" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="176" fontId="54" fillId="9" borderId="54" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="54" fillId="0" borderId="55" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="55" fillId="0" borderId="55" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="56" fillId="12" borderId="54" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="176" fontId="48" fillId="12" borderId="54" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="49" fillId="0" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="57" fillId="12" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="58" fillId="0" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="58" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="176" fontId="53" fillId="0" borderId="54" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="173" fontId="48" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="57" fillId="12" borderId="54" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="176" fontId="49" fillId="12" borderId="54" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="50" fillId="0" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="58" fillId="12" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="47" fillId="0" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="47" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="176" fontId="54" fillId="0" borderId="54" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="173" fontId="49" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="59" fillId="13" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="60" fillId="13" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="61" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -3759,19 +3759,19 @@
     </row>
     <row r="18" ht="18.95" customHeight="1" s="130">
       <c r="A18" s="197">
-        <f>IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),1),"")</f>
+        <f>IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|1",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")</f>
         <v/>
       </c>
       <c r="B18" s="198">
-        <f>IFERROR(INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),1),"")),"")</f>
+        <f>IF(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|1",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|1",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="C18" s="199">
-        <f>IF(B18="","",IFERROR(INDEX('CONTRACT CALC'!$G:$G,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),1),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),1),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|1",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B18=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|1",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|1",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="D18" s="199">
-        <f>IF(B18="","",IFERROR(INDEX('CONTRACT CALC'!$I:$I,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),1),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),1),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|1",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B18=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|1",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|1",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="E18" s="199">
@@ -3779,7 +3779,7 @@
         <v/>
       </c>
       <c r="F18" s="199">
-        <f>IF(B18="","",IFERROR(INDEX('CONTRACT CALC'!$H:$H,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),1),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),1),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|1",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B18=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|1",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|1",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="G18" s="199">
@@ -3791,25 +3791,25 @@
         <v/>
       </c>
       <c r="I18" s="199">
-        <f>IF(B18="","",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),1),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),1),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),1),"")))))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|1",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B18=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|1",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|1",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|1",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))))</f>
         <v/>
       </c>
     </row>
     <row r="19" ht="18.95" customHeight="1" s="130">
       <c r="A19" s="197">
-        <f>IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),2),"")</f>
+        <f>IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|2",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")</f>
         <v/>
       </c>
       <c r="B19" s="198">
-        <f>IFERROR(INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),2),"")),"")</f>
+        <f>IF(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|2",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|2",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="C19" s="199">
-        <f>IF(B19="","",IFERROR(INDEX('CONTRACT CALC'!$G:$G,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),2),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),2),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|2",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B19=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|2",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|2",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="D19" s="199">
-        <f>IF(B19="","",IFERROR(INDEX('CONTRACT CALC'!$I:$I,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),2),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),2),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|2",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B19=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|2",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|2",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="E19" s="199">
@@ -3817,7 +3817,7 @@
         <v/>
       </c>
       <c r="F19" s="199">
-        <f>IF(B19="","",IFERROR(INDEX('CONTRACT CALC'!$H:$H,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),2),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),2),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|2",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B19=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|2",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|2",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="G19" s="199">
@@ -3829,25 +3829,25 @@
         <v/>
       </c>
       <c r="I19" s="199">
-        <f>IF(B19="","",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),2),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),2),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),2),"")))))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|2",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B19=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|2",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|2",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|2",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))))</f>
         <v/>
       </c>
     </row>
     <row r="20" ht="18.95" customHeight="1" s="130">
       <c r="A20" s="197">
-        <f>IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),3),"")</f>
+        <f>IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|3",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")</f>
         <v/>
       </c>
       <c r="B20" s="198">
-        <f>IFERROR(INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),3),"")),"")</f>
+        <f>IF(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|3",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|3",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="C20" s="199">
-        <f>IF(B20="","",IFERROR(INDEX('CONTRACT CALC'!$G:$G,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),3),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),3),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|3",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B20=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|3",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|3",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="D20" s="199">
-        <f>IF(B20="","",IFERROR(INDEX('CONTRACT CALC'!$I:$I,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),3),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),3),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|3",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B20=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|3",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|3",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="E20" s="199">
@@ -3855,7 +3855,7 @@
         <v/>
       </c>
       <c r="F20" s="199">
-        <f>IF(B20="","",IFERROR(INDEX('CONTRACT CALC'!$H:$H,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),3),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),3),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|3",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B20=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|3",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|3",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="G20" s="199">
@@ -3867,25 +3867,25 @@
         <v/>
       </c>
       <c r="I20" s="199">
-        <f>IF(B20="","",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),3),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),3),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),3),"")))))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|3",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B20=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|3",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|3",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|3",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))))</f>
         <v/>
       </c>
     </row>
     <row r="21" ht="18.95" customHeight="1" s="130">
       <c r="A21" s="197">
-        <f>IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),4),"")</f>
+        <f>IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|4",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")</f>
         <v/>
       </c>
       <c r="B21" s="198">
-        <f>IFERROR(INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),4),"")),"")</f>
+        <f>IF(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|4",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|4",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="C21" s="199">
-        <f>IF(B21="","",IFERROR(INDEX('CONTRACT CALC'!$G:$G,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),4),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),4),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|4",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B21=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|4",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|4",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="D21" s="199">
-        <f>IF(B21="","",IFERROR(INDEX('CONTRACT CALC'!$I:$I,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),4),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),4),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|4",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B21=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|4",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|4",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="E21" s="199">
@@ -3893,7 +3893,7 @@
         <v/>
       </c>
       <c r="F21" s="199">
-        <f>IF(B21="","",IFERROR(INDEX('CONTRACT CALC'!$H:$H,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),4),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),4),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|4",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B21=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|4",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|4",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="G21" s="199">
@@ -3905,25 +3905,25 @@
         <v/>
       </c>
       <c r="I21" s="199">
-        <f>IF(B21="","",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),4),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),4),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),4),"")))))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|4",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B21=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|4",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|4",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|4",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))))</f>
         <v/>
       </c>
     </row>
     <row r="22" ht="18.95" customHeight="1" s="130">
       <c r="A22" s="197">
-        <f>IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),5),"")</f>
+        <f>IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|5",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")</f>
         <v/>
       </c>
       <c r="B22" s="198">
-        <f>IFERROR(INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),5),"")),"")</f>
+        <f>IF(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|5",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|5",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="C22" s="199">
-        <f>IF(B22="","",IFERROR(INDEX('CONTRACT CALC'!$G:$G,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),5),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),5),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|5",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B22=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|5",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|5",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="D22" s="199">
-        <f>IF(B22="","",IFERROR(INDEX('CONTRACT CALC'!$I:$I,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),5),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),5),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|5",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B22=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|5",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|5",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="E22" s="199">
@@ -3931,7 +3931,7 @@
         <v/>
       </c>
       <c r="F22" s="199">
-        <f>IF(B22="","",IFERROR(INDEX('CONTRACT CALC'!$H:$H,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),5),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),5),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|5",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B22=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|5",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|5",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="G22" s="199">
@@ -3943,25 +3943,25 @@
         <v/>
       </c>
       <c r="I22" s="199">
-        <f>IF(B22="","",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),5),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),5),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),5),"")))))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|5",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B22=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|5",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|5",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|5",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))))</f>
         <v/>
       </c>
     </row>
     <row r="23" ht="20.1" customHeight="1" s="130">
       <c r="A23" s="197">
-        <f>IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),6),"")</f>
+        <f>IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|6",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")</f>
         <v/>
       </c>
       <c r="B23" s="198">
-        <f>IFERROR(INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),6),"")),"")</f>
+        <f>IF(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|6",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|6",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="C23" s="199">
-        <f>IF(B23="","",IFERROR(INDEX('CONTRACT CALC'!$G:$G,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),6),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),6),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|6",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B23=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|6",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|6",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="D23" s="199">
-        <f>IF(B23="","",IFERROR(INDEX('CONTRACT CALC'!$I:$I,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),6),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),6),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|6",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B23=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|6",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|6",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="E23" s="199">
@@ -3969,7 +3969,7 @@
         <v/>
       </c>
       <c r="F23" s="199">
-        <f>IF(B23="","",IFERROR(INDEX('CONTRACT CALC'!$H:$H,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),6),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),6),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|6",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B23=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|6",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|6",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="G23" s="199">
@@ -3981,25 +3981,25 @@
         <v/>
       </c>
       <c r="I23" s="199">
-        <f>IF(B23="","",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),6),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),6),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),6),"")))))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|6",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B23=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|6",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|6",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|6",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))))</f>
         <v/>
       </c>
     </row>
     <row r="24" ht="17.1" customHeight="1" s="130">
       <c r="A24" s="197">
-        <f>IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),7),"")</f>
+        <f>IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|7",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")</f>
         <v/>
       </c>
       <c r="B24" s="198">
-        <f>IFERROR(INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),7),"")),"")</f>
+        <f>IF(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|7",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|7",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="C24" s="199">
-        <f>IF(B24="","",IFERROR(INDEX('CONTRACT CALC'!$G:$G,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),7),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),7),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|7",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B24=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|7",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|7",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="D24" s="199">
-        <f>IF(B24="","",IFERROR(INDEX('CONTRACT CALC'!$I:$I,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),7),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),7),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|7",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B24=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|7",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|7",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="E24" s="199">
@@ -4007,7 +4007,7 @@
         <v/>
       </c>
       <c r="F24" s="199">
-        <f>IF(B24="","",IFERROR(INDEX('CONTRACT CALC'!$H:$H,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),7),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),7),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|7",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B24=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|7",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|7",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="G24" s="199">
@@ -4019,25 +4019,25 @@
         <v/>
       </c>
       <c r="I24" s="199">
-        <f>IF(B24="","",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),7),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),7),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),7),"")))))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|7",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B24=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|7",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|7",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|7",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))))</f>
         <v/>
       </c>
     </row>
     <row r="25" ht="20.1" customHeight="1" s="130">
       <c r="A25" s="197">
-        <f>IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),8),"")</f>
+        <f>IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|8",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")</f>
         <v/>
       </c>
       <c r="B25" s="198">
-        <f>IFERROR(INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),8),"")),"")</f>
+        <f>IF(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|8",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|8",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="C25" s="199">
-        <f>IF(B25="","",IFERROR(INDEX('CONTRACT CALC'!$G:$G,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),8),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),8),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|8",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B25=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|8",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|8",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="D25" s="199">
-        <f>IF(B25="","",IFERROR(INDEX('CONTRACT CALC'!$I:$I,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),8),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),8),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|8",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B25=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|8",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|8",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="E25" s="199">
@@ -4045,7 +4045,7 @@
         <v/>
       </c>
       <c r="F25" s="199">
-        <f>IF(B25="","",IFERROR(INDEX('CONTRACT CALC'!$H:$H,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),8),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),8),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|8",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B25=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|8",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|8",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="G25" s="200">
@@ -4057,25 +4057,25 @@
         <v/>
       </c>
       <c r="I25" s="199">
-        <f>IF(B25="","",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),8),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),8),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),8),"")))))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|8",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B25=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|8",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|8",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|8",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))))</f>
         <v/>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1" s="130">
       <c r="A26" s="197">
-        <f>IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),9),"")</f>
+        <f>IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|9",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")</f>
         <v/>
       </c>
       <c r="B26" s="198">
-        <f>IFERROR(INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),9),"")),"")</f>
+        <f>IF(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|9",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|9",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="C26" s="199">
-        <f>IF(B26="","",IFERROR(INDEX('CONTRACT CALC'!$G:$G,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),9),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),9),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|9",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B26=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|9",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|9",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="D26" s="199">
-        <f>IF(B26="","",IFERROR(INDEX('CONTRACT CALC'!$I:$I,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),9),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),9),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|9",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B26=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|9",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|9",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="E26" s="199">
@@ -4083,7 +4083,7 @@
         <v/>
       </c>
       <c r="F26" s="199">
-        <f>IF(B26="","",IFERROR(INDEX('CONTRACT CALC'!$H:$H,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),9),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),9),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|9",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B26=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|9",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|9",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="G26" s="199">
@@ -4095,25 +4095,25 @@
         <v/>
       </c>
       <c r="I26" s="199">
-        <f>IF(B26="","",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),9),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),9),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),9),"")))))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|9",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B26=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|9",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|9",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|9",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))))</f>
         <v/>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1" s="130">
       <c r="A27" s="197">
-        <f>IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),10),"")</f>
+        <f>IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|10",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")</f>
         <v/>
       </c>
       <c r="B27" s="198">
-        <f>IFERROR(INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),10),"")),"")</f>
+        <f>IF(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|10",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|10",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="C27" s="199">
-        <f>IF(B27="","",IFERROR(INDEX('CONTRACT CALC'!$G:$G,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),10),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),10),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|10",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B27=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|10",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|10",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="D27" s="199">
-        <f>IF(B27="","",IFERROR(INDEX('CONTRACT CALC'!$I:$I,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),10),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),10),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|10",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B27=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|10",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|10",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="E27" s="199">
@@ -4121,7 +4121,7 @@
         <v/>
       </c>
       <c r="F27" s="199">
-        <f>IF(B27="","",IFERROR(INDEX('CONTRACT CALC'!$H:$H,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),10),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),10),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|10",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B27=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|10",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|10",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="G27" s="199">
@@ -4133,25 +4133,25 @@
         <v/>
       </c>
       <c r="I27" s="199">
-        <f>IF(B27="","",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),10),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),10),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),10),"")))))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|10",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B27=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|10",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|10",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|10",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))))</f>
         <v/>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1" s="130">
       <c r="A28" s="197">
-        <f>IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),11),"")</f>
+        <f>IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|11",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")</f>
         <v/>
       </c>
       <c r="B28" s="198">
-        <f>IFERROR(INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),11),"")),"")</f>
+        <f>IF(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|11",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|11",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="C28" s="199">
-        <f>IF(B28="","",IFERROR(INDEX('CONTRACT CALC'!$G:$G,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),11),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),11),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|11",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B28=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|11",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|11",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="D28" s="199">
-        <f>IF(B28="","",IFERROR(INDEX('CONTRACT CALC'!$I:$I,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),11),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),11),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|11",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B28=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|11",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|11",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="E28" s="199">
@@ -4159,7 +4159,7 @@
         <v/>
       </c>
       <c r="F28" s="199">
-        <f>IF(B28="","",IFERROR(INDEX('CONTRACT CALC'!$H:$H,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),11),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),11),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|11",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B28=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|11",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|11",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="G28" s="199">
@@ -4171,25 +4171,25 @@
         <v/>
       </c>
       <c r="I28" s="199">
-        <f>IF(B28="","",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),11),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),11),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),11),"")))))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|11",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B28=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|11",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|11",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|11",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))))</f>
         <v/>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1" s="130">
       <c r="A29" s="197">
-        <f>IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),12),"")</f>
+        <f>IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|12",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")</f>
         <v/>
       </c>
       <c r="B29" s="198">
-        <f>IFERROR(INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),12),"")),"")</f>
+        <f>IF(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|12",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|12",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="C29" s="199">
-        <f>IF(B29="","",IFERROR(INDEX('CONTRACT CALC'!$G:$G,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),12),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),12),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|12",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B29=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|12",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|12",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="D29" s="199">
-        <f>IF(B29="","",IFERROR(INDEX('CONTRACT CALC'!$I:$I,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),12),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),12),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|12",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B29=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|12",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|12",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="E29" s="199">
@@ -4197,7 +4197,7 @@
         <v/>
       </c>
       <c r="F29" s="199">
-        <f>IF(B29="","",IFERROR(INDEX('CONTRACT CALC'!$H:$H,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),12),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),12),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|12",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B29=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|12",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|12",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="G29" s="199">
@@ -4209,25 +4209,25 @@
         <v/>
       </c>
       <c r="I29" s="199">
-        <f>IF(B29="","",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),12),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),12),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),12),"")))))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|12",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B29=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|12",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|12",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|12",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))))</f>
         <v/>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1" s="130">
       <c r="A30" s="197">
-        <f>IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),13),"")</f>
+        <f>IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|13",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")</f>
         <v/>
       </c>
       <c r="B30" s="198">
-        <f>IFERROR(INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),13),"")),"")</f>
+        <f>IF(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|13",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|13",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="C30" s="199">
-        <f>IF(B30="","",IFERROR(INDEX('CONTRACT CALC'!$G:$G,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),13),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),13),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|13",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B30=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|13",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|13",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="D30" s="199">
-        <f>IF(B30="","",IFERROR(INDEX('CONTRACT CALC'!$I:$I,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),13),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),13),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|13",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B30=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|13",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|13",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="E30" s="199">
@@ -4235,7 +4235,7 @@
         <v/>
       </c>
       <c r="F30" s="199">
-        <f>IF(B30="","",IFERROR(INDEX('CONTRACT CALC'!$H:$H,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),13),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),13),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|13",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B30=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|13",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|13",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="G30" s="199">
@@ -4247,25 +4247,25 @@
         <v/>
       </c>
       <c r="I30" s="199">
-        <f>IF(B30="","",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),13),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),13),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),13),"")))))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|13",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B30=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|13",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|13",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|13",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))))</f>
         <v/>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1" s="130" thickBot="1">
       <c r="A31" s="197">
-        <f>IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),14),"")</f>
+        <f>IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|14",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")</f>
         <v/>
       </c>
       <c r="B31" s="198">
-        <f>IFERROR(INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),14),"")),"")</f>
+        <f>IF(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|14",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|14",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="C31" s="199">
-        <f>IF(B31="","",IFERROR(INDEX('CONTRACT CALC'!$G:$G,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),14),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),14),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|14",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B31=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|14",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|14",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="D31" s="199">
-        <f>IF(B31="","",IFERROR(INDEX('CONTRACT CALC'!$I:$I,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),14),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),14),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|14",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B31=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|14",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|14",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="E31" s="199">
@@ -4273,7 +4273,7 @@
         <v/>
       </c>
       <c r="F31" s="199">
-        <f>IF(B31="","",IFERROR(INDEX('CONTRACT CALC'!$H:$H,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),14),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),14),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|14",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B31=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|14",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|14",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="G31" s="199">
@@ -4285,25 +4285,25 @@
         <v/>
       </c>
       <c r="I31" s="199">
-        <f>IF(B31="","",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),14),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),14),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),14),"")))))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|14",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B31=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|14",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|14",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|14",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))))</f>
         <v/>
       </c>
     </row>
     <row r="32" ht="20.25" customHeight="1" s="130">
       <c r="A32" s="197">
-        <f>IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),15),"")</f>
+        <f>IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|15",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")</f>
         <v/>
       </c>
       <c r="B32" s="201">
-        <f>IFERROR(INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),15),"")),"")</f>
+        <f>IF(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|15",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|15",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="C32" s="202">
-        <f>IF(B32="","",IFERROR(INDEX('CONTRACT CALC'!$G:$G,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),15),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),15),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|15",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B32=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|15",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|15",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="D32" s="202">
-        <f>IF(B32="","",IFERROR(INDEX('CONTRACT CALC'!$I:$I,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),15),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),15),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|15",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B32=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|15",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|15",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="E32" s="202">
@@ -4311,7 +4311,7 @@
         <v/>
       </c>
       <c r="F32" s="199">
-        <f>IF(B32="","",IFERROR(INDEX('CONTRACT CALC'!$H:$H,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),15),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),15),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|15",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B32=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|15",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|15",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="G32" s="202">
@@ -4323,25 +4323,25 @@
         <v/>
       </c>
       <c r="I32" s="202">
-        <f>IF(B32="","",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),15),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),15),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),15),"")))))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|15",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B32=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|15",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|15",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|15",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))))</f>
         <v/>
       </c>
     </row>
     <row r="33" ht="6" customHeight="1" s="130">
       <c r="A33" s="197">
-        <f>IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),16),"")</f>
+        <f>IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|16",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")</f>
         <v/>
       </c>
       <c r="B33" s="203">
-        <f>IFERROR(INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),16),"")),"")</f>
+        <f>IF(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|16",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|16",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="C33" s="204">
-        <f>IF(B33="","",IFERROR(INDEX('CONTRACT CALC'!$G:$G,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),16),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),16),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|16",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B33=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|16",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|16",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="D33" s="204">
-        <f>IF(B33="","",IFERROR(INDEX('CONTRACT CALC'!$I:$I,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),16),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),16),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|16",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B33=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|16",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|16",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="E33" s="204">
@@ -4349,7 +4349,7 @@
         <v/>
       </c>
       <c r="F33" s="204">
-        <f>IF(B33="","",IFERROR(INDEX('CONTRACT CALC'!$H:$H,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),16),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),16),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|16",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B33=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|16",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|16",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="G33" s="204">
@@ -4361,25 +4361,25 @@
         <v/>
       </c>
       <c r="I33" s="204">
-        <f>IF(B33="","",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),16),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),16),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),16),"")))))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|16",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B33=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|16",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|16",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|16",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))))</f>
         <v/>
       </c>
     </row>
     <row r="34" ht="13.5" customHeight="1" s="130" thickBot="1">
       <c r="A34" s="197">
-        <f>IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),17),"")</f>
+        <f>IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|17",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")</f>
         <v/>
       </c>
       <c r="B34" s="201">
-        <f>IFERROR(INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),17),"")),"")</f>
+        <f>IF(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|17",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|17",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="C34" s="202">
-        <f>IF(B34="","",IFERROR(INDEX('CONTRACT CALC'!$G:$G,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),17),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),17),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|17",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B34=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|17",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|17",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="D34" s="202">
-        <f>IF(B34="","",IFERROR(INDEX('CONTRACT CALC'!$I:$I,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),17),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),17),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|17",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B34=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|17",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|17",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="E34" s="202">
@@ -4387,7 +4387,7 @@
         <v/>
       </c>
       <c r="F34" s="202">
-        <f>IF(B34="","",IFERROR(INDEX('CONTRACT CALC'!$H:$H,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),17),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),17),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|17",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B34=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|17",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|17",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="G34" s="202">
@@ -4399,25 +4399,25 @@
         <v/>
       </c>
       <c r="I34" s="202">
-        <f>IF(B34="","",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),17),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),17),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),17),"")))))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|17",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B34=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|17",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|17",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|17",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))))</f>
         <v/>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1" s="130" thickBot="1">
       <c r="A35" s="197">
-        <f>IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),18),"")</f>
+        <f>IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|18",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")</f>
         <v/>
       </c>
       <c r="B35" s="205">
-        <f>IFERROR(INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),18),"")),"")</f>
+        <f>IF(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|18",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|18",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="C35" s="199">
-        <f>IF(B35="","",IFERROR(INDEX('CONTRACT CALC'!$G:$G,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),18),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),18),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|18",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B35=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|18",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|18",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="D35" s="199">
-        <f>IF(B35="","",IFERROR(INDEX('CONTRACT CALC'!$I:$I,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),18),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),18),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|18",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B35=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|18",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|18",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="E35" s="206">
@@ -4425,7 +4425,7 @@
         <v/>
       </c>
       <c r="F35" s="199">
-        <f>IF(B35="","",IFERROR(INDEX('CONTRACT CALC'!$H:$H,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),18),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),18),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|18",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B35=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|18",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|18",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="G35" s="199">
@@ -4437,25 +4437,25 @@
         <v/>
       </c>
       <c r="I35" s="199">
-        <f>IF(B35="","",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),18),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),18),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),18),"")))))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|18",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B35=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|18",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|18",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|18",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))))</f>
         <v/>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1" s="130">
       <c r="A36" s="197">
-        <f>IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),19),"")</f>
+        <f>IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|19",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")</f>
         <v/>
       </c>
       <c r="B36" s="198">
-        <f>IFERROR(INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),19),"")),"")</f>
+        <f>IF(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|19",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|19",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="C36" s="199">
-        <f>IF(B36="","",IFERROR(INDEX('CONTRACT CALC'!$G:$G,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),19),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),19),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|19",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B36=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|19",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|19",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="D36" s="199">
-        <f>IF(B36="","",IFERROR(INDEX('CONTRACT CALC'!$I:$I,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),19),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),19),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|19",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B36=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|19",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|19",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="E36" s="207">
@@ -4463,7 +4463,7 @@
         <v/>
       </c>
       <c r="F36" s="207">
-        <f>IF(B36="","",IFERROR(INDEX('CONTRACT CALC'!$H:$H,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),19),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),19),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|19",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B36=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|19",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|19",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="G36" s="207">
@@ -4475,25 +4475,25 @@
         <v/>
       </c>
       <c r="I36" s="199">
-        <f>IF(B36="","",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),19),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),19),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),19),"")))))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|19",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B36=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|19",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|19",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|19",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))))</f>
         <v/>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1" s="130">
       <c r="A37" s="197">
-        <f>IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),20),"")</f>
+        <f>IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|20",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")</f>
         <v/>
       </c>
       <c r="B37" s="198">
-        <f>IFERROR(INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),20),"")),"")</f>
+        <f>IF(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|20",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|20",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="C37" s="199">
-        <f>IF(B37="","",IFERROR(INDEX('CONTRACT CALC'!$G:$G,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),20),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),20),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|20",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B37=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|20",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|20",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="D37" s="199">
-        <f>IF(B37="","",IFERROR(INDEX('CONTRACT CALC'!$I:$I,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),20),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),20),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|20",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B37=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|20",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|20",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="E37" s="199">
@@ -4501,7 +4501,7 @@
         <v/>
       </c>
       <c r="F37" s="199">
-        <f>IF(B37="","",IFERROR(INDEX('CONTRACT CALC'!$H:$H,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),20),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),20),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|20",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B37=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|20",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|20",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="G37" s="199">
@@ -4513,25 +4513,25 @@
         <v/>
       </c>
       <c r="I37" s="199">
-        <f>IF(B37="","",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),20),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),20),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),20),"")))))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|20",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B37=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|20",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|20",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|20",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))))</f>
         <v/>
       </c>
     </row>
     <row r="38" ht="16.5" customHeight="1" s="130">
       <c r="A38" s="197">
-        <f>IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),21),"")</f>
+        <f>IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|21",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")</f>
         <v/>
       </c>
       <c r="B38" s="198">
-        <f>IFERROR(INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),21),"")),"")</f>
+        <f>IF(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|21",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|21",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="C38" s="199">
-        <f>IF(B38="","",IFERROR(INDEX('CONTRACT CALC'!$G:$G,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),21),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),21),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|21",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B38=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|21",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|21",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="D38" s="199">
-        <f>IF(B38="","",IFERROR(INDEX('CONTRACT CALC'!$I:$I,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),21),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),21),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|21",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B38=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|21",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|21",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="E38" s="207">
@@ -4539,7 +4539,7 @@
         <v/>
       </c>
       <c r="F38" s="207">
-        <f>IF(B38="","",IFERROR(INDEX('CONTRACT CALC'!$H:$H,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),21),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),21),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|21",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B38=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|21",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|21",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="G38" s="207">
@@ -4551,25 +4551,25 @@
         <v/>
       </c>
       <c r="I38" s="199">
-        <f>IF(B38="","",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),21),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),21),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),21),"")))))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|21",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B38=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|21",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|21",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|21",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))))</f>
         <v/>
       </c>
     </row>
     <row r="39" ht="20.1" customHeight="1" s="130">
       <c r="A39" s="208">
-        <f>IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),22),"")</f>
+        <f>IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|22",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")</f>
         <v/>
       </c>
       <c r="B39" s="198">
-        <f>IFERROR(INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),22),"")),"")</f>
+        <f>IF(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|22",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|22",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="C39" s="199">
-        <f>IF(B39="","",IFERROR(INDEX('CONTRACT CALC'!$G:$G,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),22),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),22),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|22",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B39=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|22",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|22",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="D39" s="199">
-        <f>IF(B39="","",IFERROR(INDEX('CONTRACT CALC'!$I:$I,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),22),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),22),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|22",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B39=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|22",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|22",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="E39" s="199">
@@ -4577,7 +4577,7 @@
         <v/>
       </c>
       <c r="F39" s="199">
-        <f>IF(B39="","",IFERROR(INDEX('CONTRACT CALC'!$H:$H,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),22),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),22),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|22",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B39=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|22",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|22",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="G39" s="199">
@@ -4589,25 +4589,25 @@
         <v/>
       </c>
       <c r="I39" s="199">
-        <f>IF(B39="","",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),22),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),22),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),22),"")))))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|22",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B39=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|22",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|22",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|22",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))))</f>
         <v/>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="208">
-        <f>IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),23),"")</f>
+        <f>IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|23",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")</f>
         <v/>
       </c>
       <c r="B40" s="198">
-        <f>IFERROR(INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),23),"")),"")</f>
+        <f>IF(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|23",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|23",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="C40" s="199">
-        <f>IF(B40="","",IFERROR(INDEX('CONTRACT CALC'!$G:$G,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),23),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),23),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|23",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B40=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|23",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|23",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="D40" s="199">
-        <f>IF(B40="","",IFERROR(INDEX('CONTRACT CALC'!$I:$I,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),23),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),23),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|23",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B40=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|23",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|23",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="E40" s="199">
@@ -4615,7 +4615,7 @@
         <v/>
       </c>
       <c r="F40" s="199">
-        <f>IF(B40="","",IFERROR(INDEX('CONTRACT CALC'!$H:$H,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),23),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),23),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|23",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B40=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|23",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|23",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="G40" s="199">
@@ -4627,25 +4627,25 @@
         <v/>
       </c>
       <c r="I40" s="199">
-        <f>IF(B40="","",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),23),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),23),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),23),"")))))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|23",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B40=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|23",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|23",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|23",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))))</f>
         <v/>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="130">
       <c r="A41" s="208">
-        <f>IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),24),"")</f>
+        <f>IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|24",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")</f>
         <v/>
       </c>
       <c r="B41" s="198">
-        <f>IFERROR(INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),24),"")),"")</f>
+        <f>IF(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|24",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|24",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="C41" s="199">
-        <f>IF(B41="","",IFERROR(INDEX('CONTRACT CALC'!$G:$G,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),24),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),24),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|24",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B41=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|24",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|24",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="D41" s="199">
-        <f>IF(B41="","",IFERROR(INDEX('CONTRACT CALC'!$I:$I,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),24),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),24),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|24",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B41=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|24",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|24",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="E41" s="199">
@@ -4653,7 +4653,7 @@
         <v/>
       </c>
       <c r="F41" s="199">
-        <f>IF(B41="","",IFERROR(INDEX('CONTRACT CALC'!$H:$H,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),24),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),24),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|24",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B41=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|24",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|24",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="G41" s="199">
@@ -4665,25 +4665,25 @@
         <v/>
       </c>
       <c r="I41" s="199">
-        <f>IF(B41="","",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),24),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),24),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),24),"")))))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|24",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B41=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|24",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|24",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|24",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))))</f>
         <v/>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="208">
-        <f>IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),25),"")</f>
+        <f>IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|25",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")</f>
         <v/>
       </c>
       <c r="B42" s="198">
-        <f>IFERROR(INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),25),"")),"")</f>
+        <f>IF(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|25",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|25",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="C42" s="199">
-        <f>IF(B42="","",IFERROR(INDEX('CONTRACT CALC'!$G:$G,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),25),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),25),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|25",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B42=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|25",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|25",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="D42" s="199">
-        <f>IF(B42="","",IFERROR(INDEX('CONTRACT CALC'!$I:$I,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),25),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),25),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|25",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B42=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|25",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|25",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="E42" s="199">
@@ -4691,7 +4691,7 @@
         <v/>
       </c>
       <c r="F42" s="199">
-        <f>IF(B42="","",IFERROR(INDEX('CONTRACT CALC'!$H:$H,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),25),""))+11)*INDEX('CONTRACT CALC'!$F:$F,(IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),25),""))+11),""))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|25",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B42=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|25",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|25",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
       <c r="G42" s="199">
@@ -4703,7 +4703,7 @@
         <v/>
       </c>
       <c r="I42" s="199">
-        <f>IF(B42="","",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),25),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C:$C,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),25),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D:$D,IFERROR(AGGREGATE(15,6,ROW('EVENT ASSIGNMENT'!$A$2:$A$101)/((N('EVENT ASSIGNMENT'!$A$2:$A$101)=N($B$10))*('EVENT ASSIGNMENT'!$F$2:$F$101=$E$10)),25),"")))))</f>
+        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|25",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B42=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|25",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|25",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|25",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))))</f>
         <v/>
       </c>
     </row>
@@ -53472,7 +53472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I101"/>
+  <dimension ref="A1:K101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="12.75"/>
   <cols>
     <col width="14" customWidth="1" style="130" min="1" max="1"/>
@@ -53532,6 +53532,16 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="J1" s="214" t="inlineStr">
+        <is>
+          <t>Payee Seq</t>
+        </is>
+      </c>
+      <c r="K1" s="214" t="inlineStr">
+        <is>
+          <t>Payout Lookup Key</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="25.5" customHeight="1" s="130">
       <c r="A2" s="233" t="n">
@@ -53571,6 +53581,14 @@
         </is>
       </c>
       <c r="I2" s="91" t="n"/>
+      <c r="J2">
+        <f>IF(OR(A2="",F2=""),"",COUNTIFS($A$2:A2,A2,$F$2:F2,F2))</f>
+        <v/>
+      </c>
+      <c r="K2">
+        <f>IF(OR(A2="",F2="",J2=""),"",TEXT(A2,"yyyymmdd")&amp;"|"&amp;F2&amp;"|"&amp;J2)</f>
+        <v/>
+      </c>
     </row>
     <row r="3" ht="25.5" customHeight="1" s="130">
       <c r="A3" s="233" t="n">
@@ -53610,6 +53628,14 @@
         </is>
       </c>
       <c r="I3" s="91" t="n"/>
+      <c r="J3">
+        <f>IF(OR(A3="",F3=""),"",COUNTIFS($A$2:A3,A3,$F$2:F3,F3))</f>
+        <v/>
+      </c>
+      <c r="K3">
+        <f>IF(OR(A3="",F3="",J3=""),"",TEXT(A3,"yyyymmdd")&amp;"|"&amp;F3&amp;"|"&amp;J3)</f>
+        <v/>
+      </c>
     </row>
     <row r="4" ht="25.5" customHeight="1" s="130">
       <c r="A4" s="233" t="n">
@@ -53649,6 +53675,14 @@
         </is>
       </c>
       <c r="I4" s="91" t="n"/>
+      <c r="J4">
+        <f>IF(OR(A4="",F4=""),"",COUNTIFS($A$2:A4,A4,$F$2:F4,F4))</f>
+        <v/>
+      </c>
+      <c r="K4">
+        <f>IF(OR(A4="",F4="",J4=""),"",TEXT(A4,"yyyymmdd")&amp;"|"&amp;F4&amp;"|"&amp;J4)</f>
+        <v/>
+      </c>
     </row>
     <row r="5" ht="25.5" customHeight="1" s="130">
       <c r="A5" s="233" t="n">
@@ -53688,6 +53722,14 @@
         </is>
       </c>
       <c r="I5" s="91" t="n"/>
+      <c r="J5">
+        <f>IF(OR(A5="",F5=""),"",COUNTIFS($A$2:A5,A5,$F$2:F5,F5))</f>
+        <v/>
+      </c>
+      <c r="K5">
+        <f>IF(OR(A5="",F5="",J5=""),"",TEXT(A5,"yyyymmdd")&amp;"|"&amp;F5&amp;"|"&amp;J5)</f>
+        <v/>
+      </c>
     </row>
     <row r="6" ht="25.5" customHeight="1" s="130">
       <c r="A6" s="233" t="n">
@@ -53727,6 +53769,14 @@
         </is>
       </c>
       <c r="I6" s="91" t="n"/>
+      <c r="J6">
+        <f>IF(OR(A6="",F6=""),"",COUNTIFS($A$2:A6,A6,$F$2:F6,F6))</f>
+        <v/>
+      </c>
+      <c r="K6">
+        <f>IF(OR(A6="",F6="",J6=""),"",TEXT(A6,"yyyymmdd")&amp;"|"&amp;F6&amp;"|"&amp;J6)</f>
+        <v/>
+      </c>
     </row>
     <row r="7" ht="25.5" customHeight="1" s="130">
       <c r="A7" s="233" t="n">
@@ -53766,6 +53816,14 @@
         </is>
       </c>
       <c r="I7" s="91" t="n"/>
+      <c r="J7">
+        <f>IF(OR(A7="",F7=""),"",COUNTIFS($A$2:A7,A7,$F$2:F7,F7))</f>
+        <v/>
+      </c>
+      <c r="K7">
+        <f>IF(OR(A7="",F7="",J7=""),"",TEXT(A7,"yyyymmdd")&amp;"|"&amp;F7&amp;"|"&amp;J7)</f>
+        <v/>
+      </c>
     </row>
     <row r="8" ht="25.5" customHeight="1" s="130">
       <c r="A8" s="233" t="n">
@@ -53805,6 +53863,14 @@
         </is>
       </c>
       <c r="I8" s="91" t="n"/>
+      <c r="J8">
+        <f>IF(OR(A8="",F8=""),"",COUNTIFS($A$2:A8,A8,$F$2:F8,F8))</f>
+        <v/>
+      </c>
+      <c r="K8">
+        <f>IF(OR(A8="",F8="",J8=""),"",TEXT(A8,"yyyymmdd")&amp;"|"&amp;F8&amp;"|"&amp;J8)</f>
+        <v/>
+      </c>
     </row>
     <row r="9" ht="25.5" customHeight="1" s="130">
       <c r="A9" s="233" t="n">
@@ -53844,6 +53910,14 @@
         </is>
       </c>
       <c r="I9" s="91" t="n"/>
+      <c r="J9">
+        <f>IF(OR(A9="",F9=""),"",COUNTIFS($A$2:A9,A9,$F$2:F9,F9))</f>
+        <v/>
+      </c>
+      <c r="K9">
+        <f>IF(OR(A9="",F9="",J9=""),"",TEXT(A9,"yyyymmdd")&amp;"|"&amp;F9&amp;"|"&amp;J9)</f>
+        <v/>
+      </c>
     </row>
     <row r="10" ht="25.5" customHeight="1" s="130">
       <c r="A10" s="233" t="n">
@@ -53883,6 +53957,14 @@
         </is>
       </c>
       <c r="I10" s="91" t="n"/>
+      <c r="J10">
+        <f>IF(OR(A10="",F10=""),"",COUNTIFS($A$2:A10,A10,$F$2:F10,F10))</f>
+        <v/>
+      </c>
+      <c r="K10">
+        <f>IF(OR(A10="",F10="",J10=""),"",TEXT(A10,"yyyymmdd")&amp;"|"&amp;F10&amp;"|"&amp;J10)</f>
+        <v/>
+      </c>
     </row>
     <row r="11" ht="25.5" customHeight="1" s="130">
       <c r="A11" s="233" t="n">
@@ -53922,6 +54004,14 @@
         </is>
       </c>
       <c r="I11" s="91" t="n"/>
+      <c r="J11">
+        <f>IF(OR(A11="",F11=""),"",COUNTIFS($A$2:A11,A11,$F$2:F11,F11))</f>
+        <v/>
+      </c>
+      <c r="K11">
+        <f>IF(OR(A11="",F11="",J11=""),"",TEXT(A11,"yyyymmdd")&amp;"|"&amp;F11&amp;"|"&amp;J11)</f>
+        <v/>
+      </c>
     </row>
     <row r="12" ht="25.5" customHeight="1" s="130">
       <c r="A12" s="233" t="n">
@@ -53961,6 +54051,14 @@
         </is>
       </c>
       <c r="I12" s="91" t="n"/>
+      <c r="J12">
+        <f>IF(OR(A12="",F12=""),"",COUNTIFS($A$2:A12,A12,$F$2:F12,F12))</f>
+        <v/>
+      </c>
+      <c r="K12">
+        <f>IF(OR(A12="",F12="",J12=""),"",TEXT(A12,"yyyymmdd")&amp;"|"&amp;F12&amp;"|"&amp;J12)</f>
+        <v/>
+      </c>
     </row>
     <row r="13" ht="25.5" customHeight="1" s="130">
       <c r="A13" s="233" t="n">
@@ -54000,6 +54098,14 @@
         </is>
       </c>
       <c r="I13" s="91" t="n"/>
+      <c r="J13">
+        <f>IF(OR(A13="",F13=""),"",COUNTIFS($A$2:A13,A13,$F$2:F13,F13))</f>
+        <v/>
+      </c>
+      <c r="K13">
+        <f>IF(OR(A13="",F13="",J13=""),"",TEXT(A13,"yyyymmdd")&amp;"|"&amp;F13&amp;"|"&amp;J13)</f>
+        <v/>
+      </c>
     </row>
     <row r="14" ht="25.5" customHeight="1" s="130">
       <c r="A14" s="233" t="n">
@@ -54039,6 +54145,14 @@
         </is>
       </c>
       <c r="I14" s="91" t="n"/>
+      <c r="J14">
+        <f>IF(OR(A14="",F14=""),"",COUNTIFS($A$2:A14,A14,$F$2:F14,F14))</f>
+        <v/>
+      </c>
+      <c r="K14">
+        <f>IF(OR(A14="",F14="",J14=""),"",TEXT(A14,"yyyymmdd")&amp;"|"&amp;F14&amp;"|"&amp;J14)</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="233" t="n"/>
@@ -54050,6 +54164,14 @@
       <c r="G15" s="234" t="n"/>
       <c r="H15" s="91" t="n"/>
       <c r="I15" s="91" t="n"/>
+      <c r="J15">
+        <f>IF(OR(A15="",F15=""),"",COUNTIFS($A$2:A15,A15,$F$2:F15,F15))</f>
+        <v/>
+      </c>
+      <c r="K15">
+        <f>IF(OR(A15="",F15="",J15=""),"",TEXT(A15,"yyyymmdd")&amp;"|"&amp;F15&amp;"|"&amp;J15)</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="233" t="n"/>
@@ -54061,6 +54183,14 @@
       <c r="G16" s="234" t="n"/>
       <c r="H16" s="91" t="n"/>
       <c r="I16" s="91" t="n"/>
+      <c r="J16">
+        <f>IF(OR(A16="",F16=""),"",COUNTIFS($A$2:A16,A16,$F$2:F16,F16))</f>
+        <v/>
+      </c>
+      <c r="K16">
+        <f>IF(OR(A16="",F16="",J16=""),"",TEXT(A16,"yyyymmdd")&amp;"|"&amp;F16&amp;"|"&amp;J16)</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="233" t="n"/>
@@ -54072,6 +54202,14 @@
       <c r="G17" s="234" t="n"/>
       <c r="H17" s="91" t="n"/>
       <c r="I17" s="91" t="n"/>
+      <c r="J17">
+        <f>IF(OR(A17="",F17=""),"",COUNTIFS($A$2:A17,A17,$F$2:F17,F17))</f>
+        <v/>
+      </c>
+      <c r="K17">
+        <f>IF(OR(A17="",F17="",J17=""),"",TEXT(A17,"yyyymmdd")&amp;"|"&amp;F17&amp;"|"&amp;J17)</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="233" t="n"/>
@@ -54083,6 +54221,14 @@
       <c r="G18" s="234" t="n"/>
       <c r="H18" s="91" t="n"/>
       <c r="I18" s="91" t="n"/>
+      <c r="J18">
+        <f>IF(OR(A18="",F18=""),"",COUNTIFS($A$2:A18,A18,$F$2:F18,F18))</f>
+        <v/>
+      </c>
+      <c r="K18">
+        <f>IF(OR(A18="",F18="",J18=""),"",TEXT(A18,"yyyymmdd")&amp;"|"&amp;F18&amp;"|"&amp;J18)</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="233" t="n"/>
@@ -54094,6 +54240,14 @@
       <c r="G19" s="234" t="n"/>
       <c r="H19" s="91" t="n"/>
       <c r="I19" s="91" t="n"/>
+      <c r="J19">
+        <f>IF(OR(A19="",F19=""),"",COUNTIFS($A$2:A19,A19,$F$2:F19,F19))</f>
+        <v/>
+      </c>
+      <c r="K19">
+        <f>IF(OR(A19="",F19="",J19=""),"",TEXT(A19,"yyyymmdd")&amp;"|"&amp;F19&amp;"|"&amp;J19)</f>
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="233" t="n"/>
@@ -54105,6 +54259,14 @@
       <c r="G20" s="234" t="n"/>
       <c r="H20" s="91" t="n"/>
       <c r="I20" s="91" t="n"/>
+      <c r="J20">
+        <f>IF(OR(A20="",F20=""),"",COUNTIFS($A$2:A20,A20,$F$2:F20,F20))</f>
+        <v/>
+      </c>
+      <c r="K20">
+        <f>IF(OR(A20="",F20="",J20=""),"",TEXT(A20,"yyyymmdd")&amp;"|"&amp;F20&amp;"|"&amp;J20)</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="233" t="n"/>
@@ -54116,6 +54278,14 @@
       <c r="G21" s="234" t="n"/>
       <c r="H21" s="91" t="n"/>
       <c r="I21" s="91" t="n"/>
+      <c r="J21">
+        <f>IF(OR(A21="",F21=""),"",COUNTIFS($A$2:A21,A21,$F$2:F21,F21))</f>
+        <v/>
+      </c>
+      <c r="K21">
+        <f>IF(OR(A21="",F21="",J21=""),"",TEXT(A21,"yyyymmdd")&amp;"|"&amp;F21&amp;"|"&amp;J21)</f>
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="233" t="n"/>
@@ -54127,6 +54297,14 @@
       <c r="G22" s="234" t="n"/>
       <c r="H22" s="91" t="n"/>
       <c r="I22" s="91" t="n"/>
+      <c r="J22">
+        <f>IF(OR(A22="",F22=""),"",COUNTIFS($A$2:A22,A22,$F$2:F22,F22))</f>
+        <v/>
+      </c>
+      <c r="K22">
+        <f>IF(OR(A22="",F22="",J22=""),"",TEXT(A22,"yyyymmdd")&amp;"|"&amp;F22&amp;"|"&amp;J22)</f>
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="233" t="n"/>
@@ -54138,6 +54316,14 @@
       <c r="G23" s="234" t="n"/>
       <c r="H23" s="91" t="n"/>
       <c r="I23" s="91" t="n"/>
+      <c r="J23">
+        <f>IF(OR(A23="",F23=""),"",COUNTIFS($A$2:A23,A23,$F$2:F23,F23))</f>
+        <v/>
+      </c>
+      <c r="K23">
+        <f>IF(OR(A23="",F23="",J23=""),"",TEXT(A23,"yyyymmdd")&amp;"|"&amp;F23&amp;"|"&amp;J23)</f>
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="233" t="n"/>
@@ -54149,6 +54335,14 @@
       <c r="G24" s="234" t="n"/>
       <c r="H24" s="91" t="n"/>
       <c r="I24" s="91" t="n"/>
+      <c r="J24">
+        <f>IF(OR(A24="",F24=""),"",COUNTIFS($A$2:A24,A24,$F$2:F24,F24))</f>
+        <v/>
+      </c>
+      <c r="K24">
+        <f>IF(OR(A24="",F24="",J24=""),"",TEXT(A24,"yyyymmdd")&amp;"|"&amp;F24&amp;"|"&amp;J24)</f>
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="233" t="n"/>
@@ -54160,6 +54354,14 @@
       <c r="G25" s="234" t="n"/>
       <c r="H25" s="91" t="n"/>
       <c r="I25" s="91" t="n"/>
+      <c r="J25">
+        <f>IF(OR(A25="",F25=""),"",COUNTIFS($A$2:A25,A25,$F$2:F25,F25))</f>
+        <v/>
+      </c>
+      <c r="K25">
+        <f>IF(OR(A25="",F25="",J25=""),"",TEXT(A25,"yyyymmdd")&amp;"|"&amp;F25&amp;"|"&amp;J25)</f>
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="233" t="n"/>
@@ -54171,6 +54373,14 @@
       <c r="G26" s="234" t="n"/>
       <c r="H26" s="91" t="n"/>
       <c r="I26" s="91" t="n"/>
+      <c r="J26">
+        <f>IF(OR(A26="",F26=""),"",COUNTIFS($A$2:A26,A26,$F$2:F26,F26))</f>
+        <v/>
+      </c>
+      <c r="K26">
+        <f>IF(OR(A26="",F26="",J26=""),"",TEXT(A26,"yyyymmdd")&amp;"|"&amp;F26&amp;"|"&amp;J26)</f>
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="233" t="n"/>
@@ -54182,6 +54392,14 @@
       <c r="G27" s="234" t="n"/>
       <c r="H27" s="91" t="n"/>
       <c r="I27" s="91" t="n"/>
+      <c r="J27">
+        <f>IF(OR(A27="",F27=""),"",COUNTIFS($A$2:A27,A27,$F$2:F27,F27))</f>
+        <v/>
+      </c>
+      <c r="K27">
+        <f>IF(OR(A27="",F27="",J27=""),"",TEXT(A27,"yyyymmdd")&amp;"|"&amp;F27&amp;"|"&amp;J27)</f>
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="233" t="n"/>
@@ -54193,6 +54411,14 @@
       <c r="G28" s="234" t="n"/>
       <c r="H28" s="91" t="n"/>
       <c r="I28" s="91" t="n"/>
+      <c r="J28">
+        <f>IF(OR(A28="",F28=""),"",COUNTIFS($A$2:A28,A28,$F$2:F28,F28))</f>
+        <v/>
+      </c>
+      <c r="K28">
+        <f>IF(OR(A28="",F28="",J28=""),"",TEXT(A28,"yyyymmdd")&amp;"|"&amp;F28&amp;"|"&amp;J28)</f>
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="233" t="n"/>
@@ -54204,6 +54430,14 @@
       <c r="G29" s="234" t="n"/>
       <c r="H29" s="91" t="n"/>
       <c r="I29" s="91" t="n"/>
+      <c r="J29">
+        <f>IF(OR(A29="",F29=""),"",COUNTIFS($A$2:A29,A29,$F$2:F29,F29))</f>
+        <v/>
+      </c>
+      <c r="K29">
+        <f>IF(OR(A29="",F29="",J29=""),"",TEXT(A29,"yyyymmdd")&amp;"|"&amp;F29&amp;"|"&amp;J29)</f>
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="233" t="n"/>
@@ -54215,6 +54449,14 @@
       <c r="G30" s="234" t="n"/>
       <c r="H30" s="91" t="n"/>
       <c r="I30" s="91" t="n"/>
+      <c r="J30">
+        <f>IF(OR(A30="",F30=""),"",COUNTIFS($A$2:A30,A30,$F$2:F30,F30))</f>
+        <v/>
+      </c>
+      <c r="K30">
+        <f>IF(OR(A30="",F30="",J30=""),"",TEXT(A30,"yyyymmdd")&amp;"|"&amp;F30&amp;"|"&amp;J30)</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="233" t="n"/>
@@ -54226,6 +54468,14 @@
       <c r="G31" s="234" t="n"/>
       <c r="H31" s="91" t="n"/>
       <c r="I31" s="91" t="n"/>
+      <c r="J31">
+        <f>IF(OR(A31="",F31=""),"",COUNTIFS($A$2:A31,A31,$F$2:F31,F31))</f>
+        <v/>
+      </c>
+      <c r="K31">
+        <f>IF(OR(A31="",F31="",J31=""),"",TEXT(A31,"yyyymmdd")&amp;"|"&amp;F31&amp;"|"&amp;J31)</f>
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="233" t="n"/>
@@ -54237,6 +54487,14 @@
       <c r="G32" s="234" t="n"/>
       <c r="H32" s="91" t="n"/>
       <c r="I32" s="91" t="n"/>
+      <c r="J32">
+        <f>IF(OR(A32="",F32=""),"",COUNTIFS($A$2:A32,A32,$F$2:F32,F32))</f>
+        <v/>
+      </c>
+      <c r="K32">
+        <f>IF(OR(A32="",F32="",J32=""),"",TEXT(A32,"yyyymmdd")&amp;"|"&amp;F32&amp;"|"&amp;J32)</f>
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="233" t="n"/>
@@ -54248,6 +54506,14 @@
       <c r="G33" s="234" t="n"/>
       <c r="H33" s="91" t="n"/>
       <c r="I33" s="91" t="n"/>
+      <c r="J33">
+        <f>IF(OR(A33="",F33=""),"",COUNTIFS($A$2:A33,A33,$F$2:F33,F33))</f>
+        <v/>
+      </c>
+      <c r="K33">
+        <f>IF(OR(A33="",F33="",J33=""),"",TEXT(A33,"yyyymmdd")&amp;"|"&amp;F33&amp;"|"&amp;J33)</f>
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="233" t="n"/>
@@ -54259,6 +54525,14 @@
       <c r="G34" s="234" t="n"/>
       <c r="H34" s="91" t="n"/>
       <c r="I34" s="91" t="n"/>
+      <c r="J34">
+        <f>IF(OR(A34="",F34=""),"",COUNTIFS($A$2:A34,A34,$F$2:F34,F34))</f>
+        <v/>
+      </c>
+      <c r="K34">
+        <f>IF(OR(A34="",F34="",J34=""),"",TEXT(A34,"yyyymmdd")&amp;"|"&amp;F34&amp;"|"&amp;J34)</f>
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="233" t="n"/>
@@ -54270,6 +54544,14 @@
       <c r="G35" s="234" t="n"/>
       <c r="H35" s="91" t="n"/>
       <c r="I35" s="91" t="n"/>
+      <c r="J35">
+        <f>IF(OR(A35="",F35=""),"",COUNTIFS($A$2:A35,A35,$F$2:F35,F35))</f>
+        <v/>
+      </c>
+      <c r="K35">
+        <f>IF(OR(A35="",F35="",J35=""),"",TEXT(A35,"yyyymmdd")&amp;"|"&amp;F35&amp;"|"&amp;J35)</f>
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="233" t="n"/>
@@ -54281,6 +54563,14 @@
       <c r="G36" s="234" t="n"/>
       <c r="H36" s="91" t="n"/>
       <c r="I36" s="91" t="n"/>
+      <c r="J36">
+        <f>IF(OR(A36="",F36=""),"",COUNTIFS($A$2:A36,A36,$F$2:F36,F36))</f>
+        <v/>
+      </c>
+      <c r="K36">
+        <f>IF(OR(A36="",F36="",J36=""),"",TEXT(A36,"yyyymmdd")&amp;"|"&amp;F36&amp;"|"&amp;J36)</f>
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="233" t="n"/>
@@ -54292,6 +54582,14 @@
       <c r="G37" s="234" t="n"/>
       <c r="H37" s="91" t="n"/>
       <c r="I37" s="91" t="n"/>
+      <c r="J37">
+        <f>IF(OR(A37="",F37=""),"",COUNTIFS($A$2:A37,A37,$F$2:F37,F37))</f>
+        <v/>
+      </c>
+      <c r="K37">
+        <f>IF(OR(A37="",F37="",J37=""),"",TEXT(A37,"yyyymmdd")&amp;"|"&amp;F37&amp;"|"&amp;J37)</f>
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="233" t="n"/>
@@ -54303,6 +54601,14 @@
       <c r="G38" s="234" t="n"/>
       <c r="H38" s="91" t="n"/>
       <c r="I38" s="91" t="n"/>
+      <c r="J38">
+        <f>IF(OR(A38="",F38=""),"",COUNTIFS($A$2:A38,A38,$F$2:F38,F38))</f>
+        <v/>
+      </c>
+      <c r="K38">
+        <f>IF(OR(A38="",F38="",J38=""),"",TEXT(A38,"yyyymmdd")&amp;"|"&amp;F38&amp;"|"&amp;J38)</f>
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="233" t="n"/>
@@ -54314,6 +54620,14 @@
       <c r="G39" s="234" t="n"/>
       <c r="H39" s="91" t="n"/>
       <c r="I39" s="91" t="n"/>
+      <c r="J39">
+        <f>IF(OR(A39="",F39=""),"",COUNTIFS($A$2:A39,A39,$F$2:F39,F39))</f>
+        <v/>
+      </c>
+      <c r="K39">
+        <f>IF(OR(A39="",F39="",J39=""),"",TEXT(A39,"yyyymmdd")&amp;"|"&amp;F39&amp;"|"&amp;J39)</f>
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="233" t="n"/>
@@ -54325,6 +54639,14 @@
       <c r="G40" s="234" t="n"/>
       <c r="H40" s="91" t="n"/>
       <c r="I40" s="91" t="n"/>
+      <c r="J40">
+        <f>IF(OR(A40="",F40=""),"",COUNTIFS($A$2:A40,A40,$F$2:F40,F40))</f>
+        <v/>
+      </c>
+      <c r="K40">
+        <f>IF(OR(A40="",F40="",J40=""),"",TEXT(A40,"yyyymmdd")&amp;"|"&amp;F40&amp;"|"&amp;J40)</f>
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="233" t="n"/>
@@ -54336,6 +54658,14 @@
       <c r="G41" s="234" t="n"/>
       <c r="H41" s="91" t="n"/>
       <c r="I41" s="91" t="n"/>
+      <c r="J41">
+        <f>IF(OR(A41="",F41=""),"",COUNTIFS($A$2:A41,A41,$F$2:F41,F41))</f>
+        <v/>
+      </c>
+      <c r="K41">
+        <f>IF(OR(A41="",F41="",J41=""),"",TEXT(A41,"yyyymmdd")&amp;"|"&amp;F41&amp;"|"&amp;J41)</f>
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="233" t="n"/>
@@ -54347,6 +54677,14 @@
       <c r="G42" s="234" t="n"/>
       <c r="H42" s="91" t="n"/>
       <c r="I42" s="91" t="n"/>
+      <c r="J42">
+        <f>IF(OR(A42="",F42=""),"",COUNTIFS($A$2:A42,A42,$F$2:F42,F42))</f>
+        <v/>
+      </c>
+      <c r="K42">
+        <f>IF(OR(A42="",F42="",J42=""),"",TEXT(A42,"yyyymmdd")&amp;"|"&amp;F42&amp;"|"&amp;J42)</f>
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="233" t="n"/>
@@ -54358,6 +54696,14 @@
       <c r="G43" s="234" t="n"/>
       <c r="H43" s="91" t="n"/>
       <c r="I43" s="91" t="n"/>
+      <c r="J43">
+        <f>IF(OR(A43="",F43=""),"",COUNTIFS($A$2:A43,A43,$F$2:F43,F43))</f>
+        <v/>
+      </c>
+      <c r="K43">
+        <f>IF(OR(A43="",F43="",J43=""),"",TEXT(A43,"yyyymmdd")&amp;"|"&amp;F43&amp;"|"&amp;J43)</f>
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="233" t="n"/>
@@ -54369,6 +54715,14 @@
       <c r="G44" s="234" t="n"/>
       <c r="H44" s="91" t="n"/>
       <c r="I44" s="91" t="n"/>
+      <c r="J44">
+        <f>IF(OR(A44="",F44=""),"",COUNTIFS($A$2:A44,A44,$F$2:F44,F44))</f>
+        <v/>
+      </c>
+      <c r="K44">
+        <f>IF(OR(A44="",F44="",J44=""),"",TEXT(A44,"yyyymmdd")&amp;"|"&amp;F44&amp;"|"&amp;J44)</f>
+        <v/>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="233" t="n"/>
@@ -54380,6 +54734,14 @@
       <c r="G45" s="234" t="n"/>
       <c r="H45" s="91" t="n"/>
       <c r="I45" s="91" t="n"/>
+      <c r="J45">
+        <f>IF(OR(A45="",F45=""),"",COUNTIFS($A$2:A45,A45,$F$2:F45,F45))</f>
+        <v/>
+      </c>
+      <c r="K45">
+        <f>IF(OR(A45="",F45="",J45=""),"",TEXT(A45,"yyyymmdd")&amp;"|"&amp;F45&amp;"|"&amp;J45)</f>
+        <v/>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="233" t="n"/>
@@ -54391,6 +54753,14 @@
       <c r="G46" s="234" t="n"/>
       <c r="H46" s="91" t="n"/>
       <c r="I46" s="91" t="n"/>
+      <c r="J46">
+        <f>IF(OR(A46="",F46=""),"",COUNTIFS($A$2:A46,A46,$F$2:F46,F46))</f>
+        <v/>
+      </c>
+      <c r="K46">
+        <f>IF(OR(A46="",F46="",J46=""),"",TEXT(A46,"yyyymmdd")&amp;"|"&amp;F46&amp;"|"&amp;J46)</f>
+        <v/>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="233" t="n"/>
@@ -54402,6 +54772,14 @@
       <c r="G47" s="234" t="n"/>
       <c r="H47" s="91" t="n"/>
       <c r="I47" s="91" t="n"/>
+      <c r="J47">
+        <f>IF(OR(A47="",F47=""),"",COUNTIFS($A$2:A47,A47,$F$2:F47,F47))</f>
+        <v/>
+      </c>
+      <c r="K47">
+        <f>IF(OR(A47="",F47="",J47=""),"",TEXT(A47,"yyyymmdd")&amp;"|"&amp;F47&amp;"|"&amp;J47)</f>
+        <v/>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="233" t="n"/>
@@ -54413,6 +54791,14 @@
       <c r="G48" s="234" t="n"/>
       <c r="H48" s="91" t="n"/>
       <c r="I48" s="91" t="n"/>
+      <c r="J48">
+        <f>IF(OR(A48="",F48=""),"",COUNTIFS($A$2:A48,A48,$F$2:F48,F48))</f>
+        <v/>
+      </c>
+      <c r="K48">
+        <f>IF(OR(A48="",F48="",J48=""),"",TEXT(A48,"yyyymmdd")&amp;"|"&amp;F48&amp;"|"&amp;J48)</f>
+        <v/>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="233" t="n"/>
@@ -54424,6 +54810,14 @@
       <c r="G49" s="234" t="n"/>
       <c r="H49" s="91" t="n"/>
       <c r="I49" s="91" t="n"/>
+      <c r="J49">
+        <f>IF(OR(A49="",F49=""),"",COUNTIFS($A$2:A49,A49,$F$2:F49,F49))</f>
+        <v/>
+      </c>
+      <c r="K49">
+        <f>IF(OR(A49="",F49="",J49=""),"",TEXT(A49,"yyyymmdd")&amp;"|"&amp;F49&amp;"|"&amp;J49)</f>
+        <v/>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="233" t="n"/>
@@ -54435,6 +54829,14 @@
       <c r="G50" s="234" t="n"/>
       <c r="H50" s="91" t="n"/>
       <c r="I50" s="91" t="n"/>
+      <c r="J50">
+        <f>IF(OR(A50="",F50=""),"",COUNTIFS($A$2:A50,A50,$F$2:F50,F50))</f>
+        <v/>
+      </c>
+      <c r="K50">
+        <f>IF(OR(A50="",F50="",J50=""),"",TEXT(A50,"yyyymmdd")&amp;"|"&amp;F50&amp;"|"&amp;J50)</f>
+        <v/>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="233" t="n"/>
@@ -54446,6 +54848,14 @@
       <c r="G51" s="234" t="n"/>
       <c r="H51" s="91" t="n"/>
       <c r="I51" s="91" t="n"/>
+      <c r="J51">
+        <f>IF(OR(A51="",F51=""),"",COUNTIFS($A$2:A51,A51,$F$2:F51,F51))</f>
+        <v/>
+      </c>
+      <c r="K51">
+        <f>IF(OR(A51="",F51="",J51=""),"",TEXT(A51,"yyyymmdd")&amp;"|"&amp;F51&amp;"|"&amp;J51)</f>
+        <v/>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="233" t="n"/>
@@ -54457,6 +54867,14 @@
       <c r="G52" s="234" t="n"/>
       <c r="H52" s="91" t="n"/>
       <c r="I52" s="91" t="n"/>
+      <c r="J52">
+        <f>IF(OR(A52="",F52=""),"",COUNTIFS($A$2:A52,A52,$F$2:F52,F52))</f>
+        <v/>
+      </c>
+      <c r="K52">
+        <f>IF(OR(A52="",F52="",J52=""),"",TEXT(A52,"yyyymmdd")&amp;"|"&amp;F52&amp;"|"&amp;J52)</f>
+        <v/>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="233" t="n"/>
@@ -54468,6 +54886,14 @@
       <c r="G53" s="234" t="n"/>
       <c r="H53" s="91" t="n"/>
       <c r="I53" s="91" t="n"/>
+      <c r="J53">
+        <f>IF(OR(A53="",F53=""),"",COUNTIFS($A$2:A53,A53,$F$2:F53,F53))</f>
+        <v/>
+      </c>
+      <c r="K53">
+        <f>IF(OR(A53="",F53="",J53=""),"",TEXT(A53,"yyyymmdd")&amp;"|"&amp;F53&amp;"|"&amp;J53)</f>
+        <v/>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="233" t="n"/>
@@ -54479,6 +54905,14 @@
       <c r="G54" s="234" t="n"/>
       <c r="H54" s="91" t="n"/>
       <c r="I54" s="91" t="n"/>
+      <c r="J54">
+        <f>IF(OR(A54="",F54=""),"",COUNTIFS($A$2:A54,A54,$F$2:F54,F54))</f>
+        <v/>
+      </c>
+      <c r="K54">
+        <f>IF(OR(A54="",F54="",J54=""),"",TEXT(A54,"yyyymmdd")&amp;"|"&amp;F54&amp;"|"&amp;J54)</f>
+        <v/>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="233" t="n"/>
@@ -54490,6 +54924,14 @@
       <c r="G55" s="234" t="n"/>
       <c r="H55" s="91" t="n"/>
       <c r="I55" s="91" t="n"/>
+      <c r="J55">
+        <f>IF(OR(A55="",F55=""),"",COUNTIFS($A$2:A55,A55,$F$2:F55,F55))</f>
+        <v/>
+      </c>
+      <c r="K55">
+        <f>IF(OR(A55="",F55="",J55=""),"",TEXT(A55,"yyyymmdd")&amp;"|"&amp;F55&amp;"|"&amp;J55)</f>
+        <v/>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="233" t="n"/>
@@ -54501,6 +54943,14 @@
       <c r="G56" s="234" t="n"/>
       <c r="H56" s="91" t="n"/>
       <c r="I56" s="91" t="n"/>
+      <c r="J56">
+        <f>IF(OR(A56="",F56=""),"",COUNTIFS($A$2:A56,A56,$F$2:F56,F56))</f>
+        <v/>
+      </c>
+      <c r="K56">
+        <f>IF(OR(A56="",F56="",J56=""),"",TEXT(A56,"yyyymmdd")&amp;"|"&amp;F56&amp;"|"&amp;J56)</f>
+        <v/>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="233" t="n"/>
@@ -54512,6 +54962,14 @@
       <c r="G57" s="234" t="n"/>
       <c r="H57" s="91" t="n"/>
       <c r="I57" s="91" t="n"/>
+      <c r="J57">
+        <f>IF(OR(A57="",F57=""),"",COUNTIFS($A$2:A57,A57,$F$2:F57,F57))</f>
+        <v/>
+      </c>
+      <c r="K57">
+        <f>IF(OR(A57="",F57="",J57=""),"",TEXT(A57,"yyyymmdd")&amp;"|"&amp;F57&amp;"|"&amp;J57)</f>
+        <v/>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="233" t="n"/>
@@ -54523,6 +54981,14 @@
       <c r="G58" s="234" t="n"/>
       <c r="H58" s="91" t="n"/>
       <c r="I58" s="91" t="n"/>
+      <c r="J58">
+        <f>IF(OR(A58="",F58=""),"",COUNTIFS($A$2:A58,A58,$F$2:F58,F58))</f>
+        <v/>
+      </c>
+      <c r="K58">
+        <f>IF(OR(A58="",F58="",J58=""),"",TEXT(A58,"yyyymmdd")&amp;"|"&amp;F58&amp;"|"&amp;J58)</f>
+        <v/>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="233" t="n"/>
@@ -54534,6 +55000,14 @@
       <c r="G59" s="234" t="n"/>
       <c r="H59" s="91" t="n"/>
       <c r="I59" s="91" t="n"/>
+      <c r="J59">
+        <f>IF(OR(A59="",F59=""),"",COUNTIFS($A$2:A59,A59,$F$2:F59,F59))</f>
+        <v/>
+      </c>
+      <c r="K59">
+        <f>IF(OR(A59="",F59="",J59=""),"",TEXT(A59,"yyyymmdd")&amp;"|"&amp;F59&amp;"|"&amp;J59)</f>
+        <v/>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="233" t="n"/>
@@ -54545,6 +55019,14 @@
       <c r="G60" s="234" t="n"/>
       <c r="H60" s="91" t="n"/>
       <c r="I60" s="91" t="n"/>
+      <c r="J60">
+        <f>IF(OR(A60="",F60=""),"",COUNTIFS($A$2:A60,A60,$F$2:F60,F60))</f>
+        <v/>
+      </c>
+      <c r="K60">
+        <f>IF(OR(A60="",F60="",J60=""),"",TEXT(A60,"yyyymmdd")&amp;"|"&amp;F60&amp;"|"&amp;J60)</f>
+        <v/>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="233" t="n"/>
@@ -54556,6 +55038,14 @@
       <c r="G61" s="234" t="n"/>
       <c r="H61" s="91" t="n"/>
       <c r="I61" s="91" t="n"/>
+      <c r="J61">
+        <f>IF(OR(A61="",F61=""),"",COUNTIFS($A$2:A61,A61,$F$2:F61,F61))</f>
+        <v/>
+      </c>
+      <c r="K61">
+        <f>IF(OR(A61="",F61="",J61=""),"",TEXT(A61,"yyyymmdd")&amp;"|"&amp;F61&amp;"|"&amp;J61)</f>
+        <v/>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="233" t="n"/>
@@ -54567,6 +55057,14 @@
       <c r="G62" s="234" t="n"/>
       <c r="H62" s="91" t="n"/>
       <c r="I62" s="91" t="n"/>
+      <c r="J62">
+        <f>IF(OR(A62="",F62=""),"",COUNTIFS($A$2:A62,A62,$F$2:F62,F62))</f>
+        <v/>
+      </c>
+      <c r="K62">
+        <f>IF(OR(A62="",F62="",J62=""),"",TEXT(A62,"yyyymmdd")&amp;"|"&amp;F62&amp;"|"&amp;J62)</f>
+        <v/>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="233" t="n"/>
@@ -54578,6 +55076,14 @@
       <c r="G63" s="234" t="n"/>
       <c r="H63" s="91" t="n"/>
       <c r="I63" s="91" t="n"/>
+      <c r="J63">
+        <f>IF(OR(A63="",F63=""),"",COUNTIFS($A$2:A63,A63,$F$2:F63,F63))</f>
+        <v/>
+      </c>
+      <c r="K63">
+        <f>IF(OR(A63="",F63="",J63=""),"",TEXT(A63,"yyyymmdd")&amp;"|"&amp;F63&amp;"|"&amp;J63)</f>
+        <v/>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="233" t="n"/>
@@ -54589,6 +55095,14 @@
       <c r="G64" s="234" t="n"/>
       <c r="H64" s="91" t="n"/>
       <c r="I64" s="91" t="n"/>
+      <c r="J64">
+        <f>IF(OR(A64="",F64=""),"",COUNTIFS($A$2:A64,A64,$F$2:F64,F64))</f>
+        <v/>
+      </c>
+      <c r="K64">
+        <f>IF(OR(A64="",F64="",J64=""),"",TEXT(A64,"yyyymmdd")&amp;"|"&amp;F64&amp;"|"&amp;J64)</f>
+        <v/>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="233" t="n"/>
@@ -54600,6 +55114,14 @@
       <c r="G65" s="234" t="n"/>
       <c r="H65" s="91" t="n"/>
       <c r="I65" s="91" t="n"/>
+      <c r="J65">
+        <f>IF(OR(A65="",F65=""),"",COUNTIFS($A$2:A65,A65,$F$2:F65,F65))</f>
+        <v/>
+      </c>
+      <c r="K65">
+        <f>IF(OR(A65="",F65="",J65=""),"",TEXT(A65,"yyyymmdd")&amp;"|"&amp;F65&amp;"|"&amp;J65)</f>
+        <v/>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="233" t="n"/>
@@ -54611,6 +55133,14 @@
       <c r="G66" s="234" t="n"/>
       <c r="H66" s="91" t="n"/>
       <c r="I66" s="91" t="n"/>
+      <c r="J66">
+        <f>IF(OR(A66="",F66=""),"",COUNTIFS($A$2:A66,A66,$F$2:F66,F66))</f>
+        <v/>
+      </c>
+      <c r="K66">
+        <f>IF(OR(A66="",F66="",J66=""),"",TEXT(A66,"yyyymmdd")&amp;"|"&amp;F66&amp;"|"&amp;J66)</f>
+        <v/>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="233" t="n"/>
@@ -54622,6 +55152,14 @@
       <c r="G67" s="234" t="n"/>
       <c r="H67" s="91" t="n"/>
       <c r="I67" s="91" t="n"/>
+      <c r="J67">
+        <f>IF(OR(A67="",F67=""),"",COUNTIFS($A$2:A67,A67,$F$2:F67,F67))</f>
+        <v/>
+      </c>
+      <c r="K67">
+        <f>IF(OR(A67="",F67="",J67=""),"",TEXT(A67,"yyyymmdd")&amp;"|"&amp;F67&amp;"|"&amp;J67)</f>
+        <v/>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="233" t="n"/>
@@ -54633,6 +55171,14 @@
       <c r="G68" s="234" t="n"/>
       <c r="H68" s="91" t="n"/>
       <c r="I68" s="91" t="n"/>
+      <c r="J68">
+        <f>IF(OR(A68="",F68=""),"",COUNTIFS($A$2:A68,A68,$F$2:F68,F68))</f>
+        <v/>
+      </c>
+      <c r="K68">
+        <f>IF(OR(A68="",F68="",J68=""),"",TEXT(A68,"yyyymmdd")&amp;"|"&amp;F68&amp;"|"&amp;J68)</f>
+        <v/>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="233" t="n"/>
@@ -54644,6 +55190,14 @@
       <c r="G69" s="234" t="n"/>
       <c r="H69" s="91" t="n"/>
       <c r="I69" s="91" t="n"/>
+      <c r="J69">
+        <f>IF(OR(A69="",F69=""),"",COUNTIFS($A$2:A69,A69,$F$2:F69,F69))</f>
+        <v/>
+      </c>
+      <c r="K69">
+        <f>IF(OR(A69="",F69="",J69=""),"",TEXT(A69,"yyyymmdd")&amp;"|"&amp;F69&amp;"|"&amp;J69)</f>
+        <v/>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="233" t="n"/>
@@ -54655,6 +55209,14 @@
       <c r="G70" s="234" t="n"/>
       <c r="H70" s="91" t="n"/>
       <c r="I70" s="91" t="n"/>
+      <c r="J70">
+        <f>IF(OR(A70="",F70=""),"",COUNTIFS($A$2:A70,A70,$F$2:F70,F70))</f>
+        <v/>
+      </c>
+      <c r="K70">
+        <f>IF(OR(A70="",F70="",J70=""),"",TEXT(A70,"yyyymmdd")&amp;"|"&amp;F70&amp;"|"&amp;J70)</f>
+        <v/>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="233" t="n"/>
@@ -54666,6 +55228,14 @@
       <c r="G71" s="234" t="n"/>
       <c r="H71" s="91" t="n"/>
       <c r="I71" s="91" t="n"/>
+      <c r="J71">
+        <f>IF(OR(A71="",F71=""),"",COUNTIFS($A$2:A71,A71,$F$2:F71,F71))</f>
+        <v/>
+      </c>
+      <c r="K71">
+        <f>IF(OR(A71="",F71="",J71=""),"",TEXT(A71,"yyyymmdd")&amp;"|"&amp;F71&amp;"|"&amp;J71)</f>
+        <v/>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="233" t="n"/>
@@ -54677,6 +55247,14 @@
       <c r="G72" s="234" t="n"/>
       <c r="H72" s="91" t="n"/>
       <c r="I72" s="91" t="n"/>
+      <c r="J72">
+        <f>IF(OR(A72="",F72=""),"",COUNTIFS($A$2:A72,A72,$F$2:F72,F72))</f>
+        <v/>
+      </c>
+      <c r="K72">
+        <f>IF(OR(A72="",F72="",J72=""),"",TEXT(A72,"yyyymmdd")&amp;"|"&amp;F72&amp;"|"&amp;J72)</f>
+        <v/>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="233" t="n"/>
@@ -54688,6 +55266,14 @@
       <c r="G73" s="234" t="n"/>
       <c r="H73" s="91" t="n"/>
       <c r="I73" s="91" t="n"/>
+      <c r="J73">
+        <f>IF(OR(A73="",F73=""),"",COUNTIFS($A$2:A73,A73,$F$2:F73,F73))</f>
+        <v/>
+      </c>
+      <c r="K73">
+        <f>IF(OR(A73="",F73="",J73=""),"",TEXT(A73,"yyyymmdd")&amp;"|"&amp;F73&amp;"|"&amp;J73)</f>
+        <v/>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="233" t="n"/>
@@ -54699,6 +55285,14 @@
       <c r="G74" s="234" t="n"/>
       <c r="H74" s="91" t="n"/>
       <c r="I74" s="91" t="n"/>
+      <c r="J74">
+        <f>IF(OR(A74="",F74=""),"",COUNTIFS($A$2:A74,A74,$F$2:F74,F74))</f>
+        <v/>
+      </c>
+      <c r="K74">
+        <f>IF(OR(A74="",F74="",J74=""),"",TEXT(A74,"yyyymmdd")&amp;"|"&amp;F74&amp;"|"&amp;J74)</f>
+        <v/>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="233" t="n"/>
@@ -54710,6 +55304,14 @@
       <c r="G75" s="234" t="n"/>
       <c r="H75" s="91" t="n"/>
       <c r="I75" s="91" t="n"/>
+      <c r="J75">
+        <f>IF(OR(A75="",F75=""),"",COUNTIFS($A$2:A75,A75,$F$2:F75,F75))</f>
+        <v/>
+      </c>
+      <c r="K75">
+        <f>IF(OR(A75="",F75="",J75=""),"",TEXT(A75,"yyyymmdd")&amp;"|"&amp;F75&amp;"|"&amp;J75)</f>
+        <v/>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="233" t="n"/>
@@ -54721,6 +55323,14 @@
       <c r="G76" s="234" t="n"/>
       <c r="H76" s="91" t="n"/>
       <c r="I76" s="91" t="n"/>
+      <c r="J76">
+        <f>IF(OR(A76="",F76=""),"",COUNTIFS($A$2:A76,A76,$F$2:F76,F76))</f>
+        <v/>
+      </c>
+      <c r="K76">
+        <f>IF(OR(A76="",F76="",J76=""),"",TEXT(A76,"yyyymmdd")&amp;"|"&amp;F76&amp;"|"&amp;J76)</f>
+        <v/>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="233" t="n"/>
@@ -54732,6 +55342,14 @@
       <c r="G77" s="234" t="n"/>
       <c r="H77" s="91" t="n"/>
       <c r="I77" s="91" t="n"/>
+      <c r="J77">
+        <f>IF(OR(A77="",F77=""),"",COUNTIFS($A$2:A77,A77,$F$2:F77,F77))</f>
+        <v/>
+      </c>
+      <c r="K77">
+        <f>IF(OR(A77="",F77="",J77=""),"",TEXT(A77,"yyyymmdd")&amp;"|"&amp;F77&amp;"|"&amp;J77)</f>
+        <v/>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="233" t="n"/>
@@ -54743,6 +55361,14 @@
       <c r="G78" s="234" t="n"/>
       <c r="H78" s="91" t="n"/>
       <c r="I78" s="91" t="n"/>
+      <c r="J78">
+        <f>IF(OR(A78="",F78=""),"",COUNTIFS($A$2:A78,A78,$F$2:F78,F78))</f>
+        <v/>
+      </c>
+      <c r="K78">
+        <f>IF(OR(A78="",F78="",J78=""),"",TEXT(A78,"yyyymmdd")&amp;"|"&amp;F78&amp;"|"&amp;J78)</f>
+        <v/>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="233" t="n"/>
@@ -54754,6 +55380,14 @@
       <c r="G79" s="234" t="n"/>
       <c r="H79" s="91" t="n"/>
       <c r="I79" s="91" t="n"/>
+      <c r="J79">
+        <f>IF(OR(A79="",F79=""),"",COUNTIFS($A$2:A79,A79,$F$2:F79,F79))</f>
+        <v/>
+      </c>
+      <c r="K79">
+        <f>IF(OR(A79="",F79="",J79=""),"",TEXT(A79,"yyyymmdd")&amp;"|"&amp;F79&amp;"|"&amp;J79)</f>
+        <v/>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="233" t="n"/>
@@ -54765,6 +55399,14 @@
       <c r="G80" s="234" t="n"/>
       <c r="H80" s="91" t="n"/>
       <c r="I80" s="91" t="n"/>
+      <c r="J80">
+        <f>IF(OR(A80="",F80=""),"",COUNTIFS($A$2:A80,A80,$F$2:F80,F80))</f>
+        <v/>
+      </c>
+      <c r="K80">
+        <f>IF(OR(A80="",F80="",J80=""),"",TEXT(A80,"yyyymmdd")&amp;"|"&amp;F80&amp;"|"&amp;J80)</f>
+        <v/>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="233" t="n"/>
@@ -54776,6 +55418,14 @@
       <c r="G81" s="234" t="n"/>
       <c r="H81" s="91" t="n"/>
       <c r="I81" s="91" t="n"/>
+      <c r="J81">
+        <f>IF(OR(A81="",F81=""),"",COUNTIFS($A$2:A81,A81,$F$2:F81,F81))</f>
+        <v/>
+      </c>
+      <c r="K81">
+        <f>IF(OR(A81="",F81="",J81=""),"",TEXT(A81,"yyyymmdd")&amp;"|"&amp;F81&amp;"|"&amp;J81)</f>
+        <v/>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="233" t="n"/>
@@ -54787,6 +55437,14 @@
       <c r="G82" s="234" t="n"/>
       <c r="H82" s="91" t="n"/>
       <c r="I82" s="91" t="n"/>
+      <c r="J82">
+        <f>IF(OR(A82="",F82=""),"",COUNTIFS($A$2:A82,A82,$F$2:F82,F82))</f>
+        <v/>
+      </c>
+      <c r="K82">
+        <f>IF(OR(A82="",F82="",J82=""),"",TEXT(A82,"yyyymmdd")&amp;"|"&amp;F82&amp;"|"&amp;J82)</f>
+        <v/>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="233" t="n"/>
@@ -54798,6 +55456,14 @@
       <c r="G83" s="234" t="n"/>
       <c r="H83" s="91" t="n"/>
       <c r="I83" s="91" t="n"/>
+      <c r="J83">
+        <f>IF(OR(A83="",F83=""),"",COUNTIFS($A$2:A83,A83,$F$2:F83,F83))</f>
+        <v/>
+      </c>
+      <c r="K83">
+        <f>IF(OR(A83="",F83="",J83=""),"",TEXT(A83,"yyyymmdd")&amp;"|"&amp;F83&amp;"|"&amp;J83)</f>
+        <v/>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="233" t="n"/>
@@ -54809,6 +55475,14 @@
       <c r="G84" s="234" t="n"/>
       <c r="H84" s="91" t="n"/>
       <c r="I84" s="91" t="n"/>
+      <c r="J84">
+        <f>IF(OR(A84="",F84=""),"",COUNTIFS($A$2:A84,A84,$F$2:F84,F84))</f>
+        <v/>
+      </c>
+      <c r="K84">
+        <f>IF(OR(A84="",F84="",J84=""),"",TEXT(A84,"yyyymmdd")&amp;"|"&amp;F84&amp;"|"&amp;J84)</f>
+        <v/>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="233" t="n"/>
@@ -54820,6 +55494,14 @@
       <c r="G85" s="234" t="n"/>
       <c r="H85" s="91" t="n"/>
       <c r="I85" s="91" t="n"/>
+      <c r="J85">
+        <f>IF(OR(A85="",F85=""),"",COUNTIFS($A$2:A85,A85,$F$2:F85,F85))</f>
+        <v/>
+      </c>
+      <c r="K85">
+        <f>IF(OR(A85="",F85="",J85=""),"",TEXT(A85,"yyyymmdd")&amp;"|"&amp;F85&amp;"|"&amp;J85)</f>
+        <v/>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="233" t="n"/>
@@ -54831,6 +55513,14 @@
       <c r="G86" s="234" t="n"/>
       <c r="H86" s="91" t="n"/>
       <c r="I86" s="91" t="n"/>
+      <c r="J86">
+        <f>IF(OR(A86="",F86=""),"",COUNTIFS($A$2:A86,A86,$F$2:F86,F86))</f>
+        <v/>
+      </c>
+      <c r="K86">
+        <f>IF(OR(A86="",F86="",J86=""),"",TEXT(A86,"yyyymmdd")&amp;"|"&amp;F86&amp;"|"&amp;J86)</f>
+        <v/>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="233" t="n"/>
@@ -54842,6 +55532,14 @@
       <c r="G87" s="234" t="n"/>
       <c r="H87" s="91" t="n"/>
       <c r="I87" s="91" t="n"/>
+      <c r="J87">
+        <f>IF(OR(A87="",F87=""),"",COUNTIFS($A$2:A87,A87,$F$2:F87,F87))</f>
+        <v/>
+      </c>
+      <c r="K87">
+        <f>IF(OR(A87="",F87="",J87=""),"",TEXT(A87,"yyyymmdd")&amp;"|"&amp;F87&amp;"|"&amp;J87)</f>
+        <v/>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="233" t="n"/>
@@ -54853,6 +55551,14 @@
       <c r="G88" s="234" t="n"/>
       <c r="H88" s="91" t="n"/>
       <c r="I88" s="91" t="n"/>
+      <c r="J88">
+        <f>IF(OR(A88="",F88=""),"",COUNTIFS($A$2:A88,A88,$F$2:F88,F88))</f>
+        <v/>
+      </c>
+      <c r="K88">
+        <f>IF(OR(A88="",F88="",J88=""),"",TEXT(A88,"yyyymmdd")&amp;"|"&amp;F88&amp;"|"&amp;J88)</f>
+        <v/>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="233" t="n"/>
@@ -54864,6 +55570,14 @@
       <c r="G89" s="234" t="n"/>
       <c r="H89" s="91" t="n"/>
       <c r="I89" s="91" t="n"/>
+      <c r="J89">
+        <f>IF(OR(A89="",F89=""),"",COUNTIFS($A$2:A89,A89,$F$2:F89,F89))</f>
+        <v/>
+      </c>
+      <c r="K89">
+        <f>IF(OR(A89="",F89="",J89=""),"",TEXT(A89,"yyyymmdd")&amp;"|"&amp;F89&amp;"|"&amp;J89)</f>
+        <v/>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="233" t="n"/>
@@ -54875,6 +55589,14 @@
       <c r="G90" s="234" t="n"/>
       <c r="H90" s="91" t="n"/>
       <c r="I90" s="91" t="n"/>
+      <c r="J90">
+        <f>IF(OR(A90="",F90=""),"",COUNTIFS($A$2:A90,A90,$F$2:F90,F90))</f>
+        <v/>
+      </c>
+      <c r="K90">
+        <f>IF(OR(A90="",F90="",J90=""),"",TEXT(A90,"yyyymmdd")&amp;"|"&amp;F90&amp;"|"&amp;J90)</f>
+        <v/>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="233" t="n"/>
@@ -54886,6 +55608,14 @@
       <c r="G91" s="234" t="n"/>
       <c r="H91" s="91" t="n"/>
       <c r="I91" s="91" t="n"/>
+      <c r="J91">
+        <f>IF(OR(A91="",F91=""),"",COUNTIFS($A$2:A91,A91,$F$2:F91,F91))</f>
+        <v/>
+      </c>
+      <c r="K91">
+        <f>IF(OR(A91="",F91="",J91=""),"",TEXT(A91,"yyyymmdd")&amp;"|"&amp;F91&amp;"|"&amp;J91)</f>
+        <v/>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="233" t="n"/>
@@ -54897,6 +55627,14 @@
       <c r="G92" s="234" t="n"/>
       <c r="H92" s="91" t="n"/>
       <c r="I92" s="91" t="n"/>
+      <c r="J92">
+        <f>IF(OR(A92="",F92=""),"",COUNTIFS($A$2:A92,A92,$F$2:F92,F92))</f>
+        <v/>
+      </c>
+      <c r="K92">
+        <f>IF(OR(A92="",F92="",J92=""),"",TEXT(A92,"yyyymmdd")&amp;"|"&amp;F92&amp;"|"&amp;J92)</f>
+        <v/>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="233" t="n"/>
@@ -54908,6 +55646,14 @@
       <c r="G93" s="234" t="n"/>
       <c r="H93" s="91" t="n"/>
       <c r="I93" s="91" t="n"/>
+      <c r="J93">
+        <f>IF(OR(A93="",F93=""),"",COUNTIFS($A$2:A93,A93,$F$2:F93,F93))</f>
+        <v/>
+      </c>
+      <c r="K93">
+        <f>IF(OR(A93="",F93="",J93=""),"",TEXT(A93,"yyyymmdd")&amp;"|"&amp;F93&amp;"|"&amp;J93)</f>
+        <v/>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="233" t="n"/>
@@ -54919,6 +55665,14 @@
       <c r="G94" s="234" t="n"/>
       <c r="H94" s="91" t="n"/>
       <c r="I94" s="91" t="n"/>
+      <c r="J94">
+        <f>IF(OR(A94="",F94=""),"",COUNTIFS($A$2:A94,A94,$F$2:F94,F94))</f>
+        <v/>
+      </c>
+      <c r="K94">
+        <f>IF(OR(A94="",F94="",J94=""),"",TEXT(A94,"yyyymmdd")&amp;"|"&amp;F94&amp;"|"&amp;J94)</f>
+        <v/>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="233" t="n"/>
@@ -54930,6 +55684,14 @@
       <c r="G95" s="234" t="n"/>
       <c r="H95" s="91" t="n"/>
       <c r="I95" s="91" t="n"/>
+      <c r="J95">
+        <f>IF(OR(A95="",F95=""),"",COUNTIFS($A$2:A95,A95,$F$2:F95,F95))</f>
+        <v/>
+      </c>
+      <c r="K95">
+        <f>IF(OR(A95="",F95="",J95=""),"",TEXT(A95,"yyyymmdd")&amp;"|"&amp;F95&amp;"|"&amp;J95)</f>
+        <v/>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="233" t="n"/>
@@ -54941,6 +55703,14 @@
       <c r="G96" s="234" t="n"/>
       <c r="H96" s="91" t="n"/>
       <c r="I96" s="91" t="n"/>
+      <c r="J96">
+        <f>IF(OR(A96="",F96=""),"",COUNTIFS($A$2:A96,A96,$F$2:F96,F96))</f>
+        <v/>
+      </c>
+      <c r="K96">
+        <f>IF(OR(A96="",F96="",J96=""),"",TEXT(A96,"yyyymmdd")&amp;"|"&amp;F96&amp;"|"&amp;J96)</f>
+        <v/>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="233" t="n"/>
@@ -54952,6 +55722,14 @@
       <c r="G97" s="234" t="n"/>
       <c r="H97" s="91" t="n"/>
       <c r="I97" s="91" t="n"/>
+      <c r="J97">
+        <f>IF(OR(A97="",F97=""),"",COUNTIFS($A$2:A97,A97,$F$2:F97,F97))</f>
+        <v/>
+      </c>
+      <c r="K97">
+        <f>IF(OR(A97="",F97="",J97=""),"",TEXT(A97,"yyyymmdd")&amp;"|"&amp;F97&amp;"|"&amp;J97)</f>
+        <v/>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="233" t="n"/>
@@ -54963,6 +55741,14 @@
       <c r="G98" s="234" t="n"/>
       <c r="H98" s="91" t="n"/>
       <c r="I98" s="91" t="n"/>
+      <c r="J98">
+        <f>IF(OR(A98="",F98=""),"",COUNTIFS($A$2:A98,A98,$F$2:F98,F98))</f>
+        <v/>
+      </c>
+      <c r="K98">
+        <f>IF(OR(A98="",F98="",J98=""),"",TEXT(A98,"yyyymmdd")&amp;"|"&amp;F98&amp;"|"&amp;J98)</f>
+        <v/>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="233" t="n"/>
@@ -54974,6 +55760,14 @@
       <c r="G99" s="234" t="n"/>
       <c r="H99" s="91" t="n"/>
       <c r="I99" s="91" t="n"/>
+      <c r="J99">
+        <f>IF(OR(A99="",F99=""),"",COUNTIFS($A$2:A99,A99,$F$2:F99,F99))</f>
+        <v/>
+      </c>
+      <c r="K99">
+        <f>IF(OR(A99="",F99="",J99=""),"",TEXT(A99,"yyyymmdd")&amp;"|"&amp;F99&amp;"|"&amp;J99)</f>
+        <v/>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="233" t="n"/>
@@ -54985,6 +55779,14 @@
       <c r="G100" s="234" t="n"/>
       <c r="H100" s="91" t="n"/>
       <c r="I100" s="91" t="n"/>
+      <c r="J100">
+        <f>IF(OR(A100="",F100=""),"",COUNTIFS($A$2:A100,A100,$F$2:F100,F100))</f>
+        <v/>
+      </c>
+      <c r="K100">
+        <f>IF(OR(A100="",F100="",J100=""),"",TEXT(A100,"yyyymmdd")&amp;"|"&amp;F100&amp;"|"&amp;J100)</f>
+        <v/>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="233" t="n"/>
@@ -54996,6 +55798,14 @@
       <c r="G101" s="234" t="n"/>
       <c r="H101" s="91" t="n"/>
       <c r="I101" s="91" t="n"/>
+      <c r="J101">
+        <f>IF(OR(A101="",F101=""),"",COUNTIFS($A$2:A101,A101,$F$2:F101,F101))</f>
+        <v/>
+      </c>
+      <c r="K101">
+        <f>IF(OR(A101="",F101="",J101=""),"",TEXT(A101,"yyyymmdd")&amp;"|"&amp;F101&amp;"|"&amp;J101)</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="2">

</xml_diff>

<commit_message>
Key supplemental payout amounts by Event + Payee
Keep a single VENDOR PAYOUT template for all vendors. Move Bonus and
other supplemental lines to SUPPLEMENTAL DATA so switching Payee cannot
carry another vendor's adjustments into the next statement.

Co-authored-by: unmegonzales <unmegonzales@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/npo-payout/NPO_Payout_Vendor_Template.xlsx
+++ b/npo-payout/NPO_Payout_Vendor_Template.xlsx
@@ -14,6 +14,7 @@
     <sheet name="CONTRACT CALC" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="EVENT ASSIGNMENT" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="TIPS DATA" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="SUPPLEMENTAL DATA" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'VENDOR PAYOUT'!$B$2:$I$61</definedName>
@@ -37,12 +38,12 @@
     <numFmt numFmtId="171" formatCode="mm/dd/yyyy"/>
     <numFmt numFmtId="172" formatCode="\$#,##0.00;\(\$#,##0.00\);\-"/>
     <numFmt numFmtId="173" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
-    <numFmt numFmtId="174" formatCode="mmmm d, yyyy"/>
-    <numFmt numFmtId="175" formatCode="\$#,##0.00;\($#,##0.00\);\-"/>
+    <numFmt numFmtId="174" formatCode="\$#,##0.00;\($#,##0.00\);\-"/>
+    <numFmt numFmtId="175" formatCode="mmmm d, yyyy"/>
     <numFmt numFmtId="176" formatCode="\$#,##0.00;[Red]\($#,##0.00\);\-"/>
     <numFmt numFmtId="177" formatCode="_($* #,##0.00_);_($* (#,##0.00);_($* -??_);_(@_)"/>
   </numFmts>
-  <fonts count="64">
+  <fonts count="65">
     <font>
       <name val="Arial"/>
       <charset val="1"/>
@@ -361,6 +362,12 @@
     <font>
       <name val="Aptos"/>
       <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Aptos"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="10"/>
     </font>
     <font>
@@ -1153,7 +1160,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="22"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="22"/>
   </cellStyleXfs>
-  <cellXfs count="236">
+  <cellXfs count="241">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
@@ -1571,94 +1578,94 @@
     <xf numFmtId="167" fontId="34" fillId="15" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="50" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="48" fillId="10" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="51" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="49" fillId="10" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="49" fillId="11" borderId="38" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="50" fillId="11" borderId="38" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="49" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="175" fontId="51" fillId="11" borderId="39" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="174" fontId="52" fillId="11" borderId="39" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="51" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="52" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="49" fillId="12" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="50" fillId="12" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="174" fontId="49" fillId="19" borderId="32" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="175" fontId="50" fillId="19" borderId="32" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="49" fillId="19" borderId="32" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="50" fillId="19" borderId="32" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="50" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="52" fillId="0" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="51" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="53" fillId="0" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="52" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="53" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="52" fillId="0" borderId="43" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="53" fillId="0" borderId="43" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="53" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="53" fillId="13" borderId="54" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="54" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="54" fillId="13" borderId="54" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="53" fillId="13" borderId="54" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
+    <xf numFmtId="0" fontId="54" fillId="13" borderId="54" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="55" fillId="10" borderId="55" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="56" fillId="10" borderId="55" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="56" fillId="0" borderId="54" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="57" fillId="0" borderId="54" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="54" fillId="0" borderId="54" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="176" fontId="55" fillId="0" borderId="54" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="54" fillId="12" borderId="54" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="176" fontId="55" fillId="12" borderId="54" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="56" fillId="10" borderId="54" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="57" fillId="10" borderId="54" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="54" fillId="10" borderId="54" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="176" fontId="55" fillId="10" borderId="54" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="56" fillId="13" borderId="54" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="57" fillId="13" borderId="54" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="54" fillId="13" borderId="54" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="176" fontId="55" fillId="13" borderId="54" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="56" fillId="17" borderId="54" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="57" fillId="17" borderId="54" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="54" fillId="18" borderId="54" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="176" fontId="55" fillId="18" borderId="54" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="54" fillId="9" borderId="54" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="176" fontId="55" fillId="9" borderId="54" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="55" fillId="0" borderId="55" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="56" fillId="0" borderId="55" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="57" fillId="12" borderId="54" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="176" fontId="49" fillId="12" borderId="54" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="50" fillId="0" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="58" fillId="12" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="58" fillId="12" borderId="54" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="176" fontId="50" fillId="12" borderId="54" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="51" fillId="0" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="59" fillId="12" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="47" fillId="0" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="47" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="176" fontId="54" fillId="0" borderId="54" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="173" fontId="49" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="59" fillId="13" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="176" fontId="55" fillId="0" borderId="54" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="173" fontId="50" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="60" fillId="13" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="61" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="61" fillId="13" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="62" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="177" fontId="63" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="63" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="177" fontId="64" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="170" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="32" fillId="14" borderId="41" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1693,6 +1700,13 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="171" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="48" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="175" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="174" fontId="52" fillId="11" borderId="39" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="64" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3461,7 +3475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L80"/>
+  <dimension ref="A1:I61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="12.75"/>
   <cols>
     <col width="6" customWidth="1" style="130" min="1" max="1"/>
@@ -3537,7 +3551,7 @@
           <t>UNM FOOTBALL • GAME 1</t>
         </is>
       </c>
-      <c r="G6" s="184">
+      <c r="G6" s="239">
         <f>SUM(H43,I43,I46,I47,I48,I49,I50,I51)</f>
         <v/>
       </c>
@@ -4767,8 +4781,9 @@
           <t>Sales Incentive</t>
         </is>
       </c>
-      <c r="I46" s="215" t="n">
-        <v>0</v>
+      <c r="I46" s="215">
+        <f>IFERROR(SUMIFS('SUPPLEMENTAL DATA'!$C$2:$C$101,'SUPPLEMENTAL DATA'!$A$2:$A$101,$B$10,'SUPPLEMENTAL DATA'!$B$2:$B$101,$E$10),0)</f>
+        <v/>
       </c>
     </row>
     <row r="47">
@@ -4778,8 +4793,9 @@
           <t>Culinary - Cook Fee</t>
         </is>
       </c>
-      <c r="I47" s="215" t="n">
-        <v>0</v>
+      <c r="I47" s="215">
+        <f>IFERROR(SUMIFS('SUPPLEMENTAL DATA'!$D$2:$D$101,'SUPPLEMENTAL DATA'!$A$2:$A$101,$B$10,'SUPPLEMENTAL DATA'!$B$2:$B$101,$E$10),0)</f>
+        <v/>
       </c>
     </row>
     <row r="48">
@@ -4788,8 +4804,9 @@
           <t>Minimum Donation</t>
         </is>
       </c>
-      <c r="I48" s="215" t="n">
-        <v>0</v>
+      <c r="I48" s="215">
+        <f>IFERROR(SUMIFS('SUPPLEMENTAL DATA'!$E$2:$E$101,'SUPPLEMENTAL DATA'!$A$2:$A$101,$B$10,'SUPPLEMENTAL DATA'!$B$2:$B$101,$E$10),0)</f>
+        <v/>
       </c>
     </row>
     <row r="49">
@@ -4798,8 +4815,9 @@
           <t>Bonus (Other)</t>
         </is>
       </c>
-      <c r="I49" s="215" t="n">
-        <v>0</v>
+      <c r="I49" s="215">
+        <f>IFERROR(SUMIFS('SUPPLEMENTAL DATA'!$F$2:$F$101,'SUPPLEMENTAL DATA'!$A$2:$A$101,$B$10,'SUPPLEMENTAL DATA'!$B$2:$B$101,$E$10),0)</f>
+        <v/>
       </c>
     </row>
     <row r="50">
@@ -4808,8 +4826,9 @@
           <t>Deductible POS Shortages</t>
         </is>
       </c>
-      <c r="I50" s="215" t="n">
-        <v>0</v>
+      <c r="I50" s="215">
+        <f>IFERROR(SUMIFS('SUPPLEMENTAL DATA'!$G$2:$G$101,'SUPPLEMENTAL DATA'!$A$2:$A$101,$B$10,'SUPPLEMENTAL DATA'!$B$2:$B$101,$E$10),0)</f>
+        <v/>
       </c>
     </row>
     <row r="51">
@@ -4818,8 +4837,9 @@
           <t>Uniform / Staffing / Cleaning Fees</t>
         </is>
       </c>
-      <c r="I51" s="215" t="n">
-        <v>0</v>
+      <c r="I51" s="215">
+        <f>IFERROR(SUMIFS('SUPPLEMENTAL DATA'!$H$2:$H$101,'SUPPLEMENTAL DATA'!$A$2:$A$101,$B$10,'SUPPLEMENTAL DATA'!$B$2:$B$101,$E$10),0)</f>
+        <v/>
       </c>
     </row>
     <row r="52">
@@ -4828,8 +4848,6 @@
         <v/>
       </c>
     </row>
-    <row r="53"/>
-    <row r="54"/>
     <row r="55">
       <c r="B55" s="217" t="inlineStr">
         <is>
@@ -4862,7 +4880,7 @@
           <t>241 | 36127 | GL:611225</t>
         </is>
       </c>
-      <c r="G56" s="221">
+      <c r="G56" s="240">
         <f>H43</f>
         <v/>
       </c>
@@ -4883,7 +4901,7 @@
           <t>241 | 36127 | GL:212113</t>
         </is>
       </c>
-      <c r="G57" s="221">
+      <c r="G57" s="240">
         <f>I43</f>
         <v/>
       </c>
@@ -4908,7 +4926,7 @@
           <t>241 | 36127 | GL:673000</t>
         </is>
       </c>
-      <c r="G58" s="221">
+      <c r="G58" s="240">
         <f>SUM(I46:I50)</f>
         <v/>
       </c>
@@ -4929,7 +4947,7 @@
           <t>241 | 36127 | GL:674102</t>
         </is>
       </c>
-      <c r="G59" s="221">
+      <c r="G59" s="240">
         <f>I51</f>
         <v/>
       </c>
@@ -4952,40 +4970,21 @@
         </is>
       </c>
     </row>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
   </sheetData>
   <mergeCells count="17">
     <mergeCell ref="E12:F12"/>
-    <mergeCell ref="G6:H7"/>
-    <mergeCell ref="C2:G2"/>
-    <mergeCell ref="B16:I16"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="B47:E51"/>
     <mergeCell ref="B55:C55"/>
     <mergeCell ref="E55:G55"/>
     <mergeCell ref="B6:F6"/>
     <mergeCell ref="E10:F10"/>
+    <mergeCell ref="G6:H7"/>
+    <mergeCell ref="C2:G2"/>
+    <mergeCell ref="B16:I16"/>
     <mergeCell ref="B44:H44"/>
     <mergeCell ref="G45:I45"/>
     <mergeCell ref="B5:F5"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="B47:E51"/>
     <mergeCell ref="C9:D9"/>
     <mergeCell ref="E9:F9"/>
     <mergeCell ref="B46:E46"/>
@@ -56703,4 +56702,282 @@
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" style="130" min="1" max="1"/>
+    <col width="18" customWidth="1" style="130" min="2" max="2"/>
+    <col width="14" customWidth="1" style="130" min="3" max="3"/>
+    <col width="16" customWidth="1" style="130" min="4" max="4"/>
+    <col width="14" customWidth="1" style="130" min="5" max="5"/>
+    <col width="14" customWidth="1" style="130" min="6" max="6"/>
+    <col width="18" customWidth="1" style="130" min="7" max="7"/>
+    <col width="22" customWidth="1" style="130" min="8" max="8"/>
+    <col width="40" customWidth="1" style="130" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="236" t="inlineStr">
+        <is>
+          <t>Event Date</t>
+        </is>
+      </c>
+      <c r="B1" s="236" t="inlineStr">
+        <is>
+          <t>NPO</t>
+        </is>
+      </c>
+      <c r="C1" s="236" t="inlineStr">
+        <is>
+          <t>Sales Incentive</t>
+        </is>
+      </c>
+      <c r="D1" s="236" t="inlineStr">
+        <is>
+          <t>Culinary - Cook Fee</t>
+        </is>
+      </c>
+      <c r="E1" s="236" t="inlineStr">
+        <is>
+          <t>Minimum Donation</t>
+        </is>
+      </c>
+      <c r="F1" s="236" t="inlineStr">
+        <is>
+          <t>Bonus (Other)</t>
+        </is>
+      </c>
+      <c r="G1" s="236" t="inlineStr">
+        <is>
+          <t>Deductible POS Shortages</t>
+        </is>
+      </c>
+      <c r="H1" s="236" t="inlineStr">
+        <is>
+          <t>Uniform / Staffing / Cleaning Fees</t>
+        </is>
+      </c>
+      <c r="I1" s="236" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="237" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ARVC</t>
+        </is>
+      </c>
+      <c r="C2" s="238" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" s="238" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" s="238" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" s="238" t="n">
+        <v>250</v>
+      </c>
+      <c r="G2" s="238" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" s="238" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Enter vendor-specific adjustments by Event + Payee. VENDOR PAYOUT reads these; it does not store them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="237" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>AIRFORCE</t>
+        </is>
+      </c>
+      <c r="C3" s="238" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" s="238" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" s="238" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="238" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="238" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" s="238" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="237" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>UNITED FIT</t>
+        </is>
+      </c>
+      <c r="C4" s="238" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="238" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="238" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="238" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="238" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="238" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="237" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>DCVA</t>
+        </is>
+      </c>
+      <c r="C5" s="238" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="238" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="238" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="238" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="238" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="238" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="237" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>DEL N CHEER</t>
+        </is>
+      </c>
+      <c r="C6" s="238" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="238" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="238" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="238" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="238" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="238" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="237" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>RIO GRANDE RGHS</t>
+        </is>
+      </c>
+      <c r="C7" s="238" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="238" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="238" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="238" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="238" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="238" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="237" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>VICTORY OUTREACH</t>
+        </is>
+      </c>
+      <c r="C8" s="238" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="238" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="238" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="238" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="238" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="238" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="B2:B101" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>='SET-UP &amp; SUMMARY'!$A$12:$A$18</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Reset supplemental seed amounts to zero
Co-authored-by: unmegonzales <unmegonzales@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/npo-payout/NPO_Payout_Vendor_Template.xlsx
+++ b/npo-payout/NPO_Payout_Vendor_Template.xlsx
@@ -27,7 +27,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="14">
+  <numFmts count="15">
     <numFmt numFmtId="164" formatCode="dddd"/>
     <numFmt numFmtId="165" formatCode="[$-F800]dddd&quot;, &quot;mmmm\ dd&quot;, &quot;yyyy"/>
     <numFmt numFmtId="166" formatCode="_(\$* #,##0.00_);_(\$* \(#,##0.00\);_(\$* \-??_);_(@_)"/>
@@ -38,10 +38,11 @@
     <numFmt numFmtId="171" formatCode="mm/dd/yyyy"/>
     <numFmt numFmtId="172" formatCode="\$#,##0.00;\(\$#,##0.00\);\-"/>
     <numFmt numFmtId="173" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
-    <numFmt numFmtId="174" formatCode="\$#,##0.00;\($#,##0.00\);\-"/>
+    <numFmt numFmtId="174" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="175" formatCode="mmmm d, yyyy"/>
     <numFmt numFmtId="176" formatCode="\$#,##0.00;[Red]\($#,##0.00\);\-"/>
-    <numFmt numFmtId="177" formatCode="_($* #,##0.00_);_($* (#,##0.00);_($* -??_);_(@_)"/>
+    <numFmt numFmtId="177" formatCode="\$#,##0.00;\($#,##0.00\);\-"/>
+    <numFmt numFmtId="178" formatCode="_($* #,##0.00_);_($* (#,##0.00);_($* -??_);_(@_)"/>
   </numFmts>
   <fonts count="65">
     <font>
@@ -1160,7 +1161,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="22"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="22"/>
   </cellStyleXfs>
-  <cellXfs count="241">
+  <cellXfs count="239">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
@@ -1586,7 +1587,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="49" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="174" fontId="52" fillId="11" borderId="39" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="177" fontId="52" fillId="11" borderId="39" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="51" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1665,7 +1666,7 @@
     <xf numFmtId="0" fontId="61" fillId="13" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="62" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="63" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="177" fontId="64" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="178" fontId="64" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="170" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="32" fillId="14" borderId="41" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1703,10 +1704,6 @@
     <xf numFmtId="0" fontId="48" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="175" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="174" fontId="52" fillId="11" borderId="39" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="64" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3475,7 +3472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I61"/>
+  <dimension ref="A1:L80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="12.75"/>
   <cols>
     <col width="6" customWidth="1" style="130" min="1" max="1"/>
@@ -3551,7 +3548,7 @@
           <t>UNM FOOTBALL • GAME 1</t>
         </is>
       </c>
-      <c r="G6" s="239">
+      <c r="G6" s="184">
         <f>SUM(H43,I43,I46,I47,I48,I49,I50,I51)</f>
         <v/>
       </c>
@@ -4848,6 +4845,8 @@
         <v/>
       </c>
     </row>
+    <row r="53"/>
+    <row r="54"/>
     <row r="55">
       <c r="B55" s="217" t="inlineStr">
         <is>
@@ -4880,7 +4879,7 @@
           <t>241 | 36127 | GL:611225</t>
         </is>
       </c>
-      <c r="G56" s="240">
+      <c r="G56" s="221">
         <f>H43</f>
         <v/>
       </c>
@@ -4901,7 +4900,7 @@
           <t>241 | 36127 | GL:212113</t>
         </is>
       </c>
-      <c r="G57" s="240">
+      <c r="G57" s="221">
         <f>I43</f>
         <v/>
       </c>
@@ -4926,7 +4925,7 @@
           <t>241 | 36127 | GL:673000</t>
         </is>
       </c>
-      <c r="G58" s="240">
+      <c r="G58" s="221">
         <f>SUM(I46:I50)</f>
         <v/>
       </c>
@@ -4947,7 +4946,7 @@
           <t>241 | 36127 | GL:674102</t>
         </is>
       </c>
-      <c r="G59" s="240">
+      <c r="G59" s="221">
         <f>I51</f>
         <v/>
       </c>
@@ -4970,21 +4969,40 @@
         </is>
       </c>
     </row>
+    <row r="62"/>
+    <row r="63"/>
+    <row r="64"/>
+    <row r="65"/>
+    <row r="66"/>
+    <row r="67"/>
+    <row r="68"/>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
+    <row r="72"/>
+    <row r="73"/>
+    <row r="74"/>
+    <row r="75"/>
+    <row r="76"/>
+    <row r="77"/>
+    <row r="78"/>
+    <row r="79"/>
+    <row r="80"/>
   </sheetData>
   <mergeCells count="17">
     <mergeCell ref="E12:F12"/>
+    <mergeCell ref="G6:H7"/>
+    <mergeCell ref="C2:G2"/>
+    <mergeCell ref="B16:I16"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="B47:E51"/>
     <mergeCell ref="B55:C55"/>
     <mergeCell ref="E55:G55"/>
     <mergeCell ref="B6:F6"/>
     <mergeCell ref="E10:F10"/>
-    <mergeCell ref="G6:H7"/>
-    <mergeCell ref="C2:G2"/>
-    <mergeCell ref="B16:I16"/>
     <mergeCell ref="B44:H44"/>
     <mergeCell ref="G45:I45"/>
     <mergeCell ref="B5:F5"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="B47:E51"/>
     <mergeCell ref="C9:D9"/>
     <mergeCell ref="E9:F9"/>
     <mergeCell ref="B46:E46"/>
@@ -56790,7 +56808,7 @@
         <v>0</v>
       </c>
       <c r="F2" s="238" t="n">
-        <v>250</v>
+        <v>0</v>
       </c>
       <c r="G2" s="238" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Cap Vendor Payout location detail at 10 rows
Remove excess empty location slots so the statement stays compact.
TOTAL, supplemental, notes, and auth sections shift up accordingly.

Co-authored-by: unmegonzales <unmegonzales@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/npo-payout/NPO_Payout_Vendor_Template.xlsx
+++ b/npo-payout/NPO_Payout_Vendor_Template.xlsx
@@ -18,7 +18,7 @@
     <sheet name="SUPPLEMENTAL DATA" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">'VENDOR PAYOUT'!$B$2:$I$51</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'VENDOR PAYOUT'!$B$2:$I$46</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'MSR RAW'!$A$1:$W$175</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'CONTRACT CALC'!$A$12:$L$112</definedName>
   </definedNames>
@@ -28,7 +28,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="11">
+  <numFmts count="12">
     <numFmt numFmtId="164" formatCode="dddd"/>
     <numFmt numFmtId="165" formatCode="[$-F800]dddd&quot;, &quot;mmmm\ dd&quot;, &quot;yyyy"/>
     <numFmt numFmtId="166" formatCode="_(\$* #,##0.00_);_(\$* \(#,##0.00\);_(\$* \-??_);_(@_)"/>
@@ -40,8 +40,9 @@
     <numFmt numFmtId="172" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
     <numFmt numFmtId="173" formatCode="\$#,##0.00;\(\$#,##0.00\);\-"/>
     <numFmt numFmtId="174" formatCode="\$#,##0.00;[Red]\($#,##0.00\);\-"/>
+    <numFmt numFmtId="175" formatCode="_($* #,##0.00_);_($* (#,##0.00);_($* -??_);_(@_)"/>
   </numFmts>
-  <fonts count="50">
+  <fonts count="57">
     <font>
       <name val="Arial"/>
       <charset val="1"/>
@@ -353,6 +354,40 @@
       <color rgb="FF990000"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Aptos"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Aptos"/>
+      <b val="1"/>
+      <sz val="8.5"/>
+    </font>
+    <font>
+      <name val="Aptos"/>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="18">
     <fill>
@@ -451,7 +486,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="32">
+  <borders count="34">
     <border>
       <left/>
       <right/>
@@ -787,12 +822,27 @@
         <color rgb="FFB0B7C3"/>
       </bottom>
     </border>
+    <border/>
+    <border>
+      <left style="thin">
+        <color rgb="FFB0B7C3"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB0B7C3"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB0B7C3"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF17365D"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="25"/>
   </cellStyleXfs>
-  <cellXfs count="179">
+  <cellXfs count="212">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="14" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
@@ -1182,6 +1232,77 @@
     <xf numFmtId="169" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="170" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="171" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="28" fillId="0" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="0" borderId="32" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="51" fillId="11" borderId="33" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="174" fontId="52" fillId="11" borderId="33" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="0" borderId="32" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="32" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="50" fillId="0" borderId="32" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="44" fillId="12" borderId="32" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="12" borderId="32" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="45" fillId="0" borderId="32" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="174" fontId="46" fillId="17" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="174" fontId="47" fillId="11" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="17" borderId="32" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="50" fillId="0" borderId="32" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="171" fontId="45" fillId="0" borderId="32" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="45" fillId="0" borderId="32" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="45" fillId="0" borderId="32" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="174" fontId="46" fillId="17" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="174" fontId="47" fillId="11" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="0" borderId="32" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="174" fontId="48" fillId="0" borderId="32" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="174" fontId="52" fillId="0" borderId="32" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="32" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="174" fontId="50" fillId="0" borderId="32" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="44" fillId="12" borderId="32" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="53" fillId="12" borderId="32" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="54" fillId="0" borderId="32" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="55" fillId="0" borderId="32" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="175" fontId="56" fillId="0" borderId="32" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="45" fillId="0" borderId="32" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="50" fillId="0" borderId="32" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="50" fillId="0" borderId="32" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1509,7 +1630,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G80"/>
+  <dimension ref="A1:E80"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="12.75" customHeight="1"/>
   <cols>
     <col width="21" customWidth="1" style="126" min="1" max="1"/>
@@ -3218,11 +3339,6 @@
           <t>Albuquerque Rugby Volleyball Club</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>ARVC</t>
@@ -3233,7 +3349,6 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
       <c r="L2" s="140" t="inlineStr">
         <is>
           <t>One row per NPO/vendor group. Alias must match EVENT ASSIGNMENT NPO and VENDOR PAYOUT Payee. SAP/BSS fill the settlement header automatically. Standing Notes are permanent group info — not event-specific settlement notes.</t>
@@ -3251,11 +3366,6 @@
           <t>Air Force Association / Support Group</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
           <t>AIRFORCE</t>
@@ -3266,7 +3376,6 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3279,11 +3388,6 @@
           <t>United Fitness / Booster Group</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
           <t>UNITED FIT</t>
@@ -3294,7 +3398,6 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3307,11 +3410,6 @@
           <t>Duke City Volleyball Association</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
           <t>DCVA</t>
@@ -3322,7 +3420,6 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3335,11 +3432,6 @@
           <t>Del Norte Cheer</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
           <t>DEL N CHEER</t>
@@ -3350,7 +3442,6 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3363,11 +3454,6 @@
           <t>Rio Grande High School</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
           <t>RIO GRANDE RGHS</t>
@@ -3378,7 +3464,6 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3391,11 +3476,6 @@
           <t>Victory Outreach Albuquerque</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
           <t>VICTORY OUTREACH</t>
@@ -3406,7 +3486,6 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -3423,7 +3502,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I52"/>
+  <dimension ref="A1:K79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="12.75"/>
   <cols>
     <col width="6" customWidth="1" style="126" min="1" max="1"/>
@@ -3499,7 +3578,7 @@
         <v/>
       </c>
       <c r="G6" s="145">
-        <f>SUM(H33,I33,H36,H37,H38,H39,H40,H41)</f>
+        <f>SUM(H28,I28,H31,H32,H33,H34,H35,H36)</f>
         <v/>
       </c>
       <c r="H6" s="99" t="n"/>
@@ -3643,23 +3722,23 @@
     <row r="14" ht="24" customHeight="1" s="126">
       <c r="A14" s="32" t="n"/>
       <c r="B14" s="75">
-        <f>D33</f>
+        <f>D28</f>
         <v/>
       </c>
       <c r="C14" s="75">
-        <f>F33</f>
+        <f>F28</f>
         <v/>
       </c>
       <c r="D14" s="76">
-        <f>C33</f>
+        <f>C28</f>
         <v/>
       </c>
       <c r="E14" s="77">
-        <f>D33</f>
+        <f>D28</f>
         <v/>
       </c>
       <c r="F14" s="76">
-        <f>E33</f>
+        <f>E28</f>
         <v/>
       </c>
       <c r="H14" s="106" t="n"/>
@@ -3732,35 +3811,35 @@
         <f>IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|1",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")</f>
         <v/>
       </c>
-      <c r="B18" s="82">
+      <c r="B18" s="179">
         <f>IF(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|1",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|1",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
-      <c r="C18" s="151">
+      <c r="C18" s="180">
         <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|1",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B18=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|1",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|1",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
-      <c r="D18" s="151">
+      <c r="D18" s="180">
         <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|1",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B18=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|1",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|1",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
-      <c r="E18" s="151">
+      <c r="E18" s="180">
         <f>IF(D18="","",D18*'CONTRACT CALC'!$B$4)</f>
         <v/>
       </c>
-      <c r="F18" s="151">
+      <c r="F18" s="180">
         <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|1",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B18=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|1",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|1",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
-      <c r="G18" s="151">
+      <c r="G18" s="180">
         <f>IF(F18="","",F18*'CONTRACT CALC'!$B$5)</f>
         <v/>
       </c>
-      <c r="H18" s="151">
+      <c r="H18" s="180">
         <f>IF(B18="","",N(E18)+N(G18))</f>
         <v/>
       </c>
-      <c r="I18" s="151">
+      <c r="I18" s="180">
         <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|1",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B18=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|1",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|1",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|1",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))))</f>
         <v/>
       </c>
@@ -3770,35 +3849,35 @@
         <f>IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|2",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")</f>
         <v/>
       </c>
-      <c r="B19" s="82">
+      <c r="B19" s="179">
         <f>IF(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|2",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|2",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
-      <c r="C19" s="151">
+      <c r="C19" s="180">
         <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|2",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B19=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|2",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|2",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
-      <c r="D19" s="151">
+      <c r="D19" s="180">
         <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|2",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B19=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|2",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|2",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
-      <c r="E19" s="151">
+      <c r="E19" s="180">
         <f>IF(D19="","",D19*'CONTRACT CALC'!$B$4)</f>
         <v/>
       </c>
-      <c r="F19" s="151">
+      <c r="F19" s="180">
         <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|2",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B19=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|2",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|2",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
-      <c r="G19" s="151">
+      <c r="G19" s="180">
         <f>IF(F19="","",F19*'CONTRACT CALC'!$B$5)</f>
         <v/>
       </c>
-      <c r="H19" s="151">
+      <c r="H19" s="180">
         <f>IF(B19="","",N(E19)+N(G19))</f>
         <v/>
       </c>
-      <c r="I19" s="151">
+      <c r="I19" s="180">
         <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|2",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B19=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|2",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|2",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|2",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))))</f>
         <v/>
       </c>
@@ -3808,35 +3887,35 @@
         <f>IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|3",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")</f>
         <v/>
       </c>
-      <c r="B20" s="82">
+      <c r="B20" s="179">
         <f>IF(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|3",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|3",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
-      <c r="C20" s="151">
+      <c r="C20" s="180">
         <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|3",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B20=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|3",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|3",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
-      <c r="D20" s="151">
+      <c r="D20" s="180">
         <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|3",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B20=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|3",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|3",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
-      <c r="E20" s="151">
+      <c r="E20" s="180">
         <f>IF(D20="","",D20*'CONTRACT CALC'!$B$4)</f>
         <v/>
       </c>
-      <c r="F20" s="151">
+      <c r="F20" s="180">
         <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|3",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B20=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|3",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|3",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
-      <c r="G20" s="151">
+      <c r="G20" s="180">
         <f>IF(F20="","",F20*'CONTRACT CALC'!$B$5)</f>
         <v/>
       </c>
-      <c r="H20" s="151">
+      <c r="H20" s="180">
         <f>IF(B20="","",N(E20)+N(G20))</f>
         <v/>
       </c>
-      <c r="I20" s="151">
+      <c r="I20" s="180">
         <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|3",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B20=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|3",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|3",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|3",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))))</f>
         <v/>
       </c>
@@ -3846,35 +3925,35 @@
         <f>IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|4",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")</f>
         <v/>
       </c>
-      <c r="B21" s="82">
+      <c r="B21" s="179">
         <f>IF(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|4",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|4",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
-      <c r="C21" s="151">
+      <c r="C21" s="180">
         <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|4",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B21=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|4",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|4",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
-      <c r="D21" s="151">
+      <c r="D21" s="180">
         <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|4",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B21=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|4",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|4",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
-      <c r="E21" s="151">
+      <c r="E21" s="180">
         <f>IF(D21="","",D21*'CONTRACT CALC'!$B$4)</f>
         <v/>
       </c>
-      <c r="F21" s="151">
+      <c r="F21" s="180">
         <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|4",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B21=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|4",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|4",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
-      <c r="G21" s="151">
+      <c r="G21" s="180">
         <f>IF(F21="","",F21*'CONTRACT CALC'!$B$5)</f>
         <v/>
       </c>
-      <c r="H21" s="151">
+      <c r="H21" s="180">
         <f>IF(B21="","",N(E21)+N(G21))</f>
         <v/>
       </c>
-      <c r="I21" s="151">
+      <c r="I21" s="180">
         <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|4",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B21=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|4",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|4",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|4",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))))</f>
         <v/>
       </c>
@@ -3884,35 +3963,35 @@
         <f>IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|5",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")</f>
         <v/>
       </c>
-      <c r="B22" s="82">
+      <c r="B22" s="179">
         <f>IF(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|5",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|5",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
-      <c r="C22" s="151">
+      <c r="C22" s="180">
         <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|5",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B22=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|5",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|5",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
-      <c r="D22" s="151">
+      <c r="D22" s="180">
         <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|5",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B22=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|5",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|5",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
-      <c r="E22" s="151">
+      <c r="E22" s="180">
         <f>IF(D22="","",D22*'CONTRACT CALC'!$B$4)</f>
         <v/>
       </c>
-      <c r="F22" s="151">
+      <c r="F22" s="180">
         <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|5",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B22=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|5",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|5",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
-      <c r="G22" s="151">
+      <c r="G22" s="180">
         <f>IF(F22="","",F22*'CONTRACT CALC'!$B$5)</f>
         <v/>
       </c>
-      <c r="H22" s="151">
+      <c r="H22" s="180">
         <f>IF(B22="","",N(E22)+N(G22))</f>
         <v/>
       </c>
-      <c r="I22" s="151">
+      <c r="I22" s="180">
         <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|5",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B22=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|5",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|5",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|5",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))))</f>
         <v/>
       </c>
@@ -3922,35 +4001,35 @@
         <f>IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|6",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")</f>
         <v/>
       </c>
-      <c r="B23" s="82">
+      <c r="B23" s="179">
         <f>IF(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|6",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|6",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
-      <c r="C23" s="151">
+      <c r="C23" s="180">
         <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|6",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B23=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|6",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|6",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
-      <c r="D23" s="151">
+      <c r="D23" s="180">
         <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|6",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B23=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|6",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|6",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
-      <c r="E23" s="151">
+      <c r="E23" s="180">
         <f>IF(D23="","",D23*'CONTRACT CALC'!$B$4)</f>
         <v/>
       </c>
-      <c r="F23" s="151">
+      <c r="F23" s="180">
         <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|6",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B23=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|6",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|6",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
-      <c r="G23" s="151">
+      <c r="G23" s="180">
         <f>IF(F23="","",F23*'CONTRACT CALC'!$B$5)</f>
         <v/>
       </c>
-      <c r="H23" s="151">
+      <c r="H23" s="180">
         <f>IF(B23="","",N(E23)+N(G23))</f>
         <v/>
       </c>
-      <c r="I23" s="151">
+      <c r="I23" s="180">
         <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|6",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B23=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|6",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|6",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|6",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))))</f>
         <v/>
       </c>
@@ -3960,35 +4039,35 @@
         <f>IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|7",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")</f>
         <v/>
       </c>
-      <c r="B24" s="82">
+      <c r="B24" s="179">
         <f>IF(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|7",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|7",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
-      <c r="C24" s="151">
+      <c r="C24" s="180">
         <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|7",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B24=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|7",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|7",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
-      <c r="D24" s="151">
+      <c r="D24" s="180">
         <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|7",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B24=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|7",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|7",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
-      <c r="E24" s="151">
+      <c r="E24" s="180">
         <f>IF(D24="","",D24*'CONTRACT CALC'!$B$4)</f>
         <v/>
       </c>
-      <c r="F24" s="151">
+      <c r="F24" s="180">
         <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|7",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B24=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|7",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|7",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
-      <c r="G24" s="151">
+      <c r="G24" s="180">
         <f>IF(F24="","",F24*'CONTRACT CALC'!$B$5)</f>
         <v/>
       </c>
-      <c r="H24" s="151">
+      <c r="H24" s="180">
         <f>IF(B24="","",N(E24)+N(G24))</f>
         <v/>
       </c>
-      <c r="I24" s="151">
+      <c r="I24" s="180">
         <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|7",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B24=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|7",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|7",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|7",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))))</f>
         <v/>
       </c>
@@ -3998,35 +4077,35 @@
         <f>IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|8",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")</f>
         <v/>
       </c>
-      <c r="B25" s="82">
+      <c r="B25" s="179">
         <f>IF(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|8",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|8",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
-      <c r="C25" s="151">
+      <c r="C25" s="180">
         <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|8",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B25=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|8",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|8",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
-      <c r="D25" s="151">
+      <c r="D25" s="180">
         <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|8",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B25=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|8",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|8",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
-      <c r="E25" s="151">
+      <c r="E25" s="180">
         <f>IF(D25="","",D25*'CONTRACT CALC'!$B$4)</f>
         <v/>
       </c>
-      <c r="F25" s="151">
+      <c r="F25" s="180">
         <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|8",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B25=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|8",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|8",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
-      <c r="G25" s="151">
+      <c r="G25" s="180">
         <f>IF(F25="","",F25*'CONTRACT CALC'!$B$5)</f>
         <v/>
       </c>
-      <c r="H25" s="151">
+      <c r="H25" s="180">
         <f>IF(B25="","",N(E25)+N(G25))</f>
         <v/>
       </c>
-      <c r="I25" s="151">
+      <c r="I25" s="180">
         <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|8",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B25=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|8",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|8",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|8",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))))</f>
         <v/>
       </c>
@@ -4036,35 +4115,35 @@
         <f>IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|9",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")</f>
         <v/>
       </c>
-      <c r="B26" s="82">
+      <c r="B26" s="179">
         <f>IF(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|9",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|9",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
-      <c r="C26" s="151">
+      <c r="C26" s="180">
         <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|9",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B26=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|9",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|9",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
-      <c r="D26" s="151">
+      <c r="D26" s="180">
         <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|9",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B26=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|9",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|9",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
-      <c r="E26" s="151">
+      <c r="E26" s="180">
         <f>IF(D26="","",D26*'CONTRACT CALC'!$B$4)</f>
         <v/>
       </c>
-      <c r="F26" s="151">
+      <c r="F26" s="180">
         <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|9",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B26=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|9",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|9",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
-      <c r="G26" s="151">
+      <c r="G26" s="180">
         <f>IF(F26="","",F26*'CONTRACT CALC'!$B$5)</f>
         <v/>
       </c>
-      <c r="H26" s="151">
+      <c r="H26" s="180">
         <f>IF(B26="","",N(E26)+N(G26))</f>
         <v/>
       </c>
-      <c r="I26" s="151">
+      <c r="I26" s="180">
         <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|9",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B26=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|9",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|9",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|9",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))))</f>
         <v/>
       </c>
@@ -4074,543 +4153,923 @@
         <f>IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|10",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")</f>
         <v/>
       </c>
-      <c r="B27" s="82">
+      <c r="B27" s="179">
         <f>IF(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|10",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|10",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
-      <c r="C27" s="151">
+      <c r="C27" s="180">
         <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|10",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B27=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|10",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|10",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
-      <c r="D27" s="151">
+      <c r="D27" s="180">
         <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|10",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B27=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|10",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|10",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
-      <c r="E27" s="151">
+      <c r="E27" s="180">
         <f>IF(D27="","",D27*'CONTRACT CALC'!$B$4)</f>
         <v/>
       </c>
-      <c r="F27" s="151">
+      <c r="F27" s="180">
         <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|10",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B27=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|10",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|10",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
         <v/>
       </c>
-      <c r="G27" s="151">
+      <c r="G27" s="180">
         <f>IF(F27="","",F27*'CONTRACT CALC'!$B$5)</f>
         <v/>
       </c>
-      <c r="H27" s="151">
+      <c r="H27" s="180">
         <f>IF(B27="","",N(E27)+N(G27))</f>
         <v/>
       </c>
-      <c r="I27" s="151">
+      <c r="I27" s="180">
         <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|10",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B27=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|10",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|10",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|10",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))))</f>
         <v/>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1" s="126">
-      <c r="A28" s="81">
-        <f>IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|11",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")</f>
-        <v/>
-      </c>
-      <c r="B28" s="82">
-        <f>IF(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|11",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|11",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
-        <v/>
-      </c>
-      <c r="C28" s="151">
-        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|11",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B28=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|11",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|11",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
-        <v/>
-      </c>
-      <c r="D28" s="151">
-        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|11",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B28=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|11",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|11",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
-        <v/>
-      </c>
-      <c r="E28" s="151">
-        <f>IF(D28="","",D28*'CONTRACT CALC'!$B$4)</f>
-        <v/>
-      </c>
-      <c r="F28" s="151">
-        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|11",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B28=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|11",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|11",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
-        <v/>
-      </c>
-      <c r="G28" s="151">
-        <f>IF(F28="","",F28*'CONTRACT CALC'!$B$5)</f>
-        <v/>
-      </c>
-      <c r="H28" s="151">
-        <f>IF(B28="","",N(E28)+N(G28))</f>
-        <v/>
-      </c>
-      <c r="I28" s="151">
-        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|11",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B28=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|11",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|11",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|11",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))))</f>
-        <v/>
-      </c>
+      <c r="A28" s="181" t="n"/>
+      <c r="B28" s="182" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="C28" s="183">
+        <f>SUM(C18:C27)</f>
+        <v/>
+      </c>
+      <c r="D28" s="183">
+        <f>SUM(D18:D27)</f>
+        <v/>
+      </c>
+      <c r="E28" s="183">
+        <f>SUM(E18:E27)</f>
+        <v/>
+      </c>
+      <c r="F28" s="183">
+        <f>SUM(F18:F27)</f>
+        <v/>
+      </c>
+      <c r="G28" s="183">
+        <f>SUM(G18:G27)</f>
+        <v/>
+      </c>
+      <c r="H28" s="183">
+        <f>SUM(H18:H27)</f>
+        <v/>
+      </c>
+      <c r="I28" s="183">
+        <f>SUM(I18:I27)</f>
+        <v/>
+      </c>
+      <c r="J28" s="184" t="n"/>
+      <c r="K28" s="184" t="n"/>
     </row>
     <row r="29" ht="18" customHeight="1" s="126">
-      <c r="A29" s="81">
-        <f>IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|12",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")</f>
-        <v/>
-      </c>
-      <c r="B29" s="82">
-        <f>IF(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|12",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|12",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
-        <v/>
-      </c>
-      <c r="C29" s="151">
-        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|12",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B29=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|12",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|12",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
-        <v/>
-      </c>
-      <c r="D29" s="151">
-        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|12",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B29=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|12",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|12",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
-        <v/>
-      </c>
-      <c r="E29" s="151">
-        <f>IF(D29="","",D29*'CONTRACT CALC'!$B$4)</f>
-        <v/>
-      </c>
-      <c r="F29" s="151">
-        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|12",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B29=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|12",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|12",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
-        <v/>
-      </c>
-      <c r="G29" s="151">
-        <f>IF(F29="","",F29*'CONTRACT CALC'!$B$5)</f>
-        <v/>
-      </c>
-      <c r="H29" s="151">
-        <f>IF(B29="","",N(E29)+N(G29))</f>
-        <v/>
-      </c>
-      <c r="I29" s="151">
-        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|12",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B29=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|12",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|12",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|12",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30" ht="15.75" customHeight="1" s="126">
-      <c r="A30" s="84">
-        <f>IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|13",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")</f>
-        <v/>
-      </c>
-      <c r="B30" s="82">
-        <f>IF(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|13",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|13",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
-        <v/>
-      </c>
-      <c r="C30" s="151">
-        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|13",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B30=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|13",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|13",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
-        <v/>
-      </c>
-      <c r="D30" s="151">
-        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|13",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B30=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|13",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|13",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
-        <v/>
-      </c>
-      <c r="E30" s="151">
-        <f>IF(D30="","",D30*'CONTRACT CALC'!$B$4)</f>
-        <v/>
-      </c>
-      <c r="F30" s="151">
-        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|13",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B30=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|13",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|13",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
-        <v/>
-      </c>
-      <c r="G30" s="151">
-        <f>IF(F30="","",F30*'CONTRACT CALC'!$B$5)</f>
-        <v/>
-      </c>
-      <c r="H30" s="151">
-        <f>IF(B30="","",N(E30)+N(G30))</f>
-        <v/>
-      </c>
-      <c r="I30" s="151">
-        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|13",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B30=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|13",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|13",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|13",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31" ht="15" customHeight="1" s="126">
-      <c r="A31" s="84">
-        <f>IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|14",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")</f>
-        <v/>
-      </c>
-      <c r="B31" s="82">
-        <f>IF(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|14",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|14",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
-        <v/>
-      </c>
-      <c r="C31" s="151">
-        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|14",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B31=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|14",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|14",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
-        <v/>
-      </c>
-      <c r="D31" s="151">
-        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|14",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B31=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|14",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|14",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
-        <v/>
-      </c>
-      <c r="E31" s="151">
-        <f>IF(D31="","",D31*'CONTRACT CALC'!$B$4)</f>
-        <v/>
-      </c>
-      <c r="F31" s="151">
-        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|14",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B31=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|14",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|14",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
-        <v/>
-      </c>
-      <c r="G31" s="151">
-        <f>IF(F31="","",F31*'CONTRACT CALC'!$B$5)</f>
-        <v/>
-      </c>
-      <c r="H31" s="151">
-        <f>IF(B31="","",N(E31)+N(G31))</f>
-        <v/>
-      </c>
-      <c r="I31" s="151">
-        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|14",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B31=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|14",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|14",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|14",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32" ht="15.75" customHeight="1" s="126">
-      <c r="A32" s="84">
-        <f>IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|15",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")</f>
-        <v/>
-      </c>
-      <c r="B32" s="82">
-        <f>IF(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|15",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="","",IFERROR(INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|15",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
-        <v/>
-      </c>
-      <c r="C32" s="151">
-        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|15",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B32=""),"",IFERROR(INDEX('CONTRACT CALC'!$G$13:$G$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|15",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|15",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
-        <v/>
-      </c>
-      <c r="D32" s="151">
-        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|15",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B32=""),"",IFERROR(INDEX('CONTRACT CALC'!$I$13:$I$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|15",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|15",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
-        <v/>
-      </c>
-      <c r="E32" s="151">
-        <f>IF(D32="","",D32*'CONTRACT CALC'!$B$4)</f>
-        <v/>
-      </c>
-      <c r="F32" s="151">
-        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|15",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B32=""),"",IFERROR(INDEX('CONTRACT CALC'!$H$13:$H$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|15",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))*INDEX('CONTRACT CALC'!$F$13:$F$112,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|15",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")),""))</f>
-        <v/>
-      </c>
-      <c r="G32" s="151">
-        <f>IF(F32="","",F32*'CONTRACT CALC'!$B$5)</f>
-        <v/>
-      </c>
-      <c r="H32" s="151">
-        <f>IF(B32="","",N(E32)+N(G32))</f>
-        <v/>
-      </c>
-      <c r="I32" s="151">
-        <f>IF(OR(IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|15",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")="",B32=""),"",IF(COUNTIFS('TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|15",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))&gt;0,SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$D$2:$D$101,INDEX('EVENT ASSIGNMENT'!$C$2:$C$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|15",'EVENT ASSIGNMENT'!$K$2:$K$101,0),""))),SUMIFS('TIPS DATA'!$H$2:$H$101,'TIPS DATA'!$A$2:$A$101,$B$10,'TIPS DATA'!$C$2:$C$101,$E$10,'TIPS DATA'!$E$2:$E$101,INDEX('EVENT ASSIGNMENT'!$D$2:$D$101,IFERROR(MATCH(TEXT($B$10,"yyyymmdd")&amp;"|"&amp;$E$10&amp;"|15",'EVENT ASSIGNMENT'!$K$2:$K$101,0),"")))))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33" ht="15.75" customHeight="1" s="126">
-      <c r="B33" s="85" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="C33" s="152">
-        <f>SUM(C18:C32)</f>
-        <v/>
-      </c>
-      <c r="D33" s="152">
-        <f>SUM(D18:D32)</f>
-        <v/>
-      </c>
-      <c r="E33" s="152">
-        <f>SUM(E18:E32)</f>
-        <v/>
-      </c>
-      <c r="F33" s="152">
-        <f>SUM(F18:F32)</f>
-        <v/>
-      </c>
-      <c r="G33" s="152">
-        <f>SUM(G18:G32)</f>
-        <v/>
-      </c>
-      <c r="H33" s="152">
-        <f>SUM(H18:H32)</f>
-        <v/>
-      </c>
-      <c r="I33" s="152">
-        <f>SUM(I18:I32)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34">
-      <c r="B34" s="153" t="inlineStr">
-        <is>
-          <t>Location rows are filtered from EVENT ASSIGNMENT / CONTRACT CALC by Event Date + Payee. Location Total = Contractual Donation + Gratuities; commission rates are shown explicitly by sales category above.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="32" customHeight="1" s="126">
-      <c r="G35" s="154" t="inlineStr">
+      <c r="A29" s="181" t="n"/>
+      <c r="B29" s="185" t="inlineStr">
+        <is>
+          <t>Max 10 locations per payee. Rows filter from EVENT ASSIGNMENT / CONTRACT CALC by Event Date + Payee. Location Total = Contractual Donation + Gratuities.</t>
+        </is>
+      </c>
+      <c r="C29" s="167" t="n"/>
+      <c r="D29" s="167" t="n"/>
+      <c r="E29" s="167" t="n"/>
+      <c r="F29" s="167" t="n"/>
+      <c r="G29" s="167" t="n"/>
+      <c r="H29" s="167" t="n"/>
+      <c r="I29" s="186" t="n"/>
+      <c r="J29" s="184" t="n"/>
+      <c r="K29" s="184" t="n"/>
+    </row>
+    <row r="30" ht="32" customHeight="1" s="126">
+      <c r="A30" s="181" t="n"/>
+      <c r="B30" s="181" t="n"/>
+      <c r="C30" s="186" t="n"/>
+      <c r="D30" s="186" t="n"/>
+      <c r="E30" s="186" t="n"/>
+      <c r="F30" s="186" t="n"/>
+      <c r="G30" s="187" t="inlineStr">
         <is>
           <t>SUPPLEMENTAL PAYOUT</t>
         </is>
       </c>
-      <c r="H35" s="155" t="inlineStr">
+      <c r="H30" s="187" t="inlineStr">
         <is>
           <t>THIS STATEMENT
 (edit for PDF)</t>
         </is>
       </c>
-      <c r="I35" s="155" t="inlineStr">
+      <c r="I30" s="187" t="inlineStr">
         <is>
           <t>SAVED REF
 (SUPPLEMENTAL DATA)</t>
         </is>
       </c>
+      <c r="J30" s="184" t="n"/>
+      <c r="K30" s="184" t="n"/>
+    </row>
+    <row r="31" ht="15" customHeight="1" s="126">
+      <c r="A31" s="181" t="n"/>
+      <c r="B31" s="188" t="inlineStr">
+        <is>
+          <t>SETTLEMENT NOTES (this document — edit freely before PDF)</t>
+        </is>
+      </c>
+      <c r="C31" s="167" t="n"/>
+      <c r="D31" s="167" t="n"/>
+      <c r="E31" s="167" t="n"/>
+      <c r="F31" s="186" t="n"/>
+      <c r="G31" s="189" t="inlineStr">
+        <is>
+          <t>Sales Incentive</t>
+        </is>
+      </c>
+      <c r="H31" s="190" t="n">
+        <v>0</v>
+      </c>
+      <c r="I31" s="191">
+        <f>IFERROR(SUMIFS('SUPPLEMENTAL DATA'!$C$2:$C$101,'SUPPLEMENTAL DATA'!$A$2:$A$101,$B$10,'SUPPLEMENTAL DATA'!$B$2:$B$101,$E$10),0)</f>
+        <v/>
+      </c>
+      <c r="J31" s="184" t="n"/>
+      <c r="K31" s="184" t="n"/>
+    </row>
+    <row r="32" ht="15.75" customHeight="1" s="126">
+      <c r="A32" s="181" t="n"/>
+      <c r="B32" s="192" t="inlineStr"/>
+      <c r="C32" s="167" t="n"/>
+      <c r="D32" s="167" t="n"/>
+      <c r="E32" s="167" t="n"/>
+      <c r="F32" s="186" t="n"/>
+      <c r="G32" s="189" t="inlineStr">
+        <is>
+          <t>Culinary - Cook Fee</t>
+        </is>
+      </c>
+      <c r="H32" s="190" t="n">
+        <v>0</v>
+      </c>
+      <c r="I32" s="191">
+        <f>IFERROR(SUMIFS('SUPPLEMENTAL DATA'!$D$2:$D$101,'SUPPLEMENTAL DATA'!$A$2:$A$101,$B$10,'SUPPLEMENTAL DATA'!$B$2:$B$101,$E$10),0)</f>
+        <v/>
+      </c>
+      <c r="J32" s="184" t="n"/>
+      <c r="K32" s="184" t="n"/>
+    </row>
+    <row r="33" ht="15.75" customHeight="1" s="126">
+      <c r="A33" s="184" t="n"/>
+      <c r="B33" s="167" t="n"/>
+      <c r="E33" s="167" t="n"/>
+      <c r="F33" s="193" t="n"/>
+      <c r="G33" s="194" t="inlineStr">
+        <is>
+          <t>Minimum Donation</t>
+        </is>
+      </c>
+      <c r="H33" s="158" t="n">
+        <v>0</v>
+      </c>
+      <c r="I33" s="159">
+        <f>IFERROR(SUMIFS('SUPPLEMENTAL DATA'!$E$2:$E$101,'SUPPLEMENTAL DATA'!$A$2:$A$101,$B$10,'SUPPLEMENTAL DATA'!$B$2:$B$101,$E$10),0)</f>
+        <v/>
+      </c>
+      <c r="J33" s="184" t="n"/>
+      <c r="K33" s="184" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="184" t="n"/>
+      <c r="B34" s="167" t="n"/>
+      <c r="E34" s="167" t="n"/>
+      <c r="F34" s="184" t="n"/>
+      <c r="G34" s="195" t="inlineStr">
+        <is>
+          <t>Bonus (Other)</t>
+        </is>
+      </c>
+      <c r="H34" s="158" t="n">
+        <v>0</v>
+      </c>
+      <c r="I34" s="159">
+        <f>IFERROR(SUMIFS('SUPPLEMENTAL DATA'!$F$2:$F$101,'SUPPLEMENTAL DATA'!$A$2:$A$101,$B$10,'SUPPLEMENTAL DATA'!$B$2:$B$101,$E$10),0)</f>
+        <v/>
+      </c>
+      <c r="J34" s="184" t="n"/>
+      <c r="K34" s="184" t="n"/>
+    </row>
+    <row r="35" ht="32" customHeight="1" s="126">
+      <c r="A35" s="184" t="n"/>
+      <c r="B35" s="167" t="n"/>
+      <c r="E35" s="167" t="n"/>
+      <c r="F35" s="184" t="n"/>
+      <c r="G35" s="196" t="inlineStr">
+        <is>
+          <t>Deductible POS Shortages</t>
+        </is>
+      </c>
+      <c r="H35" s="197" t="n">
+        <v>0</v>
+      </c>
+      <c r="I35" s="198">
+        <f>IFERROR(SUMIFS('SUPPLEMENTAL DATA'!$G$2:$G$101,'SUPPLEMENTAL DATA'!$A$2:$A$101,$B$10,'SUPPLEMENTAL DATA'!$B$2:$B$101,$E$10),0)</f>
+        <v/>
+      </c>
+      <c r="J35" s="184" t="n"/>
+      <c r="K35" s="184" t="n"/>
     </row>
     <row r="36" ht="15.75" customHeight="1" s="126">
-      <c r="B36" s="156" t="inlineStr">
-        <is>
-          <t>SETTLEMENT NOTES (this document — edit freely before PDF)</t>
-        </is>
-      </c>
-      <c r="G36" s="157" t="inlineStr">
-        <is>
-          <t>Sales Incentive</t>
+      <c r="A36" s="184" t="n"/>
+      <c r="B36" s="167" t="n"/>
+      <c r="C36" s="167" t="n"/>
+      <c r="D36" s="167" t="n"/>
+      <c r="E36" s="167" t="n"/>
+      <c r="F36" s="184" t="n"/>
+      <c r="G36" s="195" t="inlineStr">
+        <is>
+          <t>Uniform / Staffing / Cleaning Fees</t>
         </is>
       </c>
       <c r="H36" s="158" t="n">
         <v>0</v>
       </c>
       <c r="I36" s="159">
-        <f>IFERROR(SUMIFS('SUPPLEMENTAL DATA'!$C$2:$C$101,'SUPPLEMENTAL DATA'!$A$2:$A$101,$B$10,'SUPPLEMENTAL DATA'!$B$2:$B$101,$E$10),0)</f>
-        <v/>
-      </c>
+        <f>IFERROR(SUMIFS('SUPPLEMENTAL DATA'!$H$2:$H$101,'SUPPLEMENTAL DATA'!$A$2:$A$101,$B$10,'SUPPLEMENTAL DATA'!$B$2:$B$101,$E$10),0)</f>
+        <v/>
+      </c>
+      <c r="J36" s="184" t="n"/>
+      <c r="K36" s="184" t="n"/>
     </row>
     <row r="37" ht="15.75" customHeight="1" s="126">
-      <c r="B37" s="160" t="inlineStr"/>
-      <c r="G37" s="157" t="inlineStr">
-        <is>
-          <t>Culinary - Cook Fee</t>
-        </is>
-      </c>
-      <c r="H37" s="158" t="n">
-        <v>0</v>
-      </c>
-      <c r="I37" s="159">
-        <f>IFERROR(SUMIFS('SUPPLEMENTAL DATA'!$D$2:$D$101,'SUPPLEMENTAL DATA'!$A$2:$A$101,$B$10,'SUPPLEMENTAL DATA'!$B$2:$B$101,$E$10),0)</f>
-        <v/>
-      </c>
+      <c r="A37" s="184" t="n"/>
+      <c r="B37" s="199" t="n"/>
+      <c r="C37" s="184" t="n"/>
+      <c r="D37" s="184" t="n"/>
+      <c r="E37" s="184" t="n"/>
+      <c r="F37" s="184" t="n"/>
+      <c r="G37" s="184" t="n"/>
+      <c r="H37" s="200" t="inlineStr">
+        <is>
+          <t>Statement supplemental total →</t>
+        </is>
+      </c>
+      <c r="I37" s="201">
+        <f>SUM(H31:H36)</f>
+        <v/>
+      </c>
+      <c r="J37" s="184" t="n"/>
+      <c r="K37" s="184" t="n"/>
     </row>
     <row r="38" ht="15.75" customHeight="1" s="126">
-      <c r="G38" s="157" t="inlineStr">
-        <is>
-          <t>Minimum Donation</t>
-        </is>
-      </c>
-      <c r="H38" s="158" t="n">
-        <v>0</v>
-      </c>
-      <c r="I38" s="159">
-        <f>IFERROR(SUMIFS('SUPPLEMENTAL DATA'!$E$2:$E$101,'SUPPLEMENTAL DATA'!$A$2:$A$101,$B$10,'SUPPLEMENTAL DATA'!$B$2:$B$101,$E$10),0)</f>
-        <v/>
-      </c>
+      <c r="A38" s="184" t="n"/>
+      <c r="B38" s="202" t="inlineStr">
+        <is>
+          <t>Tip: yellow H31:H36 + notes = this statement only. Grey I31:I36 = saved for Event+Payee. After PDF, zero H31:H36 before the next vendor — or copy H into SUPPLEMENTAL DATA to remember.</t>
+        </is>
+      </c>
+      <c r="C38" s="184" t="n"/>
+      <c r="D38" s="184" t="n"/>
+      <c r="E38" s="184" t="n"/>
+      <c r="F38" s="184" t="n"/>
+      <c r="G38" s="184" t="n"/>
+      <c r="H38" s="203" t="n"/>
+      <c r="I38" s="203" t="n"/>
+      <c r="J38" s="184" t="n"/>
+      <c r="K38" s="184" t="n"/>
     </row>
     <row r="39" ht="15.75" customHeight="1" s="126">
-      <c r="G39" s="157" t="inlineStr">
-        <is>
-          <t>Bonus (Other)</t>
-        </is>
-      </c>
-      <c r="H39" s="158" t="n">
-        <v>0</v>
-      </c>
-      <c r="I39" s="159">
-        <f>IFERROR(SUMIFS('SUPPLEMENTAL DATA'!$F$2:$F$101,'SUPPLEMENTAL DATA'!$A$2:$A$101,$B$10,'SUPPLEMENTAL DATA'!$B$2:$B$101,$E$10),0)</f>
-        <v/>
-      </c>
+      <c r="A39" s="184" t="n"/>
+      <c r="B39" s="184" t="n"/>
+      <c r="C39" s="184" t="n"/>
+      <c r="D39" s="184" t="n"/>
+      <c r="E39" s="184" t="n"/>
+      <c r="F39" s="184" t="n"/>
+      <c r="G39" s="184" t="n"/>
+      <c r="H39" s="203" t="n"/>
+      <c r="I39" s="203" t="n"/>
+      <c r="J39" s="184" t="n"/>
+      <c r="K39" s="184" t="n"/>
     </row>
     <row r="40" ht="15.75" customHeight="1" s="126">
-      <c r="G40" s="157" t="inlineStr">
-        <is>
-          <t>Deductible POS Shortages</t>
-        </is>
-      </c>
-      <c r="H40" s="158" t="n">
-        <v>0</v>
-      </c>
-      <c r="I40" s="159">
-        <f>IFERROR(SUMIFS('SUPPLEMENTAL DATA'!$G$2:$G$101,'SUPPLEMENTAL DATA'!$A$2:$A$101,$B$10,'SUPPLEMENTAL DATA'!$B$2:$B$101,$E$10),0)</f>
-        <v/>
-      </c>
+      <c r="A40" s="184" t="n"/>
+      <c r="B40" s="204" t="inlineStr">
+        <is>
+          <t>INTERNAL AUTHORIZATION CHECK REQUEST</t>
+        </is>
+      </c>
+      <c r="C40" s="167" t="n"/>
+      <c r="D40" s="184" t="n"/>
+      <c r="E40" s="205" t="inlineStr">
+        <is>
+          <t>INTERNAL - ACCOUNTING GL ENTRY - SUMMARY</t>
+        </is>
+      </c>
+      <c r="F40" s="167" t="n"/>
+      <c r="G40" s="167" t="n"/>
+      <c r="H40" s="203" t="n"/>
+      <c r="I40" s="203" t="n"/>
+      <c r="J40" s="184" t="n"/>
+      <c r="K40" s="184" t="n"/>
     </row>
     <row r="41" ht="15.75" customHeight="1" s="126">
-      <c r="G41" s="157" t="inlineStr">
-        <is>
-          <t>Uniform / Staffing / Cleaning Fees</t>
-        </is>
-      </c>
-      <c r="H41" s="158" t="n">
-        <v>0</v>
-      </c>
-      <c r="I41" s="159">
-        <f>IFERROR(SUMIFS('SUPPLEMENTAL DATA'!$H$2:$H$101,'SUPPLEMENTAL DATA'!$A$2:$A$101,$B$10,'SUPPLEMENTAL DATA'!$B$2:$B$101,$E$10),0)</f>
-        <v/>
-      </c>
+      <c r="A41" s="184" t="n"/>
+      <c r="B41" s="195" t="inlineStr">
+        <is>
+          <t>Abigail Tenorio</t>
+        </is>
+      </c>
+      <c r="C41" s="184">
+        <f>TODAY()</f>
+        <v/>
+      </c>
+      <c r="D41" s="184" t="n"/>
+      <c r="E41" s="206" t="inlineStr">
+        <is>
+          <t>Group Commission</t>
+        </is>
+      </c>
+      <c r="F41" s="207" t="inlineStr">
+        <is>
+          <t>241 | 36127 | GL:611225</t>
+        </is>
+      </c>
+      <c r="G41" s="208">
+        <f>H28</f>
+        <v/>
+      </c>
+      <c r="H41" s="203" t="n"/>
+      <c r="I41" s="203" t="n"/>
+      <c r="J41" s="184" t="n"/>
+      <c r="K41" s="184" t="n"/>
     </row>
     <row r="42" ht="15.75" customHeight="1" s="126">
-      <c r="H42" s="161" t="inlineStr">
-        <is>
-          <t>Statement supplemental total →</t>
-        </is>
-      </c>
-      <c r="I42" s="162">
-        <f>SUM(H36:H41)</f>
-        <v/>
-      </c>
+      <c r="A42" s="184" t="n"/>
+      <c r="B42" s="195" t="inlineStr">
+        <is>
+          <t>Concessions Manager</t>
+        </is>
+      </c>
+      <c r="C42" s="184" t="n"/>
+      <c r="D42" s="184" t="n"/>
+      <c r="E42" s="206" t="inlineStr">
+        <is>
+          <t>Gratuities</t>
+        </is>
+      </c>
+      <c r="F42" s="207" t="inlineStr">
+        <is>
+          <t>241 | 36127 | GL:212113</t>
+        </is>
+      </c>
+      <c r="G42" s="208">
+        <f>I28</f>
+        <v/>
+      </c>
+      <c r="H42" s="184" t="n"/>
+      <c r="I42" s="203" t="n"/>
+      <c r="J42" s="184" t="n"/>
+      <c r="K42" s="184" t="n"/>
     </row>
     <row r="43">
-      <c r="B43" s="140" t="inlineStr">
-        <is>
-          <t>Tip: yellow H36:H41 + notes = this statement only. Grey I36:I41 = saved for Event+Payee. After PDF, zero H36:H41 before the next vendor — or copy H into SUPPLEMENTAL DATA to remember.</t>
-        </is>
-      </c>
+      <c r="A43" s="184" t="n"/>
+      <c r="B43" s="209" t="inlineStr">
+        <is>
+          <t>Ray Velasquez</t>
+        </is>
+      </c>
+      <c r="C43" s="184">
+        <f>TODAY()</f>
+        <v/>
+      </c>
+      <c r="D43" s="184" t="n"/>
+      <c r="E43" s="206" t="inlineStr">
+        <is>
+          <t>Misc. (to be reclassed)</t>
+        </is>
+      </c>
+      <c r="F43" s="207" t="inlineStr">
+        <is>
+          <t>241 | 36127 | GL:673000</t>
+        </is>
+      </c>
+      <c r="G43" s="208">
+        <f>SUM(H31:H35)</f>
+        <v/>
+      </c>
+      <c r="H43" s="184" t="n"/>
+      <c r="I43" s="184" t="n"/>
+      <c r="J43" s="184" t="n"/>
+      <c r="K43" s="184" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="184" t="n"/>
+      <c r="B44" s="195" t="inlineStr">
+        <is>
+          <t>Director of Operations</t>
+        </is>
+      </c>
+      <c r="C44" s="184" t="n"/>
+      <c r="D44" s="184" t="n"/>
+      <c r="E44" s="206" t="inlineStr">
+        <is>
+          <t>Cleaning Fee - Expense</t>
+        </is>
+      </c>
+      <c r="F44" s="207" t="inlineStr">
+        <is>
+          <t>241 | 36127 | GL:674102</t>
+        </is>
+      </c>
+      <c r="G44" s="208">
+        <f>H36</f>
+        <v/>
+      </c>
+      <c r="H44" s="184" t="n"/>
+      <c r="I44" s="184" t="n"/>
+      <c r="J44" s="184" t="n"/>
+      <c r="K44" s="184" t="n"/>
     </row>
     <row r="45">
-      <c r="B45" s="163" t="inlineStr">
-        <is>
-          <t>INTERNAL AUTHORIZATION CHECK REQUEST</t>
-        </is>
-      </c>
-      <c r="E45" s="164" t="inlineStr">
-        <is>
-          <t>INTERNAL - ACCOUNTING GL ENTRY - SUMMARY</t>
-        </is>
-      </c>
+      <c r="A45" s="184" t="n"/>
+      <c r="B45" s="195" t="inlineStr">
+        <is>
+          <t>Evan E. Gonzales</t>
+        </is>
+      </c>
+      <c r="C45" s="184">
+        <f>TODAY()</f>
+        <v/>
+      </c>
+      <c r="D45" s="184" t="n"/>
+      <c r="E45" s="184" t="n"/>
+      <c r="F45" s="184" t="n"/>
+      <c r="G45" s="184" t="n"/>
+      <c r="H45" s="184" t="n"/>
+      <c r="I45" s="184" t="n"/>
+      <c r="J45" s="184" t="n"/>
+      <c r="K45" s="184" t="n"/>
     </row>
     <row r="46" ht="13.5" customHeight="1" s="126">
-      <c r="B46" s="124" t="inlineStr">
-        <is>
-          <t>Abigail Tenorio</t>
-        </is>
-      </c>
-      <c r="C46" s="125">
-        <f>TODAY()</f>
-        <v/>
-      </c>
-      <c r="E46" s="90" t="inlineStr">
-        <is>
-          <t>Group Commission</t>
-        </is>
-      </c>
-      <c r="F46" s="91" t="inlineStr">
-        <is>
-          <t>241 | 36127 | GL:611225</t>
-        </is>
-      </c>
-      <c r="G46" s="92">
-        <f>H33</f>
-        <v/>
-      </c>
+      <c r="A46" s="184" t="n"/>
+      <c r="B46" s="195" t="inlineStr">
+        <is>
+          <t>Finance Manager</t>
+        </is>
+      </c>
+      <c r="C46" s="210" t="n"/>
+      <c r="D46" s="184" t="n"/>
+      <c r="E46" s="184" t="n"/>
+      <c r="F46" s="184" t="n"/>
+      <c r="G46" s="211" t="n"/>
+      <c r="H46" s="184" t="n"/>
+      <c r="I46" s="184" t="n"/>
+      <c r="J46" s="184" t="n"/>
+      <c r="K46" s="184" t="n"/>
     </row>
     <row r="47" ht="13.5" customHeight="1" s="126">
-      <c r="B47" s="87" t="inlineStr">
-        <is>
-          <t>Concessions Manager</t>
-        </is>
-      </c>
-      <c r="C47" s="125" t="n"/>
-      <c r="E47" s="90" t="inlineStr">
-        <is>
-          <t>Gratuities</t>
-        </is>
-      </c>
-      <c r="F47" s="91" t="inlineStr">
-        <is>
-          <t>241 | 36127 | GL:212113</t>
-        </is>
-      </c>
-      <c r="G47" s="92">
-        <f>I33</f>
-        <v/>
-      </c>
+      <c r="A47" s="184" t="n"/>
+      <c r="B47" s="184" t="n"/>
+      <c r="C47" s="210" t="n"/>
+      <c r="D47" s="184" t="n"/>
+      <c r="E47" s="184" t="n"/>
+      <c r="F47" s="184" t="n"/>
+      <c r="G47" s="211" t="n"/>
+      <c r="H47" s="184" t="n"/>
+      <c r="I47" s="184" t="n"/>
+      <c r="J47" s="184" t="n"/>
+      <c r="K47" s="184" t="n"/>
     </row>
     <row r="48" ht="13.5" customHeight="1" s="126">
-      <c r="B48" s="124" t="inlineStr">
-        <is>
-          <t>Ray Velasquez</t>
-        </is>
-      </c>
-      <c r="C48" s="125">
-        <f>TODAY()</f>
-        <v/>
-      </c>
-      <c r="E48" s="90" t="inlineStr">
-        <is>
-          <t>Misc. (to be reclassed)</t>
-        </is>
-      </c>
-      <c r="F48" s="91" t="inlineStr">
-        <is>
-          <t>241 | 36127 | GL:673000</t>
-        </is>
-      </c>
-      <c r="G48" s="92">
-        <f>SUM(H36:H40)</f>
-        <v/>
-      </c>
+      <c r="A48" s="184" t="n"/>
+      <c r="B48" s="184" t="n"/>
+      <c r="C48" s="210" t="n"/>
+      <c r="D48" s="184" t="n"/>
+      <c r="E48" s="184" t="n"/>
+      <c r="F48" s="184" t="n"/>
+      <c r="G48" s="211" t="n"/>
+      <c r="H48" s="184" t="n"/>
+      <c r="I48" s="184" t="n"/>
+      <c r="J48" s="184" t="n"/>
+      <c r="K48" s="184" t="n"/>
     </row>
     <row r="49" ht="13.5" customHeight="1" s="126">
-      <c r="B49" s="87" t="inlineStr">
-        <is>
-          <t>Director of Operations</t>
-        </is>
-      </c>
-      <c r="C49" s="125" t="n"/>
-      <c r="E49" s="90" t="inlineStr">
-        <is>
-          <t>Cleaning Fee - Expense</t>
-        </is>
-      </c>
-      <c r="F49" s="91" t="inlineStr">
-        <is>
-          <t>241 | 36127 | GL:674102</t>
-        </is>
-      </c>
-      <c r="G49" s="92">
-        <f>H41</f>
-        <v/>
-      </c>
+      <c r="A49" s="184" t="n"/>
+      <c r="B49" s="184" t="n"/>
+      <c r="C49" s="210" t="n"/>
+      <c r="D49" s="184" t="n"/>
+      <c r="E49" s="184" t="n"/>
+      <c r="F49" s="184" t="n"/>
+      <c r="G49" s="211" t="n"/>
+      <c r="H49" s="184" t="n"/>
+      <c r="I49" s="184" t="n"/>
+      <c r="J49" s="184" t="n"/>
+      <c r="K49" s="184" t="n"/>
     </row>
     <row r="50" ht="13.5" customHeight="1" s="126">
-      <c r="B50" s="124" t="inlineStr">
-        <is>
-          <t>Evan E. Gonzales</t>
-        </is>
-      </c>
-      <c r="C50" s="125">
-        <f>TODAY()</f>
-        <v/>
-      </c>
+      <c r="A50" s="184" t="n"/>
+      <c r="B50" s="184" t="n"/>
+      <c r="C50" s="210" t="n"/>
+      <c r="D50" s="184" t="n"/>
+      <c r="E50" s="184" t="n"/>
+      <c r="F50" s="184" t="n"/>
+      <c r="G50" s="184" t="n"/>
+      <c r="H50" s="184" t="n"/>
+      <c r="I50" s="184" t="n"/>
+      <c r="J50" s="184" t="n"/>
+      <c r="K50" s="184" t="n"/>
     </row>
     <row r="51" ht="13.5" customHeight="1" s="126">
-      <c r="B51" s="87" t="inlineStr">
-        <is>
-          <t>Finance Manager</t>
-        </is>
-      </c>
-      <c r="C51" s="125" t="n"/>
+      <c r="A51" s="184" t="n"/>
+      <c r="B51" s="184" t="n"/>
+      <c r="C51" s="210" t="n"/>
+      <c r="D51" s="184" t="n"/>
+      <c r="E51" s="184" t="n"/>
+      <c r="F51" s="184" t="n"/>
+      <c r="G51" s="184" t="n"/>
+      <c r="H51" s="184" t="n"/>
+      <c r="I51" s="184" t="n"/>
+      <c r="J51" s="184" t="n"/>
+      <c r="K51" s="184" t="n"/>
     </row>
     <row r="52">
-      <c r="C52" s="125" t="n"/>
+      <c r="A52" s="184" t="n"/>
+      <c r="B52" s="184" t="n"/>
+      <c r="C52" s="210" t="n"/>
+      <c r="D52" s="184" t="n"/>
+      <c r="E52" s="184" t="n"/>
+      <c r="F52" s="184" t="n"/>
+      <c r="G52" s="184" t="n"/>
+      <c r="H52" s="184" t="n"/>
+      <c r="I52" s="184" t="n"/>
+      <c r="J52" s="184" t="n"/>
+      <c r="K52" s="184" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="184" t="n"/>
+      <c r="B53" s="184" t="n"/>
+      <c r="C53" s="184" t="n"/>
+      <c r="D53" s="184" t="n"/>
+      <c r="E53" s="184" t="n"/>
+      <c r="F53" s="184" t="n"/>
+      <c r="G53" s="184" t="n"/>
+      <c r="H53" s="184" t="n"/>
+      <c r="I53" s="184" t="n"/>
+      <c r="J53" s="184" t="n"/>
+      <c r="K53" s="184" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="184" t="n"/>
+      <c r="B54" s="184" t="n"/>
+      <c r="C54" s="184" t="n"/>
+      <c r="D54" s="184" t="n"/>
+      <c r="E54" s="184" t="n"/>
+      <c r="F54" s="184" t="n"/>
+      <c r="G54" s="184" t="n"/>
+      <c r="H54" s="184" t="n"/>
+      <c r="I54" s="184" t="n"/>
+      <c r="J54" s="184" t="n"/>
+      <c r="K54" s="184" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="184" t="n"/>
+      <c r="B55" s="184" t="n"/>
+      <c r="C55" s="184" t="n"/>
+      <c r="D55" s="184" t="n"/>
+      <c r="E55" s="184" t="n"/>
+      <c r="F55" s="184" t="n"/>
+      <c r="G55" s="184" t="n"/>
+      <c r="H55" s="184" t="n"/>
+      <c r="I55" s="184" t="n"/>
+      <c r="J55" s="184" t="n"/>
+      <c r="K55" s="184" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="184" t="n"/>
+      <c r="B56" s="184" t="n"/>
+      <c r="C56" s="184" t="n"/>
+      <c r="D56" s="184" t="n"/>
+      <c r="E56" s="184" t="n"/>
+      <c r="F56" s="184" t="n"/>
+      <c r="G56" s="184" t="n"/>
+      <c r="H56" s="184" t="n"/>
+      <c r="I56" s="184" t="n"/>
+      <c r="J56" s="184" t="n"/>
+      <c r="K56" s="184" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="184" t="n"/>
+      <c r="B57" s="184" t="n"/>
+      <c r="C57" s="184" t="n"/>
+      <c r="D57" s="184" t="n"/>
+      <c r="E57" s="184" t="n"/>
+      <c r="F57" s="184" t="n"/>
+      <c r="G57" s="184" t="n"/>
+      <c r="H57" s="184" t="n"/>
+      <c r="I57" s="184" t="n"/>
+      <c r="J57" s="184" t="n"/>
+      <c r="K57" s="184" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="184" t="n"/>
+      <c r="B58" s="184" t="n"/>
+      <c r="C58" s="184" t="n"/>
+      <c r="D58" s="184" t="n"/>
+      <c r="E58" s="184" t="n"/>
+      <c r="F58" s="184" t="n"/>
+      <c r="G58" s="184" t="n"/>
+      <c r="H58" s="184" t="n"/>
+      <c r="I58" s="184" t="n"/>
+      <c r="J58" s="184" t="n"/>
+      <c r="K58" s="184" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="184" t="n"/>
+      <c r="B59" s="184" t="n"/>
+      <c r="C59" s="184" t="n"/>
+      <c r="D59" s="184" t="n"/>
+      <c r="E59" s="184" t="n"/>
+      <c r="F59" s="184" t="n"/>
+      <c r="G59" s="184" t="n"/>
+      <c r="H59" s="184" t="n"/>
+      <c r="I59" s="184" t="n"/>
+      <c r="J59" s="184" t="n"/>
+      <c r="K59" s="184" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="184" t="n"/>
+      <c r="B60" s="184" t="n"/>
+      <c r="C60" s="184" t="n"/>
+      <c r="D60" s="184" t="n"/>
+      <c r="E60" s="184" t="n"/>
+      <c r="F60" s="184" t="n"/>
+      <c r="G60" s="184" t="n"/>
+      <c r="H60" s="184" t="n"/>
+      <c r="I60" s="184" t="n"/>
+      <c r="J60" s="184" t="n"/>
+      <c r="K60" s="184" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="184" t="n"/>
+      <c r="B61" s="184" t="n"/>
+      <c r="C61" s="184" t="n"/>
+      <c r="D61" s="184" t="n"/>
+      <c r="E61" s="184" t="n"/>
+      <c r="F61" s="184" t="n"/>
+      <c r="G61" s="184" t="n"/>
+      <c r="H61" s="184" t="n"/>
+      <c r="I61" s="184" t="n"/>
+      <c r="J61" s="184" t="n"/>
+      <c r="K61" s="184" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="184" t="n"/>
+      <c r="B62" s="184" t="n"/>
+      <c r="C62" s="184" t="n"/>
+      <c r="D62" s="184" t="n"/>
+      <c r="E62" s="184" t="n"/>
+      <c r="F62" s="184" t="n"/>
+      <c r="G62" s="184" t="n"/>
+      <c r="H62" s="184" t="n"/>
+      <c r="I62" s="184" t="n"/>
+      <c r="J62" s="184" t="n"/>
+      <c r="K62" s="184" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="184" t="n"/>
+      <c r="B63" s="184" t="n"/>
+      <c r="C63" s="184" t="n"/>
+      <c r="D63" s="184" t="n"/>
+      <c r="E63" s="184" t="n"/>
+      <c r="F63" s="184" t="n"/>
+      <c r="G63" s="184" t="n"/>
+      <c r="H63" s="184" t="n"/>
+      <c r="I63" s="184" t="n"/>
+      <c r="J63" s="184" t="n"/>
+      <c r="K63" s="184" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="184" t="n"/>
+      <c r="B64" s="184" t="n"/>
+      <c r="C64" s="184" t="n"/>
+      <c r="D64" s="184" t="n"/>
+      <c r="E64" s="184" t="n"/>
+      <c r="F64" s="184" t="n"/>
+      <c r="G64" s="184" t="n"/>
+      <c r="H64" s="184" t="n"/>
+      <c r="I64" s="184" t="n"/>
+      <c r="J64" s="184" t="n"/>
+      <c r="K64" s="184" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="184" t="n"/>
+      <c r="B65" s="184" t="n"/>
+      <c r="C65" s="184" t="n"/>
+      <c r="D65" s="184" t="n"/>
+      <c r="E65" s="184" t="n"/>
+      <c r="F65" s="184" t="n"/>
+      <c r="G65" s="184" t="n"/>
+      <c r="H65" s="184" t="n"/>
+      <c r="I65" s="184" t="n"/>
+      <c r="J65" s="184" t="n"/>
+      <c r="K65" s="184" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="184" t="n"/>
+      <c r="B66" s="184" t="n"/>
+      <c r="C66" s="184" t="n"/>
+      <c r="D66" s="184" t="n"/>
+      <c r="E66" s="184" t="n"/>
+      <c r="F66" s="184" t="n"/>
+      <c r="G66" s="184" t="n"/>
+      <c r="H66" s="184" t="n"/>
+      <c r="I66" s="184" t="n"/>
+      <c r="J66" s="184" t="n"/>
+      <c r="K66" s="184" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="184" t="n"/>
+      <c r="B67" s="184" t="n"/>
+      <c r="C67" s="184" t="n"/>
+      <c r="D67" s="184" t="n"/>
+      <c r="E67" s="184" t="n"/>
+      <c r="F67" s="184" t="n"/>
+      <c r="G67" s="184" t="n"/>
+      <c r="H67" s="184" t="n"/>
+      <c r="I67" s="184" t="n"/>
+      <c r="J67" s="184" t="n"/>
+      <c r="K67" s="184" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="184" t="n"/>
+      <c r="B68" s="184" t="n"/>
+      <c r="C68" s="184" t="n"/>
+      <c r="D68" s="184" t="n"/>
+      <c r="E68" s="184" t="n"/>
+      <c r="F68" s="184" t="n"/>
+      <c r="G68" s="184" t="n"/>
+      <c r="H68" s="184" t="n"/>
+      <c r="I68" s="184" t="n"/>
+      <c r="J68" s="184" t="n"/>
+      <c r="K68" s="184" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="184" t="n"/>
+      <c r="B69" s="184" t="n"/>
+      <c r="C69" s="184" t="n"/>
+      <c r="D69" s="184" t="n"/>
+      <c r="E69" s="184" t="n"/>
+      <c r="F69" s="184" t="n"/>
+      <c r="G69" s="184" t="n"/>
+      <c r="H69" s="184" t="n"/>
+      <c r="I69" s="184" t="n"/>
+      <c r="J69" s="184" t="n"/>
+      <c r="K69" s="184" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="184" t="n"/>
+      <c r="B70" s="184" t="n"/>
+      <c r="C70" s="184" t="n"/>
+      <c r="D70" s="184" t="n"/>
+      <c r="E70" s="184" t="n"/>
+      <c r="F70" s="184" t="n"/>
+      <c r="G70" s="184" t="n"/>
+      <c r="H70" s="184" t="n"/>
+      <c r="I70" s="184" t="n"/>
+      <c r="J70" s="184" t="n"/>
+      <c r="K70" s="184" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="184" t="n"/>
+      <c r="B71" s="184" t="n"/>
+      <c r="C71" s="184" t="n"/>
+      <c r="D71" s="184" t="n"/>
+      <c r="E71" s="184" t="n"/>
+      <c r="F71" s="184" t="n"/>
+      <c r="G71" s="184" t="n"/>
+      <c r="H71" s="184" t="n"/>
+      <c r="I71" s="184" t="n"/>
+      <c r="J71" s="184" t="n"/>
+      <c r="K71" s="184" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="184" t="n"/>
+      <c r="B72" s="184" t="n"/>
+      <c r="C72" s="184" t="n"/>
+      <c r="D72" s="184" t="n"/>
+      <c r="E72" s="184" t="n"/>
+      <c r="F72" s="184" t="n"/>
+      <c r="G72" s="184" t="n"/>
+      <c r="H72" s="184" t="n"/>
+      <c r="I72" s="184" t="n"/>
+      <c r="J72" s="184" t="n"/>
+      <c r="K72" s="184" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="184" t="n"/>
+      <c r="B73" s="184" t="n"/>
+      <c r="C73" s="184" t="n"/>
+      <c r="D73" s="184" t="n"/>
+      <c r="E73" s="184" t="n"/>
+      <c r="F73" s="184" t="n"/>
+      <c r="G73" s="184" t="n"/>
+      <c r="H73" s="184" t="n"/>
+      <c r="I73" s="184" t="n"/>
+      <c r="J73" s="184" t="n"/>
+      <c r="K73" s="184" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="184" t="n"/>
+      <c r="B74" s="184" t="n"/>
+      <c r="C74" s="184" t="n"/>
+      <c r="D74" s="184" t="n"/>
+      <c r="E74" s="184" t="n"/>
+      <c r="F74" s="184" t="n"/>
+      <c r="G74" s="184" t="n"/>
+      <c r="H74" s="184" t="n"/>
+      <c r="I74" s="184" t="n"/>
+      <c r="J74" s="184" t="n"/>
+      <c r="K74" s="184" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="184" t="n"/>
+      <c r="B75" s="184" t="n"/>
+      <c r="C75" s="184" t="n"/>
+      <c r="D75" s="184" t="n"/>
+      <c r="E75" s="184" t="n"/>
+      <c r="F75" s="184" t="n"/>
+      <c r="G75" s="184" t="n"/>
+      <c r="H75" s="184" t="n"/>
+      <c r="I75" s="184" t="n"/>
+      <c r="J75" s="184" t="n"/>
+      <c r="K75" s="184" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="184" t="n"/>
+      <c r="B76" s="184" t="n"/>
+      <c r="C76" s="184" t="n"/>
+      <c r="D76" s="184" t="n"/>
+      <c r="E76" s="184" t="n"/>
+      <c r="F76" s="184" t="n"/>
+      <c r="G76" s="184" t="n"/>
+      <c r="H76" s="184" t="n"/>
+      <c r="I76" s="184" t="n"/>
+      <c r="J76" s="184" t="n"/>
+      <c r="K76" s="184" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="184" t="n"/>
+      <c r="B77" s="184" t="n"/>
+      <c r="C77" s="184" t="n"/>
+      <c r="D77" s="184" t="n"/>
+      <c r="E77" s="184" t="n"/>
+      <c r="F77" s="184" t="n"/>
+      <c r="G77" s="184" t="n"/>
+      <c r="H77" s="184" t="n"/>
+      <c r="I77" s="184" t="n"/>
+      <c r="J77" s="184" t="n"/>
+      <c r="K77" s="184" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="184" t="n"/>
+      <c r="B78" s="184" t="n"/>
+      <c r="C78" s="184" t="n"/>
+      <c r="D78" s="184" t="n"/>
+      <c r="E78" s="184" t="n"/>
+      <c r="F78" s="184" t="n"/>
+      <c r="G78" s="184" t="n"/>
+      <c r="H78" s="184" t="n"/>
+      <c r="I78" s="184" t="n"/>
+      <c r="J78" s="184" t="n"/>
+      <c r="K78" s="184" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="184" t="n"/>
+      <c r="B79" s="184" t="n"/>
+      <c r="C79" s="184" t="n"/>
+      <c r="D79" s="184" t="n"/>
+      <c r="E79" s="184" t="n"/>
+      <c r="F79" s="184" t="n"/>
+      <c r="G79" s="184" t="n"/>
+      <c r="H79" s="184" t="n"/>
+      <c r="I79" s="184" t="n"/>
+      <c r="J79" s="184" t="n"/>
+      <c r="K79" s="184" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="16">
     <mergeCell ref="E12:F12"/>
-    <mergeCell ref="B6:F6"/>
-    <mergeCell ref="E10:F10"/>
-    <mergeCell ref="E45:G45"/>
+    <mergeCell ref="B31:E31"/>
     <mergeCell ref="G6:H7"/>
     <mergeCell ref="C2:G2"/>
     <mergeCell ref="B16:I16"/>
-    <mergeCell ref="B45:C45"/>
     <mergeCell ref="G5:H5"/>
+    <mergeCell ref="E40:G40"/>
+    <mergeCell ref="B32:E36"/>
+    <mergeCell ref="B40:C40"/>
+    <mergeCell ref="B6:F6"/>
+    <mergeCell ref="E10:F10"/>
     <mergeCell ref="B5:F5"/>
-    <mergeCell ref="B37:E41"/>
+    <mergeCell ref="B29:H29"/>
     <mergeCell ref="C9:D9"/>
     <mergeCell ref="E9:F9"/>
-    <mergeCell ref="B34:H34"/>
-    <mergeCell ref="B36:E36"/>
     <mergeCell ref="C3:G3"/>
   </mergeCells>
   <dataValidations count="1">

</xml_diff>